<commit_message>
fix: make Excel checkboxes editable via data validation dropdowns
Replace static Unicode checkbox text with setCheckboxCell() that adds
data validation dropdown (☑/☐) so users can toggle checkboxes after
downloading. Applied to Daily Tasks, To Do, Meeting Rails, Follow Ups,
and Personal Goals sections.
</commit_message>
<xml_diff>
--- a/backend/assets/templates/LSW_TEMPLATE.xlsx
+++ b/backend/assets/templates/LSW_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/geraldnyah/Documents/PROGRAMMING/MeetingIntelligence/dashmet-rca-backend/backend/assets/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8905907A-3BB5-6546-8429-371619201BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E421AD54-1E63-B644-B99F-3CE575D1570E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="24000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="38400" windowHeight="22300" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Operations Manager" sheetId="1" state="hidden" r:id="rId1"/>
@@ -1014,7 +1014,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1099,6 +1099,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="98">
     <border>
@@ -2847,6 +2853,111 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="80" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="80" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="93" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="79" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="86" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="95" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="86" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="94" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="81" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="80" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2856,20 +2967,11 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="80" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2886,24 +2988,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="93" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="92" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="88" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="90" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2928,120 +3012,6 @@
     <xf numFmtId="0" fontId="5" fillId="13" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="81" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="80" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="79" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="83" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="84" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="91" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="93" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="86" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="95" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="86" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="94" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3075,6 +3045,114 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="59" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -3096,150 +3174,42 @@
     <xf numFmtId="14" fontId="0" fillId="4" borderId="79" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="59" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="14" borderId="68" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -3287,6 +3257,42 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="74" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="92" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="88" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="90" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="91" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="93" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="83" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="84" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -8924,29 +8930,29 @@
       <c r="H1" s="45"/>
       <c r="I1" s="45"/>
       <c r="J1" s="35"/>
-      <c r="K1" s="279" t="s">
+      <c r="K1" s="267" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="279"/>
+      <c r="L1" s="267"/>
       <c r="M1" s="35"/>
       <c r="N1" s="34"/>
       <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="18"/>
-      <c r="B2" s="274" t="s">
+      <c r="B2" s="262" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="274"/>
-      <c r="D2" s="274"/>
-      <c r="E2" s="274"/>
-      <c r="F2" s="274"/>
-      <c r="G2" s="274"/>
-      <c r="H2" s="274"/>
-      <c r="I2" s="274"/>
+      <c r="C2" s="262"/>
+      <c r="D2" s="262"/>
+      <c r="E2" s="262"/>
+      <c r="F2" s="262"/>
+      <c r="G2" s="262"/>
+      <c r="H2" s="262"/>
+      <c r="I2" s="262"/>
       <c r="J2" s="36"/>
-      <c r="K2" s="280"/>
-      <c r="L2" s="280"/>
+      <c r="K2" s="268"/>
+      <c r="L2" s="268"/>
       <c r="M2" s="37"/>
       <c r="N2" s="38"/>
       <c r="O2" s="20"/>
@@ -9974,42 +9980,42 @@
       <c r="O40" s="13"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A41" s="275" t="s">
+      <c r="A41" s="263" t="s">
         <v>86</v>
       </c>
-      <c r="B41" s="276"/>
-      <c r="C41" s="276"/>
-      <c r="D41" s="276"/>
-      <c r="E41" s="276"/>
-      <c r="F41" s="276"/>
-      <c r="G41" s="276"/>
-      <c r="H41" s="276"/>
-      <c r="I41" s="276"/>
-      <c r="J41" s="276"/>
-      <c r="K41" s="276"/>
+      <c r="B41" s="264"/>
+      <c r="C41" s="264"/>
+      <c r="D41" s="264"/>
+      <c r="E41" s="264"/>
+      <c r="F41" s="264"/>
+      <c r="G41" s="264"/>
+      <c r="H41" s="264"/>
+      <c r="I41" s="264"/>
+      <c r="J41" s="264"/>
+      <c r="K41" s="264"/>
       <c r="L41" s="3"/>
       <c r="M41" s="28"/>
-      <c r="N41" s="276" t="s">
+      <c r="N41" s="264" t="s">
         <v>87</v>
       </c>
-      <c r="O41" s="278"/>
+      <c r="O41" s="266"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A42" s="277"/>
-      <c r="B42" s="272"/>
-      <c r="C42" s="272"/>
-      <c r="D42" s="272"/>
-      <c r="E42" s="272"/>
-      <c r="F42" s="272"/>
-      <c r="G42" s="272"/>
-      <c r="H42" s="272"/>
-      <c r="I42" s="272"/>
-      <c r="J42" s="272"/>
-      <c r="K42" s="272"/>
+      <c r="A42" s="265"/>
+      <c r="B42" s="260"/>
+      <c r="C42" s="260"/>
+      <c r="D42" s="260"/>
+      <c r="E42" s="260"/>
+      <c r="F42" s="260"/>
+      <c r="G42" s="260"/>
+      <c r="H42" s="260"/>
+      <c r="I42" s="260"/>
+      <c r="J42" s="260"/>
+      <c r="K42" s="260"/>
       <c r="L42" s="27"/>
       <c r="M42" s="29"/>
-      <c r="N42" s="272"/>
-      <c r="O42" s="273"/>
+      <c r="N42" s="260"/>
+      <c r="O42" s="261"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" s="77" t="s">
@@ -10399,10 +10405,10 @@
       <c r="K57" s="22"/>
       <c r="L57" s="22"/>
       <c r="M57" s="31"/>
-      <c r="N57" s="270" t="s">
+      <c r="N57" s="258" t="s">
         <v>144</v>
       </c>
-      <c r="O57" s="271"/>
+      <c r="O57" s="259"/>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" s="78"/>
@@ -10418,8 +10424,8 @@
       <c r="K58" s="22"/>
       <c r="L58" s="22"/>
       <c r="M58" s="31"/>
-      <c r="N58" s="272"/>
-      <c r="O58" s="273"/>
+      <c r="N58" s="260"/>
+      <c r="O58" s="261"/>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59" s="78"/>
@@ -10817,10 +10823,10 @@
         <v>160</v>
       </c>
       <c r="M75" s="31"/>
-      <c r="N75" s="270" t="s">
+      <c r="N75" s="258" t="s">
         <v>161</v>
       </c>
-      <c r="O75" s="271"/>
+      <c r="O75" s="259"/>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A76" s="18"/>
@@ -10840,8 +10846,8 @@
         <v>163</v>
       </c>
       <c r="M76" s="31"/>
-      <c r="N76" s="272"/>
-      <c r="O76" s="273"/>
+      <c r="N76" s="260"/>
+      <c r="O76" s="261"/>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A77" s="21"/>
@@ -10997,23 +11003,23 @@
         <v>176</v>
       </c>
       <c r="E1" s="35"/>
-      <c r="F1" s="279" t="s">
+      <c r="F1" s="267" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="279"/>
+      <c r="G1" s="267"/>
       <c r="H1" s="35"/>
-      <c r="I1" s="291" t="s">
+      <c r="I1" s="314" t="s">
         <v>177</v>
       </c>
-      <c r="J1" s="291"/>
-      <c r="K1" s="291"/>
-      <c r="L1" s="291"/>
-      <c r="M1" s="291"/>
-      <c r="N1" s="291"/>
-      <c r="O1" s="291"/>
-      <c r="P1" s="291"/>
-      <c r="Q1" s="291"/>
-      <c r="R1" s="292"/>
+      <c r="J1" s="314"/>
+      <c r="K1" s="314"/>
+      <c r="L1" s="314"/>
+      <c r="M1" s="314"/>
+      <c r="N1" s="314"/>
+      <c r="O1" s="314"/>
+      <c r="P1" s="314"/>
+      <c r="Q1" s="314"/>
+      <c r="R1" s="315"/>
     </row>
     <row r="2" spans="1:18" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="44" t="s">
@@ -11534,18 +11540,18 @@
       </c>
       <c r="G24" s="8"/>
       <c r="H24" s="1"/>
-      <c r="I24" s="293" t="s">
+      <c r="I24" s="316" t="s">
         <v>22</v>
       </c>
-      <c r="J24" s="293"/>
-      <c r="K24" s="293"/>
-      <c r="L24" s="293"/>
-      <c r="M24" s="293"/>
-      <c r="N24" s="293"/>
-      <c r="O24" s="293"/>
-      <c r="P24" s="293"/>
-      <c r="Q24" s="293"/>
-      <c r="R24" s="294"/>
+      <c r="J24" s="316"/>
+      <c r="K24" s="316"/>
+      <c r="L24" s="316"/>
+      <c r="M24" s="316"/>
+      <c r="N24" s="316"/>
+      <c r="O24" s="316"/>
+      <c r="P24" s="316"/>
+      <c r="Q24" s="316"/>
+      <c r="R24" s="317"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25" s="7"/>
@@ -11602,18 +11608,18 @@
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="1"/>
-      <c r="I27" s="293" t="s">
+      <c r="I27" s="316" t="s">
         <v>56</v>
       </c>
-      <c r="J27" s="293"/>
-      <c r="K27" s="293"/>
-      <c r="L27" s="293"/>
-      <c r="M27" s="293"/>
-      <c r="N27" s="293"/>
-      <c r="O27" s="293"/>
-      <c r="P27" s="293"/>
-      <c r="Q27" s="293"/>
-      <c r="R27" s="294"/>
+      <c r="J27" s="316"/>
+      <c r="K27" s="316"/>
+      <c r="L27" s="316"/>
+      <c r="M27" s="316"/>
+      <c r="N27" s="316"/>
+      <c r="O27" s="316"/>
+      <c r="P27" s="316"/>
+      <c r="Q27" s="316"/>
+      <c r="R27" s="317"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" s="7"/>
@@ -11714,18 +11720,18 @@
       </c>
       <c r="G32" s="8"/>
       <c r="H32" s="1"/>
-      <c r="I32" s="295" t="s">
+      <c r="I32" s="318" t="s">
         <v>69</v>
       </c>
-      <c r="J32" s="295"/>
-      <c r="K32" s="295"/>
-      <c r="L32" s="295"/>
-      <c r="M32" s="295"/>
-      <c r="N32" s="295"/>
-      <c r="O32" s="295"/>
-      <c r="P32" s="295"/>
-      <c r="Q32" s="295"/>
-      <c r="R32" s="296"/>
+      <c r="J32" s="318"/>
+      <c r="K32" s="318"/>
+      <c r="L32" s="318"/>
+      <c r="M32" s="318"/>
+      <c r="N32" s="318"/>
+      <c r="O32" s="318"/>
+      <c r="P32" s="318"/>
+      <c r="Q32" s="318"/>
+      <c r="R32" s="319"/>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A33" s="7"/>
@@ -11898,199 +11904,199 @@
       <c r="R40" s="9"/>
     </row>
     <row r="41" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="275"/>
-      <c r="B41" s="276"/>
-      <c r="C41" s="276"/>
-      <c r="D41" s="276"/>
-      <c r="E41" s="276"/>
-      <c r="F41" s="276"/>
+      <c r="A41" s="263"/>
+      <c r="B41" s="264"/>
+      <c r="C41" s="264"/>
+      <c r="D41" s="264"/>
+      <c r="E41" s="264"/>
+      <c r="F41" s="264"/>
       <c r="G41" s="3"/>
       <c r="H41" s="28"/>
-      <c r="I41" s="275" t="s">
+      <c r="I41" s="263" t="s">
         <v>183</v>
       </c>
-      <c r="J41" s="276"/>
-      <c r="K41" s="276"/>
-      <c r="L41" s="276"/>
-      <c r="M41" s="276"/>
-      <c r="N41" s="276"/>
-      <c r="O41" s="276"/>
-      <c r="P41" s="276"/>
-      <c r="Q41" s="276"/>
-      <c r="R41" s="278"/>
+      <c r="J41" s="264"/>
+      <c r="K41" s="264"/>
+      <c r="L41" s="264"/>
+      <c r="M41" s="264"/>
+      <c r="N41" s="264"/>
+      <c r="O41" s="264"/>
+      <c r="P41" s="264"/>
+      <c r="Q41" s="264"/>
+      <c r="R41" s="266"/>
       <c r="S41" s="159"/>
     </row>
     <row r="42" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="277"/>
-      <c r="B42" s="272"/>
-      <c r="C42" s="272"/>
-      <c r="D42" s="272"/>
-      <c r="E42" s="272"/>
-      <c r="F42" s="272"/>
+      <c r="A42" s="265"/>
+      <c r="B42" s="260"/>
+      <c r="C42" s="260"/>
+      <c r="D42" s="260"/>
+      <c r="E42" s="260"/>
+      <c r="F42" s="260"/>
       <c r="G42" s="27"/>
       <c r="H42" s="29"/>
-      <c r="I42" s="277"/>
-      <c r="J42" s="272"/>
-      <c r="K42" s="272"/>
-      <c r="L42" s="272"/>
-      <c r="M42" s="272"/>
-      <c r="N42" s="272"/>
-      <c r="O42" s="272"/>
-      <c r="P42" s="272"/>
-      <c r="Q42" s="272"/>
-      <c r="R42" s="273"/>
+      <c r="I42" s="265"/>
+      <c r="J42" s="260"/>
+      <c r="K42" s="260"/>
+      <c r="L42" s="260"/>
+      <c r="M42" s="260"/>
+      <c r="N42" s="260"/>
+      <c r="O42" s="260"/>
+      <c r="P42" s="260"/>
+      <c r="Q42" s="260"/>
+      <c r="R42" s="261"/>
       <c r="S42" s="159"/>
     </row>
     <row r="43" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="87"/>
-      <c r="B43" s="297"/>
-      <c r="C43" s="298"/>
-      <c r="D43" s="298"/>
-      <c r="E43" s="298"/>
-      <c r="F43" s="298"/>
-      <c r="G43" s="299"/>
+      <c r="B43" s="320"/>
+      <c r="C43" s="321"/>
+      <c r="D43" s="321"/>
+      <c r="E43" s="321"/>
+      <c r="F43" s="321"/>
+      <c r="G43" s="322"/>
       <c r="H43" s="30"/>
       <c r="I43" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J43" s="281" t="s">
+      <c r="J43" s="305" t="s">
         <v>184</v>
       </c>
-      <c r="K43" s="282"/>
-      <c r="L43" s="282"/>
-      <c r="M43" s="282"/>
-      <c r="N43" s="282"/>
-      <c r="O43" s="283"/>
-      <c r="P43" s="240" t="s">
+      <c r="K43" s="306"/>
+      <c r="L43" s="306"/>
+      <c r="M43" s="306"/>
+      <c r="N43" s="306"/>
+      <c r="O43" s="307"/>
+      <c r="P43" s="237" t="s">
         <v>185</v>
       </c>
-      <c r="Q43" s="240"/>
-      <c r="R43" s="290"/>
+      <c r="Q43" s="237"/>
+      <c r="R43" s="323"/>
       <c r="S43" s="159"/>
     </row>
     <row r="44" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="88"/>
-      <c r="B44" s="300"/>
-      <c r="C44" s="301"/>
-      <c r="D44" s="301"/>
-      <c r="E44" s="301"/>
-      <c r="F44" s="301"/>
-      <c r="G44" s="302"/>
+      <c r="B44" s="312"/>
+      <c r="C44" s="286"/>
+      <c r="D44" s="286"/>
+      <c r="E44" s="286"/>
+      <c r="F44" s="286"/>
+      <c r="G44" s="287"/>
       <c r="H44" s="31"/>
       <c r="I44" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J44" s="281"/>
-      <c r="K44" s="282"/>
-      <c r="L44" s="282"/>
-      <c r="M44" s="282"/>
-      <c r="N44" s="282"/>
-      <c r="O44" s="283"/>
-      <c r="P44" s="284"/>
-      <c r="Q44" s="284"/>
-      <c r="R44" s="285"/>
+      <c r="J44" s="305"/>
+      <c r="K44" s="306"/>
+      <c r="L44" s="306"/>
+      <c r="M44" s="306"/>
+      <c r="N44" s="306"/>
+      <c r="O44" s="307"/>
+      <c r="P44" s="308"/>
+      <c r="Q44" s="308"/>
+      <c r="R44" s="309"/>
       <c r="S44" s="159"/>
     </row>
     <row r="45" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="88"/>
-      <c r="B45" s="300"/>
-      <c r="C45" s="301"/>
-      <c r="D45" s="301"/>
-      <c r="E45" s="301"/>
-      <c r="F45" s="301"/>
-      <c r="G45" s="302"/>
+      <c r="B45" s="312"/>
+      <c r="C45" s="286"/>
+      <c r="D45" s="286"/>
+      <c r="E45" s="286"/>
+      <c r="F45" s="286"/>
+      <c r="G45" s="287"/>
       <c r="H45" s="31"/>
       <c r="I45" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J45" s="281"/>
-      <c r="K45" s="282"/>
-      <c r="L45" s="282"/>
-      <c r="M45" s="282"/>
-      <c r="N45" s="282"/>
-      <c r="O45" s="283"/>
-      <c r="P45" s="284"/>
-      <c r="Q45" s="284"/>
-      <c r="R45" s="285"/>
+      <c r="J45" s="305"/>
+      <c r="K45" s="306"/>
+      <c r="L45" s="306"/>
+      <c r="M45" s="306"/>
+      <c r="N45" s="306"/>
+      <c r="O45" s="307"/>
+      <c r="P45" s="308"/>
+      <c r="Q45" s="308"/>
+      <c r="R45" s="309"/>
       <c r="S45" s="159"/>
     </row>
     <row r="46" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="88"/>
-      <c r="B46" s="300"/>
-      <c r="C46" s="301"/>
-      <c r="D46" s="301"/>
-      <c r="E46" s="301"/>
-      <c r="F46" s="301"/>
-      <c r="G46" s="302"/>
+      <c r="B46" s="312"/>
+      <c r="C46" s="286"/>
+      <c r="D46" s="286"/>
+      <c r="E46" s="286"/>
+      <c r="F46" s="286"/>
+      <c r="G46" s="287"/>
       <c r="H46" s="31"/>
       <c r="I46" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J46" s="281"/>
-      <c r="K46" s="282"/>
-      <c r="L46" s="282"/>
-      <c r="M46" s="282"/>
-      <c r="N46" s="282"/>
-      <c r="O46" s="283"/>
-      <c r="P46" s="284"/>
-      <c r="Q46" s="284"/>
-      <c r="R46" s="285"/>
+      <c r="J46" s="305"/>
+      <c r="K46" s="306"/>
+      <c r="L46" s="306"/>
+      <c r="M46" s="306"/>
+      <c r="N46" s="306"/>
+      <c r="O46" s="307"/>
+      <c r="P46" s="308"/>
+      <c r="Q46" s="308"/>
+      <c r="R46" s="309"/>
       <c r="S46" s="159"/>
     </row>
     <row r="47" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="88"/>
-      <c r="B47" s="300"/>
-      <c r="C47" s="301"/>
-      <c r="D47" s="301"/>
-      <c r="E47" s="301"/>
-      <c r="F47" s="301"/>
-      <c r="G47" s="302"/>
+      <c r="B47" s="312"/>
+      <c r="C47" s="286"/>
+      <c r="D47" s="286"/>
+      <c r="E47" s="286"/>
+      <c r="F47" s="286"/>
+      <c r="G47" s="287"/>
       <c r="H47" s="31"/>
       <c r="I47" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J47" s="281"/>
-      <c r="K47" s="282"/>
-      <c r="L47" s="282"/>
-      <c r="M47" s="282"/>
-      <c r="N47" s="282"/>
-      <c r="O47" s="283"/>
-      <c r="P47" s="284"/>
-      <c r="Q47" s="284"/>
-      <c r="R47" s="285"/>
+      <c r="J47" s="305"/>
+      <c r="K47" s="306"/>
+      <c r="L47" s="306"/>
+      <c r="M47" s="306"/>
+      <c r="N47" s="306"/>
+      <c r="O47" s="307"/>
+      <c r="P47" s="308"/>
+      <c r="Q47" s="308"/>
+      <c r="R47" s="309"/>
       <c r="S47" s="159"/>
     </row>
     <row r="48" spans="1:19" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="88"/>
-      <c r="B48" s="300"/>
-      <c r="C48" s="301"/>
-      <c r="D48" s="301"/>
-      <c r="E48" s="301"/>
-      <c r="F48" s="301"/>
-      <c r="G48" s="302"/>
+      <c r="B48" s="312"/>
+      <c r="C48" s="286"/>
+      <c r="D48" s="286"/>
+      <c r="E48" s="286"/>
+      <c r="F48" s="286"/>
+      <c r="G48" s="287"/>
       <c r="H48" s="31"/>
       <c r="I48" s="96" t="s">
         <v>10</v>
       </c>
-      <c r="J48" s="281"/>
-      <c r="K48" s="282"/>
-      <c r="L48" s="282"/>
-      <c r="M48" s="282"/>
-      <c r="N48" s="282"/>
-      <c r="O48" s="283"/>
-      <c r="P48" s="286"/>
-      <c r="Q48" s="286"/>
-      <c r="R48" s="287"/>
+      <c r="J48" s="305"/>
+      <c r="K48" s="306"/>
+      <c r="L48" s="306"/>
+      <c r="M48" s="306"/>
+      <c r="N48" s="306"/>
+      <c r="O48" s="307"/>
+      <c r="P48" s="310"/>
+      <c r="Q48" s="310"/>
+      <c r="R48" s="311"/>
       <c r="S48" s="159"/>
     </row>
     <row r="49" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="88"/>
-      <c r="B49" s="300"/>
-      <c r="C49" s="301"/>
-      <c r="D49" s="301"/>
-      <c r="E49" s="301"/>
-      <c r="F49" s="301"/>
-      <c r="G49" s="302"/>
+      <c r="B49" s="312"/>
+      <c r="C49" s="286"/>
+      <c r="D49" s="286"/>
+      <c r="E49" s="286"/>
+      <c r="F49" s="286"/>
+      <c r="G49" s="287"/>
       <c r="H49" s="31"/>
       <c r="I49" s="29"/>
       <c r="J49" s="29"/>
@@ -12106,198 +12112,198 @@
     </row>
     <row r="50" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="88"/>
-      <c r="B50" s="300"/>
-      <c r="C50" s="301"/>
-      <c r="D50" s="301"/>
-      <c r="E50" s="301"/>
-      <c r="F50" s="301"/>
-      <c r="G50" s="302"/>
+      <c r="B50" s="312"/>
+      <c r="C50" s="286"/>
+      <c r="D50" s="286"/>
+      <c r="E50" s="286"/>
+      <c r="F50" s="286"/>
+      <c r="G50" s="287"/>
       <c r="H50" s="31"/>
-      <c r="I50" s="288" t="s">
+      <c r="I50" s="299" t="s">
         <v>186</v>
       </c>
-      <c r="J50" s="288"/>
-      <c r="K50" s="288"/>
-      <c r="L50" s="288"/>
-      <c r="M50" s="288"/>
-      <c r="N50" s="288"/>
-      <c r="O50" s="288"/>
-      <c r="P50" s="288"/>
-      <c r="Q50" s="288"/>
-      <c r="R50" s="289"/>
+      <c r="J50" s="299"/>
+      <c r="K50" s="299"/>
+      <c r="L50" s="299"/>
+      <c r="M50" s="299"/>
+      <c r="N50" s="299"/>
+      <c r="O50" s="299"/>
+      <c r="P50" s="299"/>
+      <c r="Q50" s="299"/>
+      <c r="R50" s="300"/>
       <c r="S50" s="105"/>
     </row>
     <row r="51" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="88"/>
-      <c r="B51" s="300"/>
-      <c r="C51" s="301"/>
-      <c r="D51" s="301"/>
-      <c r="E51" s="301"/>
-      <c r="F51" s="301"/>
-      <c r="G51" s="302"/>
+      <c r="B51" s="312"/>
+      <c r="C51" s="286"/>
+      <c r="D51" s="286"/>
+      <c r="E51" s="286"/>
+      <c r="F51" s="286"/>
+      <c r="G51" s="287"/>
       <c r="H51" s="31"/>
-      <c r="I51" s="270"/>
-      <c r="J51" s="270"/>
-      <c r="K51" s="270"/>
-      <c r="L51" s="270"/>
-      <c r="M51" s="270"/>
-      <c r="N51" s="270"/>
-      <c r="O51" s="270"/>
-      <c r="P51" s="270"/>
-      <c r="Q51" s="270"/>
-      <c r="R51" s="271"/>
+      <c r="I51" s="258"/>
+      <c r="J51" s="258"/>
+      <c r="K51" s="258"/>
+      <c r="L51" s="258"/>
+      <c r="M51" s="258"/>
+      <c r="N51" s="258"/>
+      <c r="O51" s="258"/>
+      <c r="P51" s="258"/>
+      <c r="Q51" s="258"/>
+      <c r="R51" s="259"/>
       <c r="S51" s="105"/>
     </row>
     <row r="52" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="88"/>
-      <c r="B52" s="300"/>
-      <c r="C52" s="301"/>
-      <c r="D52" s="301"/>
-      <c r="E52" s="301"/>
-      <c r="F52" s="301"/>
-      <c r="G52" s="302"/>
+      <c r="B52" s="312"/>
+      <c r="C52" s="286"/>
+      <c r="D52" s="286"/>
+      <c r="E52" s="286"/>
+      <c r="F52" s="286"/>
+      <c r="G52" s="287"/>
       <c r="H52" s="31"/>
       <c r="I52" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J52" s="281" t="s">
+      <c r="J52" s="305" t="s">
         <v>184</v>
       </c>
-      <c r="K52" s="282"/>
-      <c r="L52" s="282"/>
-      <c r="M52" s="282"/>
-      <c r="N52" s="282"/>
-      <c r="O52" s="283"/>
-      <c r="P52" s="240" t="s">
+      <c r="K52" s="306"/>
+      <c r="L52" s="306"/>
+      <c r="M52" s="306"/>
+      <c r="N52" s="306"/>
+      <c r="O52" s="307"/>
+      <c r="P52" s="237" t="s">
         <v>185</v>
       </c>
-      <c r="Q52" s="240"/>
-      <c r="R52" s="290"/>
+      <c r="Q52" s="237"/>
+      <c r="R52" s="323"/>
       <c r="S52" s="105"/>
     </row>
     <row r="53" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="88"/>
-      <c r="B53" s="300"/>
-      <c r="C53" s="301"/>
-      <c r="D53" s="301"/>
-      <c r="E53" s="301"/>
-      <c r="F53" s="301"/>
-      <c r="G53" s="302"/>
+      <c r="B53" s="312"/>
+      <c r="C53" s="286"/>
+      <c r="D53" s="286"/>
+      <c r="E53" s="286"/>
+      <c r="F53" s="286"/>
+      <c r="G53" s="287"/>
       <c r="H53" s="31"/>
       <c r="I53" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J53" s="281"/>
-      <c r="K53" s="282"/>
-      <c r="L53" s="282"/>
-      <c r="M53" s="282"/>
-      <c r="N53" s="282"/>
-      <c r="O53" s="283"/>
-      <c r="P53" s="284"/>
-      <c r="Q53" s="284"/>
-      <c r="R53" s="285"/>
+      <c r="J53" s="305"/>
+      <c r="K53" s="306"/>
+      <c r="L53" s="306"/>
+      <c r="M53" s="306"/>
+      <c r="N53" s="306"/>
+      <c r="O53" s="307"/>
+      <c r="P53" s="308"/>
+      <c r="Q53" s="308"/>
+      <c r="R53" s="309"/>
       <c r="S53" s="105"/>
     </row>
     <row r="54" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="88"/>
-      <c r="B54" s="300"/>
-      <c r="C54" s="301"/>
-      <c r="D54" s="301"/>
-      <c r="E54" s="301"/>
-      <c r="F54" s="301"/>
-      <c r="G54" s="302"/>
+      <c r="B54" s="312"/>
+      <c r="C54" s="286"/>
+      <c r="D54" s="286"/>
+      <c r="E54" s="286"/>
+      <c r="F54" s="286"/>
+      <c r="G54" s="287"/>
       <c r="H54" s="31"/>
       <c r="I54" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J54" s="281"/>
-      <c r="K54" s="282"/>
-      <c r="L54" s="282"/>
-      <c r="M54" s="282"/>
-      <c r="N54" s="282"/>
-      <c r="O54" s="283"/>
-      <c r="P54" s="284"/>
-      <c r="Q54" s="284"/>
-      <c r="R54" s="285"/>
+      <c r="J54" s="305"/>
+      <c r="K54" s="306"/>
+      <c r="L54" s="306"/>
+      <c r="M54" s="306"/>
+      <c r="N54" s="306"/>
+      <c r="O54" s="307"/>
+      <c r="P54" s="308"/>
+      <c r="Q54" s="308"/>
+      <c r="R54" s="309"/>
       <c r="S54" s="105"/>
     </row>
     <row r="55" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="88"/>
-      <c r="B55" s="300"/>
-      <c r="C55" s="301"/>
-      <c r="D55" s="301"/>
-      <c r="E55" s="301"/>
-      <c r="F55" s="301"/>
-      <c r="G55" s="302"/>
+      <c r="B55" s="312"/>
+      <c r="C55" s="286"/>
+      <c r="D55" s="286"/>
+      <c r="E55" s="286"/>
+      <c r="F55" s="286"/>
+      <c r="G55" s="287"/>
       <c r="H55" s="31"/>
       <c r="I55" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J55" s="281"/>
-      <c r="K55" s="282"/>
-      <c r="L55" s="282"/>
-      <c r="M55" s="282"/>
-      <c r="N55" s="282"/>
-      <c r="O55" s="283"/>
-      <c r="P55" s="284"/>
-      <c r="Q55" s="284"/>
-      <c r="R55" s="285"/>
+      <c r="J55" s="305"/>
+      <c r="K55" s="306"/>
+      <c r="L55" s="306"/>
+      <c r="M55" s="306"/>
+      <c r="N55" s="306"/>
+      <c r="O55" s="307"/>
+      <c r="P55" s="308"/>
+      <c r="Q55" s="308"/>
+      <c r="R55" s="309"/>
       <c r="S55" s="105"/>
     </row>
     <row r="56" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="88"/>
-      <c r="B56" s="300"/>
-      <c r="C56" s="301"/>
-      <c r="D56" s="301"/>
-      <c r="E56" s="301"/>
-      <c r="F56" s="301"/>
-      <c r="G56" s="302"/>
+      <c r="B56" s="312"/>
+      <c r="C56" s="286"/>
+      <c r="D56" s="286"/>
+      <c r="E56" s="286"/>
+      <c r="F56" s="286"/>
+      <c r="G56" s="287"/>
       <c r="H56" s="31"/>
       <c r="I56" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J56" s="281"/>
-      <c r="K56" s="282"/>
-      <c r="L56" s="282"/>
-      <c r="M56" s="282"/>
-      <c r="N56" s="282"/>
-      <c r="O56" s="283"/>
-      <c r="P56" s="284"/>
-      <c r="Q56" s="284"/>
-      <c r="R56" s="285"/>
+      <c r="J56" s="305"/>
+      <c r="K56" s="306"/>
+      <c r="L56" s="306"/>
+      <c r="M56" s="306"/>
+      <c r="N56" s="306"/>
+      <c r="O56" s="307"/>
+      <c r="P56" s="308"/>
+      <c r="Q56" s="308"/>
+      <c r="R56" s="309"/>
       <c r="S56" s="105"/>
     </row>
     <row r="57" spans="1:19" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="88"/>
-      <c r="B57" s="300"/>
-      <c r="C57" s="301"/>
-      <c r="D57" s="301"/>
-      <c r="E57" s="301"/>
-      <c r="F57" s="301"/>
-      <c r="G57" s="302"/>
+      <c r="B57" s="312"/>
+      <c r="C57" s="286"/>
+      <c r="D57" s="286"/>
+      <c r="E57" s="286"/>
+      <c r="F57" s="286"/>
+      <c r="G57" s="287"/>
       <c r="H57" s="31"/>
       <c r="I57" s="96" t="s">
         <v>10</v>
       </c>
-      <c r="J57" s="281"/>
-      <c r="K57" s="282"/>
-      <c r="L57" s="282"/>
-      <c r="M57" s="282"/>
-      <c r="N57" s="282"/>
-      <c r="O57" s="283"/>
-      <c r="P57" s="286"/>
-      <c r="Q57" s="286"/>
-      <c r="R57" s="287"/>
+      <c r="J57" s="305"/>
+      <c r="K57" s="306"/>
+      <c r="L57" s="306"/>
+      <c r="M57" s="306"/>
+      <c r="N57" s="306"/>
+      <c r="O57" s="307"/>
+      <c r="P57" s="310"/>
+      <c r="Q57" s="310"/>
+      <c r="R57" s="311"/>
       <c r="S57" s="105"/>
     </row>
     <row r="58" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="88"/>
-      <c r="B58" s="300"/>
-      <c r="C58" s="301"/>
-      <c r="D58" s="301"/>
-      <c r="E58" s="301"/>
-      <c r="F58" s="301"/>
-      <c r="G58" s="302"/>
+      <c r="B58" s="312"/>
+      <c r="C58" s="286"/>
+      <c r="D58" s="286"/>
+      <c r="E58" s="286"/>
+      <c r="F58" s="286"/>
+      <c r="G58" s="287"/>
       <c r="H58" s="31"/>
       <c r="I58" s="56"/>
       <c r="J58" s="56"/>
@@ -12313,25 +12319,25 @@
     </row>
     <row r="59" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="88"/>
-      <c r="B59" s="300"/>
-      <c r="C59" s="301"/>
-      <c r="D59" s="301"/>
-      <c r="E59" s="301"/>
-      <c r="F59" s="301"/>
-      <c r="G59" s="302"/>
+      <c r="B59" s="312"/>
+      <c r="C59" s="286"/>
+      <c r="D59" s="286"/>
+      <c r="E59" s="286"/>
+      <c r="F59" s="286"/>
+      <c r="G59" s="287"/>
       <c r="H59" s="31"/>
-      <c r="I59" s="288" t="s">
+      <c r="I59" s="299" t="s">
         <v>187</v>
       </c>
-      <c r="J59" s="288"/>
-      <c r="K59" s="288"/>
-      <c r="L59" s="288"/>
-      <c r="M59" s="288"/>
-      <c r="N59" s="288"/>
-      <c r="O59" s="288"/>
-      <c r="P59" s="288"/>
-      <c r="Q59" s="288"/>
-      <c r="R59" s="289"/>
+      <c r="J59" s="299"/>
+      <c r="K59" s="299"/>
+      <c r="L59" s="299"/>
+      <c r="M59" s="299"/>
+      <c r="N59" s="299"/>
+      <c r="O59" s="299"/>
+      <c r="P59" s="299"/>
+      <c r="Q59" s="299"/>
+      <c r="R59" s="300"/>
       <c r="S59" s="105"/>
     </row>
     <row r="60" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12343,49 +12349,49 @@
       <c r="F60" s="56"/>
       <c r="G60" s="56"/>
       <c r="H60" s="31"/>
-      <c r="I60" s="270"/>
-      <c r="J60" s="270"/>
-      <c r="K60" s="270"/>
-      <c r="L60" s="270"/>
-      <c r="M60" s="270"/>
-      <c r="N60" s="270"/>
-      <c r="O60" s="270"/>
-      <c r="P60" s="270"/>
-      <c r="Q60" s="270"/>
-      <c r="R60" s="271"/>
+      <c r="I60" s="258"/>
+      <c r="J60" s="258"/>
+      <c r="K60" s="258"/>
+      <c r="L60" s="258"/>
+      <c r="M60" s="258"/>
+      <c r="N60" s="258"/>
+      <c r="O60" s="258"/>
+      <c r="P60" s="258"/>
+      <c r="Q60" s="258"/>
+      <c r="R60" s="259"/>
       <c r="S60" s="105"/>
     </row>
     <row r="61" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="303" t="s">
+      <c r="A61" s="272" t="s">
         <v>188</v>
       </c>
-      <c r="B61" s="304"/>
+      <c r="B61" s="273"/>
       <c r="C61" s="97" t="s">
         <v>189</v>
       </c>
       <c r="D61" s="97" t="s">
         <v>190</v>
       </c>
-      <c r="E61" s="304"/>
-      <c r="F61" s="304"/>
-      <c r="G61" s="305"/>
+      <c r="E61" s="273"/>
+      <c r="F61" s="273"/>
+      <c r="G61" s="313"/>
       <c r="H61" s="31"/>
       <c r="I61" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J61" s="281" t="s">
+      <c r="J61" s="305" t="s">
         <v>184</v>
       </c>
-      <c r="K61" s="282"/>
-      <c r="L61" s="282"/>
-      <c r="M61" s="282"/>
-      <c r="N61" s="282"/>
-      <c r="O61" s="283"/>
-      <c r="P61" s="240" t="s">
+      <c r="K61" s="306"/>
+      <c r="L61" s="306"/>
+      <c r="M61" s="306"/>
+      <c r="N61" s="306"/>
+      <c r="O61" s="307"/>
+      <c r="P61" s="237" t="s">
         <v>185</v>
       </c>
-      <c r="Q61" s="240"/>
-      <c r="R61" s="290"/>
+      <c r="Q61" s="237"/>
+      <c r="R61" s="323"/>
       <c r="S61" s="105"/>
     </row>
     <row r="62" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12393,22 +12399,22 @@
       <c r="B62" s="8"/>
       <c r="C62" s="8"/>
       <c r="D62" s="10"/>
-      <c r="E62" s="312"/>
-      <c r="F62" s="312"/>
-      <c r="G62" s="313"/>
+      <c r="E62" s="296"/>
+      <c r="F62" s="296"/>
+      <c r="G62" s="297"/>
       <c r="H62" s="31"/>
       <c r="I62" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J62" s="281"/>
-      <c r="K62" s="282"/>
-      <c r="L62" s="282"/>
-      <c r="M62" s="282"/>
-      <c r="N62" s="282"/>
-      <c r="O62" s="283"/>
-      <c r="P62" s="284"/>
-      <c r="Q62" s="284"/>
-      <c r="R62" s="285"/>
+      <c r="J62" s="305"/>
+      <c r="K62" s="306"/>
+      <c r="L62" s="306"/>
+      <c r="M62" s="306"/>
+      <c r="N62" s="306"/>
+      <c r="O62" s="307"/>
+      <c r="P62" s="308"/>
+      <c r="Q62" s="308"/>
+      <c r="R62" s="309"/>
       <c r="S62" s="105"/>
     </row>
     <row r="63" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12416,22 +12422,22 @@
       <c r="B63" s="8"/>
       <c r="C63" s="8"/>
       <c r="D63" s="10"/>
-      <c r="E63" s="301"/>
-      <c r="F63" s="301"/>
-      <c r="G63" s="302"/>
+      <c r="E63" s="286"/>
+      <c r="F63" s="286"/>
+      <c r="G63" s="287"/>
       <c r="H63" s="31"/>
       <c r="I63" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J63" s="281"/>
-      <c r="K63" s="282"/>
-      <c r="L63" s="282"/>
-      <c r="M63" s="282"/>
-      <c r="N63" s="282"/>
-      <c r="O63" s="283"/>
-      <c r="P63" s="284"/>
-      <c r="Q63" s="284"/>
-      <c r="R63" s="285"/>
+      <c r="J63" s="305"/>
+      <c r="K63" s="306"/>
+      <c r="L63" s="306"/>
+      <c r="M63" s="306"/>
+      <c r="N63" s="306"/>
+      <c r="O63" s="307"/>
+      <c r="P63" s="308"/>
+      <c r="Q63" s="308"/>
+      <c r="R63" s="309"/>
       <c r="S63" s="105"/>
     </row>
     <row r="64" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12439,22 +12445,22 @@
       <c r="B64" s="8"/>
       <c r="C64" s="8"/>
       <c r="D64" s="10"/>
-      <c r="E64" s="301"/>
-      <c r="F64" s="301"/>
-      <c r="G64" s="302"/>
+      <c r="E64" s="286"/>
+      <c r="F64" s="286"/>
+      <c r="G64" s="287"/>
       <c r="H64" s="31"/>
       <c r="I64" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J64" s="281"/>
-      <c r="K64" s="282"/>
-      <c r="L64" s="282"/>
-      <c r="M64" s="282"/>
-      <c r="N64" s="282"/>
-      <c r="O64" s="283"/>
-      <c r="P64" s="284"/>
-      <c r="Q64" s="284"/>
-      <c r="R64" s="285"/>
+      <c r="J64" s="305"/>
+      <c r="K64" s="306"/>
+      <c r="L64" s="306"/>
+      <c r="M64" s="306"/>
+      <c r="N64" s="306"/>
+      <c r="O64" s="307"/>
+      <c r="P64" s="308"/>
+      <c r="Q64" s="308"/>
+      <c r="R64" s="309"/>
       <c r="S64" s="105"/>
     </row>
     <row r="65" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12462,22 +12468,22 @@
       <c r="B65" s="8"/>
       <c r="C65" s="8"/>
       <c r="D65" s="10"/>
-      <c r="E65" s="301"/>
-      <c r="F65" s="301"/>
-      <c r="G65" s="302"/>
+      <c r="E65" s="286"/>
+      <c r="F65" s="286"/>
+      <c r="G65" s="287"/>
       <c r="H65" s="31"/>
       <c r="I65" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="281"/>
-      <c r="K65" s="282"/>
-      <c r="L65" s="282"/>
-      <c r="M65" s="282"/>
-      <c r="N65" s="282"/>
-      <c r="O65" s="283"/>
-      <c r="P65" s="284"/>
-      <c r="Q65" s="284"/>
-      <c r="R65" s="285"/>
+      <c r="J65" s="305"/>
+      <c r="K65" s="306"/>
+      <c r="L65" s="306"/>
+      <c r="M65" s="306"/>
+      <c r="N65" s="306"/>
+      <c r="O65" s="307"/>
+      <c r="P65" s="308"/>
+      <c r="Q65" s="308"/>
+      <c r="R65" s="309"/>
       <c r="S65" s="105"/>
     </row>
     <row r="66" spans="1:19" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -12485,22 +12491,22 @@
       <c r="B66" s="8"/>
       <c r="C66" s="8"/>
       <c r="D66" s="10"/>
-      <c r="E66" s="301"/>
-      <c r="F66" s="301"/>
-      <c r="G66" s="302"/>
+      <c r="E66" s="286"/>
+      <c r="F66" s="286"/>
+      <c r="G66" s="287"/>
       <c r="H66" s="31"/>
       <c r="I66" s="96" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="281"/>
-      <c r="K66" s="282"/>
-      <c r="L66" s="282"/>
-      <c r="M66" s="282"/>
-      <c r="N66" s="282"/>
-      <c r="O66" s="283"/>
-      <c r="P66" s="286"/>
-      <c r="Q66" s="286"/>
-      <c r="R66" s="287"/>
+      <c r="J66" s="305"/>
+      <c r="K66" s="306"/>
+      <c r="L66" s="306"/>
+      <c r="M66" s="306"/>
+      <c r="N66" s="306"/>
+      <c r="O66" s="307"/>
+      <c r="P66" s="310"/>
+      <c r="Q66" s="310"/>
+      <c r="R66" s="311"/>
       <c r="S66" s="105"/>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.2">
@@ -12508,9 +12514,9 @@
       <c r="B67" s="8"/>
       <c r="C67" s="8"/>
       <c r="D67" s="10"/>
-      <c r="E67" s="301"/>
-      <c r="F67" s="301"/>
-      <c r="G67" s="302"/>
+      <c r="E67" s="286"/>
+      <c r="F67" s="286"/>
+      <c r="G67" s="287"/>
       <c r="H67" s="31"/>
       <c r="I67" s="56"/>
       <c r="J67" s="56"/>
@@ -12529,22 +12535,22 @@
       <c r="B68" s="8"/>
       <c r="C68" s="8"/>
       <c r="D68" s="10"/>
-      <c r="E68" s="301"/>
-      <c r="F68" s="301"/>
-      <c r="G68" s="302"/>
+      <c r="E68" s="286"/>
+      <c r="F68" s="286"/>
+      <c r="G68" s="287"/>
       <c r="H68" s="31"/>
-      <c r="I68" s="314" t="s">
+      <c r="I68" s="298" t="s">
         <v>161</v>
       </c>
-      <c r="J68" s="288"/>
-      <c r="K68" s="288"/>
-      <c r="L68" s="288"/>
-      <c r="M68" s="288"/>
-      <c r="N68" s="288"/>
-      <c r="O68" s="288"/>
-      <c r="P68" s="288"/>
-      <c r="Q68" s="288"/>
-      <c r="R68" s="289"/>
+      <c r="J68" s="299"/>
+      <c r="K68" s="299"/>
+      <c r="L68" s="299"/>
+      <c r="M68" s="299"/>
+      <c r="N68" s="299"/>
+      <c r="O68" s="299"/>
+      <c r="P68" s="299"/>
+      <c r="Q68" s="299"/>
+      <c r="R68" s="300"/>
       <c r="S68" s="106"/>
     </row>
     <row r="69" spans="1:19" ht="20" thickBot="1" x14ac:dyDescent="0.25">
@@ -12552,24 +12558,24 @@
       <c r="B69" s="8"/>
       <c r="C69" s="8"/>
       <c r="D69" s="10"/>
-      <c r="E69" s="301"/>
-      <c r="F69" s="301"/>
-      <c r="G69" s="302"/>
+      <c r="E69" s="286"/>
+      <c r="F69" s="286"/>
+      <c r="G69" s="287"/>
       <c r="H69" s="31"/>
-      <c r="I69" s="315" t="s">
+      <c r="I69" s="301" t="s">
         <v>191</v>
       </c>
-      <c r="J69" s="316"/>
-      <c r="K69" s="316"/>
-      <c r="L69" s="317"/>
-      <c r="M69" s="315" t="s">
+      <c r="J69" s="302"/>
+      <c r="K69" s="302"/>
+      <c r="L69" s="303"/>
+      <c r="M69" s="301" t="s">
         <v>192</v>
       </c>
-      <c r="N69" s="316"/>
-      <c r="O69" s="316"/>
-      <c r="P69" s="316"/>
-      <c r="Q69" s="316"/>
-      <c r="R69" s="318"/>
+      <c r="N69" s="302"/>
+      <c r="O69" s="302"/>
+      <c r="P69" s="302"/>
+      <c r="Q69" s="302"/>
+      <c r="R69" s="304"/>
       <c r="S69" s="106"/>
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.2">
@@ -12577,22 +12583,22 @@
       <c r="B70" s="8"/>
       <c r="C70" s="8"/>
       <c r="D70" s="10"/>
-      <c r="E70" s="301"/>
-      <c r="F70" s="301"/>
-      <c r="G70" s="302"/>
+      <c r="E70" s="286"/>
+      <c r="F70" s="286"/>
+      <c r="G70" s="287"/>
       <c r="H70" s="31"/>
-      <c r="I70" s="306"/>
-      <c r="J70" s="307"/>
-      <c r="K70" s="307"/>
-      <c r="L70" s="308"/>
-      <c r="M70" s="309" t="s">
+      <c r="I70" s="292"/>
+      <c r="J70" s="293"/>
+      <c r="K70" s="293"/>
+      <c r="L70" s="294"/>
+      <c r="M70" s="295" t="s">
         <v>166</v>
       </c>
-      <c r="N70" s="310"/>
-      <c r="O70" s="310"/>
-      <c r="P70" s="310"/>
-      <c r="Q70" s="310"/>
-      <c r="R70" s="311"/>
+      <c r="N70" s="284"/>
+      <c r="O70" s="284"/>
+      <c r="P70" s="284"/>
+      <c r="Q70" s="284"/>
+      <c r="R70" s="285"/>
       <c r="S70" s="106"/>
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.2">
@@ -12600,66 +12606,66 @@
       <c r="B71" s="8"/>
       <c r="C71" s="8"/>
       <c r="D71" s="10"/>
-      <c r="E71" s="301"/>
-      <c r="F71" s="301"/>
-      <c r="G71" s="302"/>
+      <c r="E71" s="286"/>
+      <c r="F71" s="286"/>
+      <c r="G71" s="287"/>
       <c r="H71" s="31"/>
-      <c r="I71" s="319"/>
-      <c r="J71" s="320"/>
-      <c r="K71" s="320"/>
-      <c r="L71" s="321"/>
-      <c r="M71" s="322" t="s">
+      <c r="I71" s="269"/>
+      <c r="J71" s="270"/>
+      <c r="K71" s="270"/>
+      <c r="L71" s="271"/>
+      <c r="M71" s="288" t="s">
         <v>169</v>
       </c>
-      <c r="N71" s="323"/>
-      <c r="O71" s="323"/>
-      <c r="P71" s="323"/>
-      <c r="Q71" s="323"/>
-      <c r="R71" s="324"/>
+      <c r="N71" s="275"/>
+      <c r="O71" s="275"/>
+      <c r="P71" s="275"/>
+      <c r="Q71" s="275"/>
+      <c r="R71" s="276"/>
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A72" s="94"/>
       <c r="B72" s="8"/>
       <c r="C72" s="8"/>
       <c r="D72" s="10"/>
-      <c r="E72" s="301"/>
-      <c r="F72" s="301"/>
-      <c r="G72" s="302"/>
+      <c r="E72" s="286"/>
+      <c r="F72" s="286"/>
+      <c r="G72" s="287"/>
       <c r="H72" s="31"/>
-      <c r="I72" s="319"/>
-      <c r="J72" s="320"/>
-      <c r="K72" s="320"/>
-      <c r="L72" s="321"/>
-      <c r="M72" s="325" t="s">
+      <c r="I72" s="269"/>
+      <c r="J72" s="270"/>
+      <c r="K72" s="270"/>
+      <c r="L72" s="271"/>
+      <c r="M72" s="289" t="s">
         <v>193</v>
       </c>
-      <c r="N72" s="326"/>
-      <c r="O72" s="326"/>
-      <c r="P72" s="326"/>
-      <c r="Q72" s="326"/>
-      <c r="R72" s="327"/>
+      <c r="N72" s="290"/>
+      <c r="O72" s="290"/>
+      <c r="P72" s="290"/>
+      <c r="Q72" s="290"/>
+      <c r="R72" s="291"/>
       <c r="S72" s="107"/>
     </row>
     <row r="73" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B73" s="8"/>
       <c r="C73" s="8"/>
       <c r="D73" s="10"/>
-      <c r="E73" s="301"/>
-      <c r="F73" s="301"/>
-      <c r="G73" s="302"/>
+      <c r="E73" s="286"/>
+      <c r="F73" s="286"/>
+      <c r="G73" s="287"/>
       <c r="H73" s="31"/>
-      <c r="I73" s="319"/>
-      <c r="J73" s="320"/>
-      <c r="K73" s="320"/>
-      <c r="L73" s="321"/>
-      <c r="M73" s="322" t="s">
+      <c r="I73" s="269"/>
+      <c r="J73" s="270"/>
+      <c r="K73" s="270"/>
+      <c r="L73" s="271"/>
+      <c r="M73" s="288" t="s">
         <v>194</v>
       </c>
-      <c r="N73" s="323"/>
-      <c r="O73" s="323"/>
-      <c r="P73" s="323"/>
-      <c r="Q73" s="323"/>
-      <c r="R73" s="324"/>
+      <c r="N73" s="275"/>
+      <c r="O73" s="275"/>
+      <c r="P73" s="275"/>
+      <c r="Q73" s="275"/>
+      <c r="R73" s="276"/>
     </row>
     <row r="74" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="56"/>
@@ -12670,10 +12676,10 @@
       <c r="F74" s="56"/>
       <c r="G74" s="56"/>
       <c r="H74" s="31"/>
-      <c r="I74" s="319"/>
-      <c r="J74" s="320"/>
-      <c r="K74" s="320"/>
-      <c r="L74" s="321"/>
+      <c r="I74" s="269"/>
+      <c r="J74" s="270"/>
+      <c r="K74" s="270"/>
+      <c r="L74" s="271"/>
       <c r="M74" s="108"/>
       <c r="N74" s="108"/>
       <c r="O74" s="108"/>
@@ -12688,16 +12694,16 @@
       </c>
       <c r="C75" s="64"/>
       <c r="D75" s="65"/>
-      <c r="E75" s="303" t="s">
+      <c r="E75" s="272" t="s">
         <v>196</v>
       </c>
-      <c r="F75" s="304"/>
-      <c r="G75" s="304"/>
+      <c r="F75" s="273"/>
+      <c r="G75" s="273"/>
       <c r="H75" s="31"/>
-      <c r="I75" s="319"/>
-      <c r="J75" s="320"/>
-      <c r="K75" s="320"/>
-      <c r="L75" s="321"/>
+      <c r="I75" s="269"/>
+      <c r="J75" s="270"/>
+      <c r="K75" s="270"/>
+      <c r="L75" s="271"/>
       <c r="M75" s="109"/>
       <c r="N75" s="109"/>
       <c r="O75" s="109"/>
@@ -12712,14 +12718,14 @@
       </c>
       <c r="C76" s="61"/>
       <c r="D76" s="62"/>
-      <c r="E76" s="335"/>
-      <c r="F76" s="310"/>
-      <c r="G76" s="311"/>
+      <c r="E76" s="283"/>
+      <c r="F76" s="284"/>
+      <c r="G76" s="285"/>
       <c r="H76" s="31"/>
-      <c r="I76" s="319"/>
-      <c r="J76" s="320"/>
-      <c r="K76" s="320"/>
-      <c r="L76" s="321"/>
+      <c r="I76" s="269"/>
+      <c r="J76" s="270"/>
+      <c r="K76" s="270"/>
+      <c r="L76" s="271"/>
       <c r="M76" s="108"/>
       <c r="N76" s="108"/>
       <c r="O76" s="108"/>
@@ -12734,14 +12740,14 @@
       </c>
       <c r="C77" s="58"/>
       <c r="D77" s="52"/>
-      <c r="E77" s="328"/>
-      <c r="F77" s="323"/>
-      <c r="G77" s="324"/>
+      <c r="E77" s="274"/>
+      <c r="F77" s="275"/>
+      <c r="G77" s="276"/>
       <c r="H77" s="31"/>
-      <c r="I77" s="319"/>
-      <c r="J77" s="320"/>
-      <c r="K77" s="320"/>
-      <c r="L77" s="321"/>
+      <c r="I77" s="269"/>
+      <c r="J77" s="270"/>
+      <c r="K77" s="270"/>
+      <c r="L77" s="271"/>
       <c r="M77" s="108"/>
       <c r="N77" s="108"/>
       <c r="O77" s="108"/>
@@ -12756,14 +12762,14 @@
       </c>
       <c r="C78" s="58"/>
       <c r="D78" s="52"/>
-      <c r="E78" s="328"/>
-      <c r="F78" s="323"/>
-      <c r="G78" s="324"/>
+      <c r="E78" s="274"/>
+      <c r="F78" s="275"/>
+      <c r="G78" s="276"/>
       <c r="H78" s="31"/>
-      <c r="I78" s="319"/>
-      <c r="J78" s="320"/>
-      <c r="K78" s="320"/>
-      <c r="L78" s="321"/>
+      <c r="I78" s="269"/>
+      <c r="J78" s="270"/>
+      <c r="K78" s="270"/>
+      <c r="L78" s="271"/>
       <c r="M78" s="108"/>
       <c r="N78" s="108"/>
       <c r="O78" s="108"/>
@@ -12778,14 +12784,14 @@
       </c>
       <c r="C79" s="58"/>
       <c r="D79" s="52"/>
-      <c r="E79" s="328"/>
-      <c r="F79" s="323"/>
-      <c r="G79" s="324"/>
+      <c r="E79" s="274"/>
+      <c r="F79" s="275"/>
+      <c r="G79" s="276"/>
       <c r="H79" s="31"/>
-      <c r="I79" s="319"/>
-      <c r="J79" s="320"/>
-      <c r="K79" s="320"/>
-      <c r="L79" s="321"/>
+      <c r="I79" s="269"/>
+      <c r="J79" s="270"/>
+      <c r="K79" s="270"/>
+      <c r="L79" s="271"/>
       <c r="M79" s="109"/>
       <c r="N79" s="109"/>
       <c r="O79" s="109"/>
@@ -12800,14 +12806,14 @@
       </c>
       <c r="C80" s="59"/>
       <c r="D80" s="53"/>
-      <c r="E80" s="329"/>
-      <c r="F80" s="330"/>
-      <c r="G80" s="331"/>
+      <c r="E80" s="277"/>
+      <c r="F80" s="278"/>
+      <c r="G80" s="279"/>
       <c r="H80" s="32"/>
-      <c r="I80" s="332"/>
-      <c r="J80" s="333"/>
-      <c r="K80" s="333"/>
-      <c r="L80" s="334"/>
+      <c r="I80" s="280"/>
+      <c r="J80" s="281"/>
+      <c r="K80" s="281"/>
+      <c r="L80" s="282"/>
       <c r="M80" s="110"/>
       <c r="N80" s="110"/>
       <c r="O80" s="110"/>
@@ -12817,28 +12823,80 @@
     </row>
   </sheetData>
   <mergeCells count="117">
-    <mergeCell ref="I74:L74"/>
-    <mergeCell ref="E75:G75"/>
-    <mergeCell ref="I75:L75"/>
-    <mergeCell ref="E79:G79"/>
-    <mergeCell ref="I79:L79"/>
-    <mergeCell ref="E80:G80"/>
-    <mergeCell ref="I80:L80"/>
-    <mergeCell ref="E76:G76"/>
-    <mergeCell ref="I76:L76"/>
-    <mergeCell ref="E77:G77"/>
-    <mergeCell ref="I77:L77"/>
-    <mergeCell ref="E78:G78"/>
-    <mergeCell ref="I78:L78"/>
-    <mergeCell ref="E71:G71"/>
-    <mergeCell ref="I71:L71"/>
-    <mergeCell ref="M71:R71"/>
-    <mergeCell ref="E72:G72"/>
-    <mergeCell ref="I72:L72"/>
-    <mergeCell ref="M72:R72"/>
-    <mergeCell ref="E73:G73"/>
-    <mergeCell ref="I73:L73"/>
-    <mergeCell ref="M73:R73"/>
+    <mergeCell ref="J53:O53"/>
+    <mergeCell ref="P53:R53"/>
+    <mergeCell ref="J54:O54"/>
+    <mergeCell ref="P54:R54"/>
+    <mergeCell ref="P46:R46"/>
+    <mergeCell ref="P47:R47"/>
+    <mergeCell ref="P48:R48"/>
+    <mergeCell ref="P62:R62"/>
+    <mergeCell ref="J63:O63"/>
+    <mergeCell ref="P63:R63"/>
+    <mergeCell ref="J55:O55"/>
+    <mergeCell ref="P55:R55"/>
+    <mergeCell ref="J56:O56"/>
+    <mergeCell ref="P56:R56"/>
+    <mergeCell ref="J57:O57"/>
+    <mergeCell ref="P57:R57"/>
+    <mergeCell ref="I59:R60"/>
+    <mergeCell ref="J61:O61"/>
+    <mergeCell ref="P61:R61"/>
+    <mergeCell ref="J44:O44"/>
+    <mergeCell ref="J45:O45"/>
+    <mergeCell ref="J46:O46"/>
+    <mergeCell ref="J47:O47"/>
+    <mergeCell ref="J48:O48"/>
+    <mergeCell ref="P43:R43"/>
+    <mergeCell ref="P44:R44"/>
+    <mergeCell ref="P45:R45"/>
+    <mergeCell ref="J52:O52"/>
+    <mergeCell ref="P52:R52"/>
+    <mergeCell ref="A41:F42"/>
+    <mergeCell ref="I41:R42"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="I1:R1"/>
+    <mergeCell ref="I24:R24"/>
+    <mergeCell ref="I27:R27"/>
+    <mergeCell ref="I32:R32"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="E43:G43"/>
+    <mergeCell ref="J43:O43"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="E45:G45"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="E46:G46"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="E47:G47"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="E48:G48"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="E49:G49"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="E50:G50"/>
+    <mergeCell ref="I50:R51"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="E51:G51"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="E52:G52"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="E53:G53"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="E54:G54"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="E55:G55"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="E56:G56"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="E58:G58"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="E59:G59"/>
     <mergeCell ref="E70:G70"/>
     <mergeCell ref="I70:L70"/>
     <mergeCell ref="M70:R70"/>
@@ -12860,80 +12918,28 @@
     <mergeCell ref="J66:O66"/>
     <mergeCell ref="P66:R66"/>
     <mergeCell ref="J62:O62"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="E53:G53"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="E54:G54"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="E61:G61"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="E55:G55"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="E56:G56"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="E57:G57"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="E58:G58"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="E59:G59"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="E49:G49"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="E50:G50"/>
-    <mergeCell ref="I50:R51"/>
-    <mergeCell ref="B51:D51"/>
-    <mergeCell ref="E51:G51"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="E52:G52"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="E45:G45"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="E46:G46"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="E47:G47"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="E48:G48"/>
-    <mergeCell ref="A41:F42"/>
-    <mergeCell ref="I41:R42"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="I1:R1"/>
-    <mergeCell ref="I24:R24"/>
-    <mergeCell ref="I27:R27"/>
-    <mergeCell ref="I32:R32"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="E43:G43"/>
-    <mergeCell ref="J43:O43"/>
-    <mergeCell ref="J44:O44"/>
-    <mergeCell ref="J45:O45"/>
-    <mergeCell ref="J46:O46"/>
-    <mergeCell ref="J47:O47"/>
-    <mergeCell ref="J48:O48"/>
-    <mergeCell ref="P43:R43"/>
-    <mergeCell ref="P44:R44"/>
-    <mergeCell ref="P45:R45"/>
-    <mergeCell ref="J52:O52"/>
-    <mergeCell ref="P52:R52"/>
-    <mergeCell ref="J53:O53"/>
-    <mergeCell ref="P53:R53"/>
-    <mergeCell ref="J54:O54"/>
-    <mergeCell ref="P54:R54"/>
-    <mergeCell ref="P46:R46"/>
-    <mergeCell ref="P47:R47"/>
-    <mergeCell ref="P48:R48"/>
-    <mergeCell ref="P62:R62"/>
-    <mergeCell ref="J63:O63"/>
-    <mergeCell ref="P63:R63"/>
-    <mergeCell ref="J55:O55"/>
-    <mergeCell ref="P55:R55"/>
-    <mergeCell ref="J56:O56"/>
-    <mergeCell ref="P56:R56"/>
-    <mergeCell ref="J57:O57"/>
-    <mergeCell ref="P57:R57"/>
-    <mergeCell ref="I59:R60"/>
-    <mergeCell ref="J61:O61"/>
-    <mergeCell ref="P61:R61"/>
+    <mergeCell ref="E71:G71"/>
+    <mergeCell ref="I71:L71"/>
+    <mergeCell ref="M71:R71"/>
+    <mergeCell ref="E72:G72"/>
+    <mergeCell ref="I72:L72"/>
+    <mergeCell ref="M72:R72"/>
+    <mergeCell ref="E73:G73"/>
+    <mergeCell ref="I73:L73"/>
+    <mergeCell ref="M73:R73"/>
+    <mergeCell ref="I74:L74"/>
+    <mergeCell ref="E75:G75"/>
+    <mergeCell ref="I75:L75"/>
+    <mergeCell ref="E79:G79"/>
+    <mergeCell ref="I79:L79"/>
+    <mergeCell ref="E80:G80"/>
+    <mergeCell ref="I80:L80"/>
+    <mergeCell ref="E76:G76"/>
+    <mergeCell ref="I76:L76"/>
+    <mergeCell ref="E77:G77"/>
+    <mergeCell ref="I77:L77"/>
+    <mergeCell ref="E78:G78"/>
+    <mergeCell ref="I78:L78"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="75" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -12970,16 +12976,16 @@
   <sheetData>
     <row r="1" spans="1:8" s="112" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="111"/>
-      <c r="B1" s="339" t="s">
+      <c r="B1" s="327" t="s">
         <v>197</v>
       </c>
-      <c r="C1" s="339"/>
-      <c r="D1" s="339"/>
-      <c r="E1" s="339"/>
+      <c r="C1" s="327"/>
+      <c r="D1" s="327"/>
+      <c r="E1" s="327"/>
     </row>
     <row r="2" spans="1:8" s="113" customFormat="1" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="340"/>
-      <c r="C2" s="341"/>
+      <c r="B2" s="328"/>
+      <c r="C2" s="329"/>
       <c r="D2" s="114" t="s">
         <v>198</v>
       </c>
@@ -12989,8 +12995,8 @@
       <c r="H2" s="118"/>
     </row>
     <row r="3" spans="1:8" s="113" customFormat="1" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="342"/>
-      <c r="C3" s="343"/>
+      <c r="B3" s="330"/>
+      <c r="C3" s="331"/>
       <c r="D3" s="119" t="s">
         <v>199</v>
       </c>
@@ -12999,8 +13005,8 @@
       <c r="H3" s="118"/>
     </row>
     <row r="4" spans="1:8" s="113" customFormat="1" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="342"/>
-      <c r="C4" s="343"/>
+      <c r="B4" s="330"/>
+      <c r="C4" s="331"/>
       <c r="D4" s="119" t="s">
         <v>189</v>
       </c>
@@ -13009,16 +13015,16 @@
       <c r="H4" s="118"/>
     </row>
     <row r="5" spans="1:8" s="113" customFormat="1" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="342"/>
-      <c r="C5" s="343"/>
+      <c r="B5" s="330"/>
+      <c r="C5" s="331"/>
       <c r="D5" s="119" t="s">
         <v>200</v>
       </c>
       <c r="E5" s="121"/>
     </row>
     <row r="6" spans="1:8" s="122" customFormat="1" ht="13.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="344"/>
-      <c r="C6" s="345"/>
+      <c r="B6" s="332"/>
+      <c r="C6" s="333"/>
       <c r="D6" s="123"/>
       <c r="E6" s="124"/>
       <c r="F6" s="113"/>
@@ -13036,7 +13042,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B8" s="346" t="s">
+      <c r="B8" s="334" t="s">
         <v>204</v>
       </c>
       <c r="C8" s="131">
@@ -13048,7 +13054,7 @@
       <c r="E8" s="133"/>
     </row>
     <row r="9" spans="1:8" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B9" s="347"/>
+      <c r="B9" s="335"/>
       <c r="C9" s="131">
         <v>2</v>
       </c>
@@ -13058,7 +13064,7 @@
       <c r="E9" s="133"/>
     </row>
     <row r="10" spans="1:8" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B10" s="347"/>
+      <c r="B10" s="335"/>
       <c r="C10" s="131">
         <v>3</v>
       </c>
@@ -13068,7 +13074,7 @@
       <c r="E10" s="133"/>
     </row>
     <row r="11" spans="1:8" s="130" customFormat="1" ht="34" x14ac:dyDescent="0.25">
-      <c r="B11" s="347"/>
+      <c r="B11" s="335"/>
       <c r="C11" s="131">
         <v>4</v>
       </c>
@@ -13078,7 +13084,7 @@
       <c r="E11" s="133"/>
     </row>
     <row r="12" spans="1:8" s="130" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="347"/>
+      <c r="B12" s="335"/>
       <c r="C12" s="131">
         <v>5</v>
       </c>
@@ -13088,13 +13094,13 @@
       <c r="E12" s="133"/>
     </row>
     <row r="13" spans="1:8" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="348"/>
+      <c r="B13" s="336"/>
       <c r="C13" s="136"/>
       <c r="D13" s="137"/>
       <c r="E13" s="138"/>
     </row>
     <row r="14" spans="1:8" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B14" s="349" t="s">
+      <c r="B14" s="337" t="s">
         <v>210</v>
       </c>
       <c r="C14" s="139">
@@ -13106,7 +13112,7 @@
       <c r="E14" s="141"/>
     </row>
     <row r="15" spans="1:8" s="130" customFormat="1" ht="34" x14ac:dyDescent="0.25">
-      <c r="B15" s="350"/>
+      <c r="B15" s="338"/>
       <c r="C15" s="142">
         <v>7</v>
       </c>
@@ -13116,19 +13122,19 @@
       <c r="E15" s="133"/>
     </row>
     <row r="16" spans="1:8" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="350"/>
+      <c r="B16" s="338"/>
       <c r="C16" s="142"/>
       <c r="D16" s="134"/>
       <c r="E16" s="133"/>
     </row>
     <row r="17" spans="2:5" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="351"/>
+      <c r="B17" s="339"/>
       <c r="C17" s="136"/>
       <c r="D17" s="137"/>
       <c r="E17" s="138"/>
     </row>
     <row r="18" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B18" s="349" t="s">
+      <c r="B18" s="337" t="s">
         <v>213</v>
       </c>
       <c r="C18" s="131">
@@ -13140,7 +13146,7 @@
       <c r="E18" s="141"/>
     </row>
     <row r="19" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B19" s="350"/>
+      <c r="B19" s="338"/>
       <c r="C19" s="131">
         <v>9</v>
       </c>
@@ -13152,7 +13158,7 @@
       </c>
     </row>
     <row r="20" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B20" s="350"/>
+      <c r="B20" s="338"/>
       <c r="C20" s="131">
         <v>10</v>
       </c>
@@ -13162,7 +13168,7 @@
       <c r="E20" s="133"/>
     </row>
     <row r="21" spans="2:5" s="130" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="350"/>
+      <c r="B21" s="338"/>
       <c r="C21" s="131">
         <v>11</v>
       </c>
@@ -13172,13 +13178,13 @@
       <c r="E21" s="133"/>
     </row>
     <row r="22" spans="2:5" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="351"/>
+      <c r="B22" s="339"/>
       <c r="C22" s="136"/>
       <c r="D22" s="137"/>
       <c r="E22" s="138"/>
     </row>
     <row r="23" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B23" s="336" t="s">
+      <c r="B23" s="324" t="s">
         <v>219</v>
       </c>
       <c r="C23" s="131">
@@ -13192,7 +13198,7 @@
       </c>
     </row>
     <row r="24" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B24" s="337"/>
+      <c r="B24" s="325"/>
       <c r="C24" s="131">
         <v>13</v>
       </c>
@@ -13204,7 +13210,7 @@
       </c>
     </row>
     <row r="25" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B25" s="337"/>
+      <c r="B25" s="325"/>
       <c r="C25" s="131">
         <v>14</v>
       </c>
@@ -13214,7 +13220,7 @@
       <c r="E25" s="133"/>
     </row>
     <row r="26" spans="2:5" s="130" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="337"/>
+      <c r="B26" s="325"/>
       <c r="C26" s="131">
         <v>15</v>
       </c>
@@ -13224,13 +13230,13 @@
       <c r="E26" s="133"/>
     </row>
     <row r="27" spans="2:5" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="338"/>
+      <c r="B27" s="326"/>
       <c r="C27" s="136"/>
       <c r="D27" s="137"/>
       <c r="E27" s="138"/>
     </row>
     <row r="28" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B28" s="336" t="s">
+      <c r="B28" s="324" t="s">
         <v>226</v>
       </c>
       <c r="C28" s="131">
@@ -13242,7 +13248,7 @@
       <c r="E28" s="133"/>
     </row>
     <row r="29" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B29" s="337"/>
+      <c r="B29" s="325"/>
       <c r="C29" s="144">
         <v>17</v>
       </c>
@@ -13254,7 +13260,7 @@
       </c>
     </row>
     <row r="30" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B30" s="337"/>
+      <c r="B30" s="325"/>
       <c r="C30" s="144">
         <v>18</v>
       </c>
@@ -13266,7 +13272,7 @@
       </c>
     </row>
     <row r="31" spans="2:5" s="130" customFormat="1" ht="34" x14ac:dyDescent="0.25">
-      <c r="B31" s="337"/>
+      <c r="B31" s="325"/>
       <c r="C31" s="131">
         <v>19</v>
       </c>
@@ -13276,7 +13282,7 @@
       <c r="E31" s="141"/>
     </row>
     <row r="32" spans="2:5" s="130" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="337"/>
+      <c r="B32" s="325"/>
       <c r="C32" s="131">
         <v>20</v>
       </c>
@@ -13286,7 +13292,7 @@
       <c r="E32" s="133"/>
     </row>
     <row r="33" spans="2:5" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="337"/>
+      <c r="B33" s="325"/>
       <c r="C33" s="146"/>
       <c r="D33" s="146"/>
       <c r="E33" s="147"/>
@@ -13378,7 +13384,7 @@
     <col min="11" max="11" width="1.33203125" style="5" customWidth="1"/>
     <col min="12" max="12" width="3" style="5" customWidth="1"/>
     <col min="13" max="13" width="30.6640625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="1.1640625" style="5" customWidth="1"/>
+    <col min="14" max="14" width="0.83203125" style="5" customWidth="1"/>
     <col min="15" max="15" width="4.1640625" style="5" customWidth="1"/>
     <col min="16" max="16" width="38.83203125" style="5" customWidth="1"/>
     <col min="17" max="17" width="21.5" style="5" customWidth="1"/>
@@ -13416,12 +13422,12 @@
       <c r="J1" s="183" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="213"/>
-      <c r="L1" s="224" t="s">
+      <c r="K1" s="245"/>
+      <c r="L1" s="250" t="s">
         <v>234</v>
       </c>
-      <c r="M1" s="225"/>
-      <c r="N1" s="232"/>
+      <c r="M1" s="251"/>
+      <c r="N1" s="343"/>
       <c r="O1" s="184" t="s">
         <v>178</v>
       </c>
@@ -13439,19 +13445,19 @@
       </c>
       <c r="C2" s="165"/>
       <c r="D2" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" s="196" t="b">
         <v>0</v>
@@ -13459,17 +13465,17 @@
       <c r="J2" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K2" s="214"/>
+      <c r="K2" s="246"/>
       <c r="L2" s="202" t="b">
         <v>0</v>
       </c>
       <c r="M2" s="172"/>
-      <c r="N2" s="233"/>
-      <c r="O2" s="226" t="s">
+      <c r="N2" s="344"/>
+      <c r="O2" s="252" t="s">
         <v>237</v>
       </c>
-      <c r="P2" s="227"/>
-      <c r="Q2" s="228"/>
+      <c r="P2" s="253"/>
+      <c r="Q2" s="254"/>
     </row>
     <row r="3" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="170"/>
@@ -13478,19 +13484,19 @@
       </c>
       <c r="C3" s="165"/>
       <c r="D3" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" s="196" t="b">
         <v>0</v>
@@ -13498,12 +13504,12 @@
       <c r="J3" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K3" s="214"/>
+      <c r="K3" s="246"/>
       <c r="L3" s="202" t="b">
         <v>0</v>
       </c>
       <c r="M3" s="172"/>
-      <c r="N3" s="233"/>
+      <c r="N3" s="344"/>
       <c r="O3" s="177"/>
       <c r="P3" s="164" t="s">
         <v>239</v>
@@ -13517,19 +13523,19 @@
       </c>
       <c r="C4" s="165"/>
       <c r="D4" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" s="196" t="b">
         <v>0</v>
@@ -13537,12 +13543,12 @@
       <c r="J4" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K4" s="214"/>
+      <c r="K4" s="246"/>
       <c r="L4" s="202" t="b">
         <v>0</v>
       </c>
       <c r="M4" s="172"/>
-      <c r="N4" s="233"/>
+      <c r="N4" s="344"/>
       <c r="O4" s="177"/>
       <c r="P4" s="164" t="s">
         <v>241</v>
@@ -13556,19 +13562,19 @@
       </c>
       <c r="C5" s="165"/>
       <c r="D5" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" s="196" t="b">
         <v>0</v>
@@ -13576,38 +13582,38 @@
       <c r="J5" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K5" s="214"/>
+      <c r="K5" s="246"/>
       <c r="L5" s="202" t="b">
         <v>0</v>
       </c>
       <c r="M5" s="172"/>
-      <c r="N5" s="233"/>
-      <c r="O5" s="229" t="s">
+      <c r="N5" s="344"/>
+      <c r="O5" s="255" t="s">
         <v>243</v>
       </c>
-      <c r="P5" s="230"/>
-      <c r="Q5" s="231"/>
-    </row>
-    <row r="6" spans="1:17" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P5" s="256"/>
+      <c r="Q5" s="257"/>
+    </row>
+    <row r="6" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="170"/>
       <c r="B6" s="194" t="s">
         <v>244</v>
       </c>
       <c r="C6" s="165"/>
       <c r="D6" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" s="196" t="b">
         <v>0</v>
@@ -13615,38 +13621,38 @@
       <c r="J6" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K6" s="214"/>
+      <c r="K6" s="246"/>
       <c r="L6" s="202" t="b">
         <v>0</v>
       </c>
       <c r="M6" s="172"/>
-      <c r="N6" s="233"/>
+      <c r="N6" s="344"/>
       <c r="O6" s="187"/>
       <c r="P6" s="204" t="s">
         <v>245</v>
       </c>
       <c r="Q6" s="189"/>
     </row>
-    <row r="7" spans="1:17" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="170"/>
       <c r="B7" s="194" t="s">
         <v>246</v>
       </c>
       <c r="C7" s="165"/>
       <c r="D7" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H7" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" s="196" t="b">
         <v>0</v>
@@ -13654,12 +13660,12 @@
       <c r="J7" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K7" s="214"/>
+      <c r="K7" s="246"/>
       <c r="L7" s="202" t="b">
         <v>0</v>
       </c>
       <c r="M7" s="172"/>
-      <c r="N7" s="233"/>
+      <c r="N7" s="344"/>
       <c r="O7" s="177"/>
       <c r="P7" s="164" t="s">
         <v>247</v>
@@ -13673,19 +13679,19 @@
       </c>
       <c r="C8" s="165"/>
       <c r="D8" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="196" t="b">
         <v>0</v>
@@ -13693,38 +13699,38 @@
       <c r="J8" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K8" s="214"/>
+      <c r="K8" s="246"/>
       <c r="L8" s="202" t="b">
         <v>0</v>
       </c>
       <c r="M8" s="186"/>
-      <c r="N8" s="233"/>
+      <c r="N8" s="344"/>
       <c r="O8" s="170"/>
       <c r="P8" s="164" t="s">
         <v>249</v>
       </c>
       <c r="Q8" s="162"/>
     </row>
-    <row r="9" spans="1:17" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="170"/>
       <c r="B9" s="194" t="s">
         <v>250</v>
       </c>
       <c r="C9" s="165"/>
       <c r="D9" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" s="196" t="b">
         <v>0</v>
@@ -13732,17 +13738,17 @@
       <c r="J9" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K9" s="214"/>
+      <c r="K9" s="246"/>
       <c r="L9" s="202" t="b">
         <v>0</v>
       </c>
       <c r="M9" s="186"/>
-      <c r="N9" s="233"/>
-      <c r="O9" s="229" t="s">
+      <c r="N9" s="344"/>
+      <c r="O9" s="255" t="s">
         <v>251</v>
       </c>
-      <c r="P9" s="230"/>
-      <c r="Q9" s="231"/>
+      <c r="P9" s="256"/>
+      <c r="Q9" s="257"/>
     </row>
     <row r="10" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="170"/>
@@ -13751,16 +13757,16 @@
       </c>
       <c r="C10" s="165"/>
       <c r="D10" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="196" t="b">
         <v>0</v>
@@ -13771,12 +13777,12 @@
       <c r="J10" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K10" s="214"/>
+      <c r="K10" s="246"/>
       <c r="L10" s="202" t="b">
         <v>0</v>
       </c>
       <c r="M10" s="186"/>
-      <c r="N10" s="233"/>
+      <c r="N10" s="344"/>
       <c r="O10" s="177"/>
       <c r="P10" s="164"/>
       <c r="Q10" s="162"/>
@@ -13788,19 +13794,19 @@
       </c>
       <c r="C11" s="165"/>
       <c r="D11" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11" s="196" t="b">
         <v>0</v>
@@ -13808,12 +13814,12 @@
       <c r="J11" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K11" s="214"/>
+      <c r="K11" s="246"/>
       <c r="L11" s="202" t="b">
         <v>0</v>
       </c>
       <c r="M11" s="172"/>
-      <c r="N11" s="233"/>
+      <c r="N11" s="344"/>
       <c r="O11" s="177"/>
       <c r="P11" s="164"/>
       <c r="Q11" s="162"/>
@@ -13825,16 +13831,16 @@
       </c>
       <c r="C12" s="165"/>
       <c r="D12" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" s="196" t="b">
         <v>0</v>
@@ -13845,36 +13851,36 @@
       <c r="J12" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K12" s="214"/>
+      <c r="K12" s="246"/>
       <c r="L12" s="202" t="b">
         <v>0</v>
       </c>
       <c r="M12" s="172"/>
-      <c r="N12" s="233"/>
+      <c r="N12" s="344"/>
       <c r="O12" s="170"/>
       <c r="P12" s="164"/>
       <c r="Q12" s="162"/>
     </row>
-    <row r="13" spans="1:17" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="170"/>
       <c r="B13" s="194" t="s">
         <v>255</v>
       </c>
       <c r="C13" s="165"/>
       <c r="D13" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="196" t="b">
         <v>0</v>
@@ -13882,17 +13888,19 @@
       <c r="J13" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K13" s="214"/>
-      <c r="L13" s="202"/>
+      <c r="K13" s="246"/>
+      <c r="L13" s="202" t="b">
+        <v>0</v>
+      </c>
       <c r="M13" s="172"/>
-      <c r="N13" s="233"/>
-      <c r="O13" s="229" t="s">
+      <c r="N13" s="344"/>
+      <c r="O13" s="255" t="s">
         <v>256</v>
       </c>
-      <c r="P13" s="230"/>
-      <c r="Q13" s="231"/>
-    </row>
-    <row r="14" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P13" s="256"/>
+      <c r="Q13" s="257"/>
+    </row>
+    <row r="14" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="170"/>
       <c r="C14" s="165"/>
       <c r="D14" s="195" t="b">
@@ -13916,25 +13924,25 @@
       <c r="J14" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K14" s="214"/>
+      <c r="K14" s="246"/>
       <c r="L14" s="202"/>
       <c r="M14" s="172"/>
-      <c r="N14" s="233"/>
+      <c r="N14" s="344"/>
       <c r="O14" s="177"/>
       <c r="P14" s="164"/>
       <c r="Q14" s="162"/>
     </row>
-    <row r="15" spans="1:17" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="170"/>
       <c r="B15" s="194" t="s">
         <v>257</v>
       </c>
       <c r="C15" s="165"/>
       <c r="D15" s="195" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" s="196" t="b">
         <v>0</v>
@@ -13951,10 +13959,10 @@
       <c r="J15" s="197" t="b">
         <v>0</v>
       </c>
-      <c r="K15" s="214"/>
+      <c r="K15" s="246"/>
       <c r="L15" s="202"/>
       <c r="M15" s="172"/>
-      <c r="N15" s="233"/>
+      <c r="N15" s="344"/>
       <c r="O15" s="177"/>
       <c r="P15" s="164"/>
       <c r="Q15" s="162"/>
@@ -13984,96 +13992,96 @@
       <c r="J16" s="201" t="b">
         <v>0</v>
       </c>
-      <c r="K16" s="214"/>
+      <c r="K16" s="246"/>
       <c r="L16" s="203"/>
       <c r="M16" s="176"/>
-      <c r="N16" s="233"/>
+      <c r="N16" s="344"/>
       <c r="O16" s="178"/>
       <c r="P16" s="175"/>
       <c r="Q16" s="180"/>
     </row>
-    <row r="17" spans="1:17" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="221"/>
-      <c r="B17" s="222"/>
-      <c r="C17" s="222"/>
-      <c r="D17" s="222"/>
-      <c r="E17" s="222"/>
-      <c r="F17" s="222"/>
-      <c r="G17" s="222"/>
-      <c r="H17" s="222"/>
-      <c r="I17" s="222"/>
-      <c r="J17" s="222"/>
-      <c r="K17" s="222"/>
-      <c r="L17" s="222"/>
-      <c r="M17" s="222"/>
-      <c r="N17" s="222"/>
-      <c r="O17" s="222"/>
-      <c r="P17" s="222"/>
-      <c r="Q17" s="223"/>
+    <row r="17" spans="1:17" ht="5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="340"/>
+      <c r="B17" s="341"/>
+      <c r="C17" s="341"/>
+      <c r="D17" s="341"/>
+      <c r="E17" s="341"/>
+      <c r="F17" s="341"/>
+      <c r="G17" s="341"/>
+      <c r="H17" s="341"/>
+      <c r="I17" s="341"/>
+      <c r="J17" s="341"/>
+      <c r="K17" s="341"/>
+      <c r="L17" s="341"/>
+      <c r="M17" s="341"/>
+      <c r="N17" s="341"/>
+      <c r="O17" s="341"/>
+      <c r="P17" s="341"/>
+      <c r="Q17" s="342"/>
     </row>
     <row r="18" spans="1:17" ht="11" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="260" t="s">
+      <c r="A18" s="208" t="s">
         <v>86</v>
       </c>
-      <c r="B18" s="261"/>
-      <c r="C18" s="261"/>
-      <c r="D18" s="261"/>
-      <c r="E18" s="261"/>
-      <c r="F18" s="261"/>
-      <c r="G18" s="261"/>
-      <c r="H18" s="261"/>
-      <c r="I18" s="261"/>
-      <c r="J18" s="261"/>
-      <c r="K18" s="261"/>
-      <c r="L18" s="261"/>
-      <c r="M18" s="262"/>
-      <c r="N18" s="258"/>
-      <c r="O18" s="260" t="s">
+      <c r="B18" s="209"/>
+      <c r="C18" s="209"/>
+      <c r="D18" s="209"/>
+      <c r="E18" s="209"/>
+      <c r="F18" s="209"/>
+      <c r="G18" s="209"/>
+      <c r="H18" s="209"/>
+      <c r="I18" s="209"/>
+      <c r="J18" s="209"/>
+      <c r="K18" s="209"/>
+      <c r="L18" s="209"/>
+      <c r="M18" s="210"/>
+      <c r="N18" s="345"/>
+      <c r="O18" s="208" t="s">
         <v>258</v>
       </c>
-      <c r="P18" s="261"/>
-      <c r="Q18" s="262"/>
+      <c r="P18" s="209"/>
+      <c r="Q18" s="210"/>
     </row>
     <row r="19" spans="1:17" ht="11" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="263"/>
-      <c r="B19" s="264"/>
-      <c r="C19" s="264"/>
-      <c r="D19" s="264"/>
-      <c r="E19" s="264"/>
-      <c r="F19" s="264"/>
-      <c r="G19" s="264"/>
-      <c r="H19" s="264"/>
-      <c r="I19" s="264"/>
-      <c r="J19" s="264"/>
-      <c r="K19" s="264"/>
-      <c r="L19" s="264"/>
-      <c r="M19" s="265"/>
-      <c r="N19" s="258"/>
-      <c r="O19" s="263"/>
-      <c r="P19" s="264"/>
-      <c r="Q19" s="265"/>
+      <c r="A19" s="211"/>
+      <c r="B19" s="212"/>
+      <c r="C19" s="212"/>
+      <c r="D19" s="212"/>
+      <c r="E19" s="212"/>
+      <c r="F19" s="212"/>
+      <c r="G19" s="212"/>
+      <c r="H19" s="212"/>
+      <c r="I19" s="212"/>
+      <c r="J19" s="212"/>
+      <c r="K19" s="212"/>
+      <c r="L19" s="212"/>
+      <c r="M19" s="213"/>
+      <c r="N19" s="345"/>
+      <c r="O19" s="211"/>
+      <c r="P19" s="212"/>
+      <c r="Q19" s="213"/>
     </row>
     <row r="20" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="173" t="s">
         <v>201</v>
       </c>
-      <c r="B20" s="244" t="s">
+      <c r="B20" s="215" t="s">
         <v>259</v>
       </c>
-      <c r="C20" s="244"/>
-      <c r="D20" s="244"/>
-      <c r="E20" s="244"/>
-      <c r="F20" s="244"/>
-      <c r="G20" s="244" t="s">
+      <c r="C20" s="215"/>
+      <c r="D20" s="215"/>
+      <c r="E20" s="215"/>
+      <c r="F20" s="215"/>
+      <c r="G20" s="215" t="s">
         <v>260</v>
       </c>
-      <c r="H20" s="244"/>
-      <c r="I20" s="244"/>
-      <c r="J20" s="244"/>
-      <c r="K20" s="244"/>
-      <c r="L20" s="244"/>
-      <c r="M20" s="269"/>
-      <c r="N20" s="258"/>
+      <c r="H20" s="215"/>
+      <c r="I20" s="215"/>
+      <c r="J20" s="215"/>
+      <c r="K20" s="215"/>
+      <c r="L20" s="215"/>
+      <c r="M20" s="221"/>
+      <c r="N20" s="345"/>
       <c r="O20" s="173" t="s">
         <v>201</v>
       </c>
@@ -14088,23 +14096,23 @@
       <c r="A21" s="170" t="s">
         <v>88</v>
       </c>
-      <c r="B21" s="208" t="s">
+      <c r="B21" s="216" t="s">
         <v>261</v>
       </c>
-      <c r="C21" s="208"/>
-      <c r="D21" s="208"/>
-      <c r="E21" s="208"/>
-      <c r="F21" s="208"/>
-      <c r="G21" s="208" t="s">
+      <c r="C21" s="216"/>
+      <c r="D21" s="216"/>
+      <c r="E21" s="216"/>
+      <c r="F21" s="216"/>
+      <c r="G21" s="216" t="s">
         <v>262</v>
       </c>
-      <c r="H21" s="208"/>
-      <c r="I21" s="208"/>
-      <c r="J21" s="208"/>
-      <c r="K21" s="208"/>
-      <c r="L21" s="208"/>
-      <c r="M21" s="209"/>
-      <c r="N21" s="258"/>
+      <c r="H21" s="216"/>
+      <c r="I21" s="216"/>
+      <c r="J21" s="216"/>
+      <c r="K21" s="216"/>
+      <c r="L21" s="216"/>
+      <c r="M21" s="217"/>
+      <c r="N21" s="345"/>
       <c r="O21" s="202" t="b">
         <v>0</v>
       </c>
@@ -14115,21 +14123,21 @@
       <c r="A22" s="170" t="s">
         <v>94</v>
       </c>
-      <c r="B22" s="208" t="s">
+      <c r="B22" s="216" t="s">
         <v>263</v>
       </c>
-      <c r="C22" s="208"/>
-      <c r="D22" s="208"/>
-      <c r="E22" s="208"/>
-      <c r="F22" s="208"/>
-      <c r="G22" s="208"/>
-      <c r="H22" s="208"/>
-      <c r="I22" s="208"/>
-      <c r="J22" s="208"/>
-      <c r="K22" s="208"/>
-      <c r="L22" s="208"/>
-      <c r="M22" s="209"/>
-      <c r="N22" s="258"/>
+      <c r="C22" s="216"/>
+      <c r="D22" s="216"/>
+      <c r="E22" s="216"/>
+      <c r="F22" s="216"/>
+      <c r="G22" s="216"/>
+      <c r="H22" s="216"/>
+      <c r="I22" s="216"/>
+      <c r="J22" s="216"/>
+      <c r="K22" s="216"/>
+      <c r="L22" s="216"/>
+      <c r="M22" s="217"/>
+      <c r="N22" s="345"/>
       <c r="O22" s="202" t="b">
         <v>0</v>
       </c>
@@ -14140,23 +14148,23 @@
       <c r="A23" s="170" t="s">
         <v>99</v>
       </c>
-      <c r="B23" s="208" t="s">
+      <c r="B23" s="216" t="s">
         <v>264</v>
       </c>
-      <c r="C23" s="208"/>
-      <c r="D23" s="208"/>
-      <c r="E23" s="208"/>
-      <c r="F23" s="208"/>
-      <c r="G23" s="208" t="s">
+      <c r="C23" s="216"/>
+      <c r="D23" s="216"/>
+      <c r="E23" s="216"/>
+      <c r="F23" s="216"/>
+      <c r="G23" s="216" t="s">
         <v>265</v>
       </c>
-      <c r="H23" s="208"/>
-      <c r="I23" s="208"/>
-      <c r="J23" s="208"/>
-      <c r="K23" s="208"/>
-      <c r="L23" s="208"/>
-      <c r="M23" s="209"/>
-      <c r="N23" s="258"/>
+      <c r="H23" s="216"/>
+      <c r="I23" s="216"/>
+      <c r="J23" s="216"/>
+      <c r="K23" s="216"/>
+      <c r="L23" s="216"/>
+      <c r="M23" s="217"/>
+      <c r="N23" s="345"/>
       <c r="O23" s="203" t="b">
         <v>0</v>
       </c>
@@ -14164,23 +14172,23 @@
       <c r="Q23" s="180"/>
     </row>
     <row r="24" spans="1:17" ht="5.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="249"/>
-      <c r="B24" s="250"/>
-      <c r="C24" s="250"/>
-      <c r="D24" s="250"/>
-      <c r="E24" s="250"/>
-      <c r="F24" s="250"/>
-      <c r="G24" s="250"/>
-      <c r="H24" s="250"/>
-      <c r="I24" s="250"/>
-      <c r="J24" s="250"/>
-      <c r="K24" s="250"/>
-      <c r="L24" s="250"/>
-      <c r="M24" s="251"/>
-      <c r="N24" s="258"/>
-      <c r="O24" s="247"/>
-      <c r="P24" s="247"/>
-      <c r="Q24" s="248"/>
+      <c r="A24" s="347"/>
+      <c r="B24" s="348"/>
+      <c r="C24" s="348"/>
+      <c r="D24" s="348"/>
+      <c r="E24" s="348"/>
+      <c r="F24" s="348"/>
+      <c r="G24" s="348"/>
+      <c r="H24" s="348"/>
+      <c r="I24" s="348"/>
+      <c r="J24" s="348"/>
+      <c r="K24" s="348"/>
+      <c r="L24" s="348"/>
+      <c r="M24" s="349"/>
+      <c r="N24" s="345"/>
+      <c r="O24" s="350"/>
+      <c r="P24" s="350"/>
+      <c r="Q24" s="351"/>
     </row>
     <row r="25" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="173" t="s">
@@ -14189,51 +14197,51 @@
       <c r="B25" s="169" t="s">
         <v>188</v>
       </c>
-      <c r="C25" s="205" t="s">
+      <c r="C25" s="240" t="s">
         <v>235</v>
       </c>
-      <c r="D25" s="206"/>
-      <c r="E25" s="207"/>
-      <c r="F25" s="205" t="s">
+      <c r="D25" s="241"/>
+      <c r="E25" s="242"/>
+      <c r="F25" s="240" t="s">
         <v>190</v>
       </c>
-      <c r="G25" s="206"/>
-      <c r="H25" s="206"/>
-      <c r="I25" s="207"/>
-      <c r="J25" s="215" t="s">
+      <c r="G25" s="241"/>
+      <c r="H25" s="241"/>
+      <c r="I25" s="242"/>
+      <c r="J25" s="247" t="s">
         <v>266</v>
       </c>
-      <c r="K25" s="216"/>
-      <c r="L25" s="216"/>
-      <c r="M25" s="217"/>
-      <c r="N25" s="258"/>
-      <c r="O25" s="260" t="s">
+      <c r="K25" s="248"/>
+      <c r="L25" s="248"/>
+      <c r="M25" s="249"/>
+      <c r="N25" s="345"/>
+      <c r="O25" s="208" t="s">
         <v>161</v>
       </c>
-      <c r="P25" s="261"/>
-      <c r="Q25" s="262"/>
+      <c r="P25" s="209"/>
+      <c r="Q25" s="210"/>
     </row>
     <row r="26" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="202" t="b">
         <v>0</v>
       </c>
       <c r="B26" s="164"/>
-      <c r="C26" s="210"/>
-      <c r="D26" s="211"/>
-      <c r="E26" s="212"/>
-      <c r="F26" s="210"/>
-      <c r="G26" s="211"/>
-      <c r="H26" s="211"/>
-      <c r="I26" s="212"/>
-      <c r="J26" s="218"/>
-      <c r="K26" s="219"/>
-      <c r="L26" s="219"/>
-      <c r="M26" s="220"/>
-      <c r="N26" s="258"/>
-      <c r="O26" s="235" t="s">
+      <c r="C26" s="205"/>
+      <c r="D26" s="206"/>
+      <c r="E26" s="207"/>
+      <c r="F26" s="205"/>
+      <c r="G26" s="206"/>
+      <c r="H26" s="206"/>
+      <c r="I26" s="207"/>
+      <c r="J26" s="222"/>
+      <c r="K26" s="223"/>
+      <c r="L26" s="223"/>
+      <c r="M26" s="224"/>
+      <c r="N26" s="345"/>
+      <c r="O26" s="243" t="s">
         <v>267</v>
       </c>
-      <c r="P26" s="236"/>
+      <c r="P26" s="244"/>
       <c r="Q26" s="190" t="s">
         <v>268</v>
       </c>
@@ -14243,20 +14251,20 @@
         <v>0</v>
       </c>
       <c r="B27" s="164"/>
-      <c r="C27" s="210"/>
-      <c r="D27" s="211"/>
-      <c r="E27" s="212"/>
-      <c r="F27" s="210"/>
-      <c r="G27" s="211"/>
-      <c r="H27" s="211"/>
-      <c r="I27" s="212"/>
-      <c r="J27" s="218"/>
-      <c r="K27" s="219"/>
-      <c r="L27" s="219"/>
-      <c r="M27" s="220"/>
-      <c r="N27" s="258"/>
-      <c r="O27" s="234"/>
-      <c r="P27" s="208"/>
+      <c r="C27" s="205"/>
+      <c r="D27" s="206"/>
+      <c r="E27" s="207"/>
+      <c r="F27" s="205"/>
+      <c r="G27" s="206"/>
+      <c r="H27" s="206"/>
+      <c r="I27" s="207"/>
+      <c r="J27" s="222"/>
+      <c r="K27" s="223"/>
+      <c r="L27" s="223"/>
+      <c r="M27" s="224"/>
+      <c r="N27" s="345"/>
+      <c r="O27" s="227"/>
+      <c r="P27" s="216"/>
       <c r="Q27" s="172"/>
     </row>
     <row r="28" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -14264,20 +14272,20 @@
         <v>0</v>
       </c>
       <c r="B28" s="164"/>
-      <c r="C28" s="210"/>
-      <c r="D28" s="211"/>
-      <c r="E28" s="212"/>
-      <c r="F28" s="210"/>
-      <c r="G28" s="211"/>
-      <c r="H28" s="211"/>
-      <c r="I28" s="212"/>
-      <c r="J28" s="218"/>
-      <c r="K28" s="219"/>
-      <c r="L28" s="219"/>
-      <c r="M28" s="220"/>
-      <c r="N28" s="258"/>
-      <c r="O28" s="234"/>
-      <c r="P28" s="208"/>
+      <c r="C28" s="205"/>
+      <c r="D28" s="206"/>
+      <c r="E28" s="207"/>
+      <c r="F28" s="205"/>
+      <c r="G28" s="206"/>
+      <c r="H28" s="206"/>
+      <c r="I28" s="207"/>
+      <c r="J28" s="222"/>
+      <c r="K28" s="223"/>
+      <c r="L28" s="223"/>
+      <c r="M28" s="224"/>
+      <c r="N28" s="345"/>
+      <c r="O28" s="227"/>
+      <c r="P28" s="216"/>
       <c r="Q28" s="172"/>
     </row>
     <row r="29" spans="1:17" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -14285,20 +14293,20 @@
         <v>0</v>
       </c>
       <c r="B29" s="175"/>
-      <c r="C29" s="252"/>
-      <c r="D29" s="253"/>
-      <c r="E29" s="254"/>
-      <c r="F29" s="252"/>
-      <c r="G29" s="253"/>
-      <c r="H29" s="253"/>
-      <c r="I29" s="254"/>
-      <c r="J29" s="255"/>
-      <c r="K29" s="256"/>
-      <c r="L29" s="256"/>
-      <c r="M29" s="257"/>
-      <c r="N29" s="258"/>
-      <c r="O29" s="234"/>
-      <c r="P29" s="208"/>
+      <c r="C29" s="228"/>
+      <c r="D29" s="229"/>
+      <c r="E29" s="230"/>
+      <c r="F29" s="228"/>
+      <c r="G29" s="229"/>
+      <c r="H29" s="229"/>
+      <c r="I29" s="230"/>
+      <c r="J29" s="231"/>
+      <c r="K29" s="232"/>
+      <c r="L29" s="232"/>
+      <c r="M29" s="233"/>
+      <c r="N29" s="345"/>
+      <c r="O29" s="227"/>
+      <c r="P29" s="216"/>
       <c r="Q29" s="172"/>
     </row>
     <row r="30" spans="1:17" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -14306,64 +14314,64 @@
         <v>0</v>
       </c>
       <c r="B30" s="175"/>
-      <c r="C30" s="252"/>
-      <c r="D30" s="253"/>
-      <c r="E30" s="254"/>
-      <c r="F30" s="252"/>
-      <c r="G30" s="253"/>
-      <c r="H30" s="253"/>
-      <c r="I30" s="254"/>
-      <c r="J30" s="255"/>
-      <c r="K30" s="256"/>
-      <c r="L30" s="256"/>
-      <c r="M30" s="257"/>
-      <c r="N30" s="258"/>
-      <c r="O30" s="234"/>
-      <c r="P30" s="208"/>
+      <c r="C30" s="228"/>
+      <c r="D30" s="229"/>
+      <c r="E30" s="230"/>
+      <c r="F30" s="228"/>
+      <c r="G30" s="229"/>
+      <c r="H30" s="229"/>
+      <c r="I30" s="230"/>
+      <c r="J30" s="231"/>
+      <c r="K30" s="232"/>
+      <c r="L30" s="232"/>
+      <c r="M30" s="233"/>
+      <c r="N30" s="345"/>
+      <c r="O30" s="227"/>
+      <c r="P30" s="216"/>
       <c r="Q30" s="171"/>
     </row>
     <row r="31" spans="1:17" ht="22.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="266" t="s">
+      <c r="A31" s="218" t="s">
         <v>269</v>
       </c>
-      <c r="B31" s="267"/>
-      <c r="C31" s="267"/>
-      <c r="D31" s="267"/>
-      <c r="E31" s="267"/>
-      <c r="F31" s="267"/>
-      <c r="G31" s="267"/>
-      <c r="H31" s="267"/>
-      <c r="I31" s="267"/>
-      <c r="J31" s="267"/>
-      <c r="K31" s="267"/>
-      <c r="L31" s="267"/>
-      <c r="M31" s="268"/>
-      <c r="N31" s="258"/>
-      <c r="O31" s="234"/>
-      <c r="P31" s="208"/>
+      <c r="B31" s="219"/>
+      <c r="C31" s="219"/>
+      <c r="D31" s="219"/>
+      <c r="E31" s="219"/>
+      <c r="F31" s="219"/>
+      <c r="G31" s="219"/>
+      <c r="H31" s="219"/>
+      <c r="I31" s="219"/>
+      <c r="J31" s="219"/>
+      <c r="K31" s="219"/>
+      <c r="L31" s="219"/>
+      <c r="M31" s="220"/>
+      <c r="N31" s="345"/>
+      <c r="O31" s="227"/>
+      <c r="P31" s="216"/>
       <c r="Q31" s="171"/>
     </row>
     <row r="32" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="242" t="s">
+      <c r="A32" s="239" t="s">
         <v>270</v>
       </c>
-      <c r="B32" s="239"/>
-      <c r="C32" s="239" t="s">
+      <c r="B32" s="236"/>
+      <c r="C32" s="236" t="s">
         <v>271</v>
       </c>
-      <c r="D32" s="239"/>
-      <c r="E32" s="239"/>
-      <c r="F32" s="239"/>
-      <c r="G32" s="244" t="s">
+      <c r="D32" s="236"/>
+      <c r="E32" s="236"/>
+      <c r="F32" s="236"/>
+      <c r="G32" s="215" t="s">
         <v>272</v>
       </c>
-      <c r="H32" s="244"/>
-      <c r="I32" s="244"/>
-      <c r="J32" s="244"/>
-      <c r="K32" s="244"/>
-      <c r="L32" s="244"/>
-      <c r="M32" s="269"/>
-      <c r="N32" s="258"/>
+      <c r="H32" s="215"/>
+      <c r="I32" s="215"/>
+      <c r="J32" s="215"/>
+      <c r="K32" s="215"/>
+      <c r="L32" s="215"/>
+      <c r="M32" s="221"/>
+      <c r="N32" s="345"/>
       <c r="O32" s="173" t="s">
         <v>201</v>
       </c>
@@ -14375,20 +14383,20 @@
       </c>
     </row>
     <row r="33" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="243"/>
-      <c r="B33" s="244"/>
-      <c r="C33" s="240"/>
-      <c r="D33" s="240"/>
-      <c r="E33" s="240"/>
-      <c r="F33" s="240"/>
-      <c r="G33" s="208"/>
-      <c r="H33" s="208"/>
-      <c r="I33" s="208"/>
-      <c r="J33" s="208"/>
-      <c r="K33" s="208"/>
-      <c r="L33" s="208"/>
-      <c r="M33" s="209"/>
-      <c r="N33" s="258"/>
+      <c r="A33" s="214"/>
+      <c r="B33" s="215"/>
+      <c r="C33" s="237"/>
+      <c r="D33" s="237"/>
+      <c r="E33" s="237"/>
+      <c r="F33" s="237"/>
+      <c r="G33" s="216"/>
+      <c r="H33" s="216"/>
+      <c r="I33" s="216"/>
+      <c r="J33" s="216"/>
+      <c r="K33" s="216"/>
+      <c r="L33" s="216"/>
+      <c r="M33" s="217"/>
+      <c r="N33" s="345"/>
       <c r="O33" s="202" t="b">
         <v>0</v>
       </c>
@@ -14396,20 +14404,20 @@
       <c r="Q33" s="162"/>
     </row>
     <row r="34" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="243"/>
-      <c r="B34" s="244"/>
-      <c r="C34" s="240"/>
-      <c r="D34" s="240"/>
-      <c r="E34" s="240"/>
-      <c r="F34" s="240"/>
-      <c r="G34" s="208"/>
-      <c r="H34" s="208"/>
-      <c r="I34" s="208"/>
-      <c r="J34" s="208"/>
-      <c r="K34" s="208"/>
-      <c r="L34" s="208"/>
-      <c r="M34" s="209"/>
-      <c r="N34" s="258"/>
+      <c r="A34" s="214"/>
+      <c r="B34" s="215"/>
+      <c r="C34" s="237"/>
+      <c r="D34" s="237"/>
+      <c r="E34" s="237"/>
+      <c r="F34" s="237"/>
+      <c r="G34" s="216"/>
+      <c r="H34" s="216"/>
+      <c r="I34" s="216"/>
+      <c r="J34" s="216"/>
+      <c r="K34" s="216"/>
+      <c r="L34" s="216"/>
+      <c r="M34" s="217"/>
+      <c r="N34" s="345"/>
       <c r="O34" s="202" t="b">
         <v>0</v>
       </c>
@@ -14417,20 +14425,20 @@
       <c r="Q34" s="162"/>
     </row>
     <row r="35" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="243"/>
-      <c r="B35" s="244"/>
-      <c r="C35" s="240"/>
-      <c r="D35" s="240"/>
-      <c r="E35" s="240"/>
-      <c r="F35" s="240"/>
-      <c r="G35" s="208"/>
-      <c r="H35" s="208"/>
-      <c r="I35" s="208"/>
-      <c r="J35" s="208"/>
-      <c r="K35" s="208"/>
-      <c r="L35" s="208"/>
-      <c r="M35" s="209"/>
-      <c r="N35" s="258"/>
+      <c r="A35" s="214"/>
+      <c r="B35" s="215"/>
+      <c r="C35" s="237"/>
+      <c r="D35" s="237"/>
+      <c r="E35" s="237"/>
+      <c r="F35" s="237"/>
+      <c r="G35" s="216"/>
+      <c r="H35" s="216"/>
+      <c r="I35" s="216"/>
+      <c r="J35" s="216"/>
+      <c r="K35" s="216"/>
+      <c r="L35" s="216"/>
+      <c r="M35" s="217"/>
+      <c r="N35" s="345"/>
       <c r="O35" s="202" t="b">
         <v>0</v>
       </c>
@@ -14438,20 +14446,20 @@
       <c r="Q35" s="162"/>
     </row>
     <row r="36" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="243"/>
-      <c r="B36" s="244"/>
-      <c r="C36" s="240"/>
-      <c r="D36" s="240"/>
-      <c r="E36" s="240"/>
-      <c r="F36" s="240"/>
-      <c r="G36" s="208"/>
-      <c r="H36" s="208"/>
-      <c r="I36" s="208"/>
-      <c r="J36" s="208"/>
-      <c r="K36" s="208"/>
-      <c r="L36" s="208"/>
-      <c r="M36" s="209"/>
-      <c r="N36" s="258"/>
+      <c r="A36" s="214"/>
+      <c r="B36" s="215"/>
+      <c r="C36" s="237"/>
+      <c r="D36" s="237"/>
+      <c r="E36" s="237"/>
+      <c r="F36" s="237"/>
+      <c r="G36" s="216"/>
+      <c r="H36" s="216"/>
+      <c r="I36" s="216"/>
+      <c r="J36" s="216"/>
+      <c r="K36" s="216"/>
+      <c r="L36" s="216"/>
+      <c r="M36" s="217"/>
+      <c r="N36" s="345"/>
       <c r="O36" s="202" t="b">
         <v>0</v>
       </c>
@@ -14459,20 +14467,20 @@
       <c r="Q36" s="162"/>
     </row>
     <row r="37" spans="1:17" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="237"/>
-      <c r="B37" s="238"/>
-      <c r="C37" s="241"/>
-      <c r="D37" s="241"/>
-      <c r="E37" s="241"/>
-      <c r="F37" s="241"/>
-      <c r="G37" s="245"/>
-      <c r="H37" s="245"/>
-      <c r="I37" s="245"/>
-      <c r="J37" s="245"/>
-      <c r="K37" s="245"/>
-      <c r="L37" s="245"/>
-      <c r="M37" s="246"/>
-      <c r="N37" s="259"/>
+      <c r="A37" s="234"/>
+      <c r="B37" s="235"/>
+      <c r="C37" s="238"/>
+      <c r="D37" s="238"/>
+      <c r="E37" s="238"/>
+      <c r="F37" s="238"/>
+      <c r="G37" s="225"/>
+      <c r="H37" s="225"/>
+      <c r="I37" s="225"/>
+      <c r="J37" s="225"/>
+      <c r="K37" s="225"/>
+      <c r="L37" s="225"/>
+      <c r="M37" s="226"/>
+      <c r="N37" s="346"/>
       <c r="O37" s="203" t="b">
         <v>0</v>
       </c>
@@ -14481,6 +14489,55 @@
     </row>
   </sheetData>
   <mergeCells count="65">
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="G35:M35"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="K1:K16"/>
+    <mergeCell ref="J25:M25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="J26:M26"/>
+    <mergeCell ref="G22:M22"/>
+    <mergeCell ref="A17:Q17"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="O9:Q9"/>
+    <mergeCell ref="O13:Q13"/>
+    <mergeCell ref="N1:N16"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="O26:P26"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="G36:M36"/>
+    <mergeCell ref="J27:M27"/>
+    <mergeCell ref="G37:M37"/>
+    <mergeCell ref="O24:Q24"/>
+    <mergeCell ref="A24:M24"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="J28:M28"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="J29:M29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="F30:I30"/>
+    <mergeCell ref="J30:M30"/>
+    <mergeCell ref="N18:N37"/>
+    <mergeCell ref="O27:P27"/>
+    <mergeCell ref="O25:Q25"/>
     <mergeCell ref="C28:E28"/>
     <mergeCell ref="O18:Q19"/>
     <mergeCell ref="A36:B36"/>
@@ -14497,58 +14554,10 @@
     <mergeCell ref="G20:M20"/>
     <mergeCell ref="G21:M21"/>
     <mergeCell ref="G32:M32"/>
-    <mergeCell ref="G36:M36"/>
-    <mergeCell ref="J27:M27"/>
-    <mergeCell ref="G37:M37"/>
-    <mergeCell ref="O24:Q24"/>
-    <mergeCell ref="A24:M24"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="J28:M28"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="J29:M29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="F30:I30"/>
-    <mergeCell ref="J30:M30"/>
-    <mergeCell ref="N18:N37"/>
-    <mergeCell ref="O27:P27"/>
-    <mergeCell ref="O25:Q25"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="N1:N16"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="O29:P29"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="O26:P26"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="G35:M35"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="K1:K16"/>
-    <mergeCell ref="J25:M25"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="J26:M26"/>
-    <mergeCell ref="G22:M22"/>
-    <mergeCell ref="A17:Q17"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="O9:Q9"/>
-    <mergeCell ref="O13:Q13"/>
   </mergeCells>
+  <printOptions headings="1" gridLines="1"/>
   <pageMargins left="0" right="0" top="1" bottom="0" header="0.05" footer="0"/>
-  <pageSetup scale="73" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="66" orientation="landscape" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;G&amp;C&amp;"-,Bold"&amp;16Name: Gerald Nyah  
 Dept: Bakery&amp;R&amp;"-,Bold"&amp;16Week: 03/02/26_03/06/26
@@ -14566,6 +14575,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AC08AA986192C8478F8DEF23E56FA25A" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c98876fc4a3c8e24f43ea00a76fc314f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f7483ffd-f6df-4187-8154-dd569cc9f787" xmlns:ns3="48dabc29-dff2-4377-b8bd-925bf704b174" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0ec66ecb060b89c2b9d672ab12a98af5" ns2:_="" ns3:_="">
     <xsd:import namespace="f7483ffd-f6df-4187-8154-dd569cc9f787"/>
@@ -14826,15 +14844,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -14854,6 +14863,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71F133E1-1A1B-43E9-A269-FAD264E0A4B3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20A5150C-F922-45AB-900D-4C80FF5C4784}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14872,14 +14889,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71F133E1-1A1B-43E9-A269-FAD264E0A4B3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CA05D3C-F01D-4E93-9CC5-047180CBB14C}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Enhance trusted device and LSW workflows
</commit_message>
<xml_diff>
--- a/backend/assets/templates/LSW_TEMPLATE.xlsx
+++ b/backend/assets/templates/LSW_TEMPLATE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/geraldnyah/Documents/PROGRAMMING/MeetingIntelligence/dashmet-rca-backend/backend/assets/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/geraldnyah/MeetingIntelligence/dashmet-rca-backend/backend/assets/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D66D41A-DA79-B540-B22F-14D346F18E4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9BBD1FF-8F95-FC45-B201-DAD446942F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="38400" windowHeight="22300" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19700" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Operations Manager" sheetId="1" state="hidden" r:id="rId1"/>
@@ -2406,7 +2406,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="395">
+  <cellXfs count="394">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -3061,210 +3061,198 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="80" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="80" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="91" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="90" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="86" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="88" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="79" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="84" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="92" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="89" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="91" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="100" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="101" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="84" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="92" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="107" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="80" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="80" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="107" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="91" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="79" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="84" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="92" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="89" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="91" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="100" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="101" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="84" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="92" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="81" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="91" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="90" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="86" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="88" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3298,6 +3286,120 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="82" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="80" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="72" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="81" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="79" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="59" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3307,21 +3409,27 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3343,126 +3451,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="59" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="54" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="82" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="4" borderId="80" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="4" borderId="72" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="4" borderId="81" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="4" borderId="79" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="14" borderId="68" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -3511,6 +3499,9 @@
     <xf numFmtId="0" fontId="12" fillId="11" borderId="74" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9147,29 +9138,29 @@
       <c r="H1" s="45"/>
       <c r="I1" s="45"/>
       <c r="J1" s="35"/>
-      <c r="K1" s="322" t="s">
+      <c r="K1" s="318" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="322"/>
+      <c r="L1" s="318"/>
       <c r="M1" s="35"/>
       <c r="N1" s="34"/>
       <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="18"/>
-      <c r="B2" s="317" t="s">
+      <c r="B2" s="313" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="317"/>
-      <c r="D2" s="317"/>
-      <c r="E2" s="317"/>
-      <c r="F2" s="317"/>
-      <c r="G2" s="317"/>
-      <c r="H2" s="317"/>
-      <c r="I2" s="317"/>
+      <c r="C2" s="313"/>
+      <c r="D2" s="313"/>
+      <c r="E2" s="313"/>
+      <c r="F2" s="313"/>
+      <c r="G2" s="313"/>
+      <c r="H2" s="313"/>
+      <c r="I2" s="313"/>
       <c r="J2" s="36"/>
-      <c r="K2" s="323"/>
-      <c r="L2" s="323"/>
+      <c r="K2" s="319"/>
+      <c r="L2" s="319"/>
       <c r="M2" s="37"/>
       <c r="N2" s="38"/>
       <c r="O2" s="20"/>
@@ -10197,42 +10188,42 @@
       <c r="O40" s="13"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A41" s="318" t="s">
+      <c r="A41" s="314" t="s">
         <v>86</v>
       </c>
-      <c r="B41" s="319"/>
-      <c r="C41" s="319"/>
-      <c r="D41" s="319"/>
-      <c r="E41" s="319"/>
-      <c r="F41" s="319"/>
-      <c r="G41" s="319"/>
-      <c r="H41" s="319"/>
-      <c r="I41" s="319"/>
-      <c r="J41" s="319"/>
-      <c r="K41" s="319"/>
+      <c r="B41" s="315"/>
+      <c r="C41" s="315"/>
+      <c r="D41" s="315"/>
+      <c r="E41" s="315"/>
+      <c r="F41" s="315"/>
+      <c r="G41" s="315"/>
+      <c r="H41" s="315"/>
+      <c r="I41" s="315"/>
+      <c r="J41" s="315"/>
+      <c r="K41" s="315"/>
       <c r="L41" s="3"/>
       <c r="M41" s="28"/>
-      <c r="N41" s="319" t="s">
+      <c r="N41" s="315" t="s">
         <v>87</v>
       </c>
-      <c r="O41" s="321"/>
+      <c r="O41" s="317"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A42" s="320"/>
-      <c r="B42" s="315"/>
-      <c r="C42" s="315"/>
-      <c r="D42" s="315"/>
-      <c r="E42" s="315"/>
-      <c r="F42" s="315"/>
-      <c r="G42" s="315"/>
-      <c r="H42" s="315"/>
-      <c r="I42" s="315"/>
-      <c r="J42" s="315"/>
-      <c r="K42" s="315"/>
+      <c r="A42" s="316"/>
+      <c r="B42" s="311"/>
+      <c r="C42" s="311"/>
+      <c r="D42" s="311"/>
+      <c r="E42" s="311"/>
+      <c r="F42" s="311"/>
+      <c r="G42" s="311"/>
+      <c r="H42" s="311"/>
+      <c r="I42" s="311"/>
+      <c r="J42" s="311"/>
+      <c r="K42" s="311"/>
       <c r="L42" s="27"/>
       <c r="M42" s="29"/>
-      <c r="N42" s="315"/>
-      <c r="O42" s="316"/>
+      <c r="N42" s="311"/>
+      <c r="O42" s="312"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" s="77" t="s">
@@ -10622,10 +10613,10 @@
       <c r="K57" s="22"/>
       <c r="L57" s="22"/>
       <c r="M57" s="31"/>
-      <c r="N57" s="313" t="s">
+      <c r="N57" s="309" t="s">
         <v>144</v>
       </c>
-      <c r="O57" s="314"/>
+      <c r="O57" s="310"/>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" s="78"/>
@@ -10641,8 +10632,8 @@
       <c r="K58" s="22"/>
       <c r="L58" s="22"/>
       <c r="M58" s="31"/>
-      <c r="N58" s="315"/>
-      <c r="O58" s="316"/>
+      <c r="N58" s="311"/>
+      <c r="O58" s="312"/>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59" s="78"/>
@@ -11040,10 +11031,10 @@
         <v>160</v>
       </c>
       <c r="M75" s="31"/>
-      <c r="N75" s="313" t="s">
+      <c r="N75" s="309" t="s">
         <v>161</v>
       </c>
-      <c r="O75" s="314"/>
+      <c r="O75" s="310"/>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A76" s="18"/>
@@ -11063,8 +11054,8 @@
         <v>163</v>
       </c>
       <c r="M76" s="31"/>
-      <c r="N76" s="315"/>
-      <c r="O76" s="316"/>
+      <c r="N76" s="311"/>
+      <c r="O76" s="312"/>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A77" s="21"/>
@@ -11220,23 +11211,23 @@
         <v>176</v>
       </c>
       <c r="E1" s="35"/>
-      <c r="F1" s="322" t="s">
+      <c r="F1" s="318" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="322"/>
+      <c r="G1" s="318"/>
       <c r="H1" s="35"/>
-      <c r="I1" s="369" t="s">
+      <c r="I1" s="330" t="s">
         <v>177</v>
       </c>
-      <c r="J1" s="369"/>
-      <c r="K1" s="369"/>
-      <c r="L1" s="369"/>
-      <c r="M1" s="369"/>
-      <c r="N1" s="369"/>
-      <c r="O1" s="369"/>
-      <c r="P1" s="369"/>
-      <c r="Q1" s="369"/>
-      <c r="R1" s="370"/>
+      <c r="J1" s="330"/>
+      <c r="K1" s="330"/>
+      <c r="L1" s="330"/>
+      <c r="M1" s="330"/>
+      <c r="N1" s="330"/>
+      <c r="O1" s="330"/>
+      <c r="P1" s="330"/>
+      <c r="Q1" s="330"/>
+      <c r="R1" s="331"/>
     </row>
     <row r="2" spans="1:18" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="44" t="s">
@@ -11757,18 +11748,18 @@
       </c>
       <c r="G24" s="8"/>
       <c r="H24" s="1"/>
-      <c r="I24" s="371" t="s">
+      <c r="I24" s="332" t="s">
         <v>22</v>
       </c>
-      <c r="J24" s="371"/>
-      <c r="K24" s="371"/>
-      <c r="L24" s="371"/>
-      <c r="M24" s="371"/>
-      <c r="N24" s="371"/>
-      <c r="O24" s="371"/>
-      <c r="P24" s="371"/>
-      <c r="Q24" s="371"/>
-      <c r="R24" s="372"/>
+      <c r="J24" s="332"/>
+      <c r="K24" s="332"/>
+      <c r="L24" s="332"/>
+      <c r="M24" s="332"/>
+      <c r="N24" s="332"/>
+      <c r="O24" s="332"/>
+      <c r="P24" s="332"/>
+      <c r="Q24" s="332"/>
+      <c r="R24" s="333"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25" s="7"/>
@@ -11825,18 +11816,18 @@
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="1"/>
-      <c r="I27" s="371" t="s">
+      <c r="I27" s="332" t="s">
         <v>56</v>
       </c>
-      <c r="J27" s="371"/>
-      <c r="K27" s="371"/>
-      <c r="L27" s="371"/>
-      <c r="M27" s="371"/>
-      <c r="N27" s="371"/>
-      <c r="O27" s="371"/>
-      <c r="P27" s="371"/>
-      <c r="Q27" s="371"/>
-      <c r="R27" s="372"/>
+      <c r="J27" s="332"/>
+      <c r="K27" s="332"/>
+      <c r="L27" s="332"/>
+      <c r="M27" s="332"/>
+      <c r="N27" s="332"/>
+      <c r="O27" s="332"/>
+      <c r="P27" s="332"/>
+      <c r="Q27" s="332"/>
+      <c r="R27" s="333"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" s="7"/>
@@ -11937,18 +11928,18 @@
       </c>
       <c r="G32" s="8"/>
       <c r="H32" s="1"/>
-      <c r="I32" s="373" t="s">
+      <c r="I32" s="334" t="s">
         <v>69</v>
       </c>
-      <c r="J32" s="373"/>
-      <c r="K32" s="373"/>
-      <c r="L32" s="373"/>
-      <c r="M32" s="373"/>
-      <c r="N32" s="373"/>
-      <c r="O32" s="373"/>
-      <c r="P32" s="373"/>
-      <c r="Q32" s="373"/>
-      <c r="R32" s="374"/>
+      <c r="J32" s="334"/>
+      <c r="K32" s="334"/>
+      <c r="L32" s="334"/>
+      <c r="M32" s="334"/>
+      <c r="N32" s="334"/>
+      <c r="O32" s="334"/>
+      <c r="P32" s="334"/>
+      <c r="Q32" s="334"/>
+      <c r="R32" s="335"/>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A33" s="7"/>
@@ -12121,199 +12112,199 @@
       <c r="R40" s="9"/>
     </row>
     <row r="41" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="318"/>
-      <c r="B41" s="319"/>
-      <c r="C41" s="319"/>
-      <c r="D41" s="319"/>
-      <c r="E41" s="319"/>
-      <c r="F41" s="319"/>
+      <c r="A41" s="314"/>
+      <c r="B41" s="315"/>
+      <c r="C41" s="315"/>
+      <c r="D41" s="315"/>
+      <c r="E41" s="315"/>
+      <c r="F41" s="315"/>
       <c r="G41" s="3"/>
       <c r="H41" s="28"/>
-      <c r="I41" s="318" t="s">
+      <c r="I41" s="314" t="s">
         <v>183</v>
       </c>
-      <c r="J41" s="319"/>
-      <c r="K41" s="319"/>
-      <c r="L41" s="319"/>
-      <c r="M41" s="319"/>
-      <c r="N41" s="319"/>
-      <c r="O41" s="319"/>
-      <c r="P41" s="319"/>
-      <c r="Q41" s="319"/>
-      <c r="R41" s="321"/>
+      <c r="J41" s="315"/>
+      <c r="K41" s="315"/>
+      <c r="L41" s="315"/>
+      <c r="M41" s="315"/>
+      <c r="N41" s="315"/>
+      <c r="O41" s="315"/>
+      <c r="P41" s="315"/>
+      <c r="Q41" s="315"/>
+      <c r="R41" s="317"/>
       <c r="S41" s="159"/>
     </row>
     <row r="42" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="320"/>
-      <c r="B42" s="315"/>
-      <c r="C42" s="315"/>
-      <c r="D42" s="315"/>
-      <c r="E42" s="315"/>
-      <c r="F42" s="315"/>
+      <c r="A42" s="316"/>
+      <c r="B42" s="311"/>
+      <c r="C42" s="311"/>
+      <c r="D42" s="311"/>
+      <c r="E42" s="311"/>
+      <c r="F42" s="311"/>
       <c r="G42" s="27"/>
       <c r="H42" s="29"/>
-      <c r="I42" s="320"/>
-      <c r="J42" s="315"/>
-      <c r="K42" s="315"/>
-      <c r="L42" s="315"/>
-      <c r="M42" s="315"/>
-      <c r="N42" s="315"/>
-      <c r="O42" s="315"/>
-      <c r="P42" s="315"/>
-      <c r="Q42" s="315"/>
-      <c r="R42" s="316"/>
+      <c r="I42" s="316"/>
+      <c r="J42" s="311"/>
+      <c r="K42" s="311"/>
+      <c r="L42" s="311"/>
+      <c r="M42" s="311"/>
+      <c r="N42" s="311"/>
+      <c r="O42" s="311"/>
+      <c r="P42" s="311"/>
+      <c r="Q42" s="311"/>
+      <c r="R42" s="312"/>
       <c r="S42" s="159"/>
     </row>
     <row r="43" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="87"/>
-      <c r="B43" s="375"/>
-      <c r="C43" s="376"/>
-      <c r="D43" s="376"/>
-      <c r="E43" s="376"/>
-      <c r="F43" s="376"/>
-      <c r="G43" s="377"/>
+      <c r="B43" s="336"/>
+      <c r="C43" s="337"/>
+      <c r="D43" s="337"/>
+      <c r="E43" s="337"/>
+      <c r="F43" s="337"/>
+      <c r="G43" s="338"/>
       <c r="H43" s="30"/>
       <c r="I43" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J43" s="360" t="s">
+      <c r="J43" s="320" t="s">
         <v>184</v>
       </c>
-      <c r="K43" s="361"/>
-      <c r="L43" s="361"/>
-      <c r="M43" s="361"/>
-      <c r="N43" s="361"/>
-      <c r="O43" s="362"/>
-      <c r="P43" s="246" t="s">
+      <c r="K43" s="321"/>
+      <c r="L43" s="321"/>
+      <c r="M43" s="321"/>
+      <c r="N43" s="321"/>
+      <c r="O43" s="322"/>
+      <c r="P43" s="255" t="s">
         <v>185</v>
       </c>
-      <c r="Q43" s="246"/>
-      <c r="R43" s="378"/>
+      <c r="Q43" s="255"/>
+      <c r="R43" s="329"/>
       <c r="S43" s="159"/>
     </row>
     <row r="44" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="88"/>
-      <c r="B44" s="367"/>
-      <c r="C44" s="341"/>
-      <c r="D44" s="341"/>
-      <c r="E44" s="341"/>
-      <c r="F44" s="341"/>
-      <c r="G44" s="342"/>
+      <c r="B44" s="339"/>
+      <c r="C44" s="340"/>
+      <c r="D44" s="340"/>
+      <c r="E44" s="340"/>
+      <c r="F44" s="340"/>
+      <c r="G44" s="341"/>
       <c r="H44" s="31"/>
       <c r="I44" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J44" s="360"/>
-      <c r="K44" s="361"/>
-      <c r="L44" s="361"/>
-      <c r="M44" s="361"/>
-      <c r="N44" s="361"/>
-      <c r="O44" s="362"/>
-      <c r="P44" s="363"/>
-      <c r="Q44" s="363"/>
-      <c r="R44" s="364"/>
+      <c r="J44" s="320"/>
+      <c r="K44" s="321"/>
+      <c r="L44" s="321"/>
+      <c r="M44" s="321"/>
+      <c r="N44" s="321"/>
+      <c r="O44" s="322"/>
+      <c r="P44" s="323"/>
+      <c r="Q44" s="323"/>
+      <c r="R44" s="324"/>
       <c r="S44" s="159"/>
     </row>
     <row r="45" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="88"/>
-      <c r="B45" s="367"/>
-      <c r="C45" s="341"/>
-      <c r="D45" s="341"/>
-      <c r="E45" s="341"/>
-      <c r="F45" s="341"/>
-      <c r="G45" s="342"/>
+      <c r="B45" s="339"/>
+      <c r="C45" s="340"/>
+      <c r="D45" s="340"/>
+      <c r="E45" s="340"/>
+      <c r="F45" s="340"/>
+      <c r="G45" s="341"/>
       <c r="H45" s="31"/>
       <c r="I45" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J45" s="360"/>
-      <c r="K45" s="361"/>
-      <c r="L45" s="361"/>
-      <c r="M45" s="361"/>
-      <c r="N45" s="361"/>
-      <c r="O45" s="362"/>
-      <c r="P45" s="363"/>
-      <c r="Q45" s="363"/>
-      <c r="R45" s="364"/>
+      <c r="J45" s="320"/>
+      <c r="K45" s="321"/>
+      <c r="L45" s="321"/>
+      <c r="M45" s="321"/>
+      <c r="N45" s="321"/>
+      <c r="O45" s="322"/>
+      <c r="P45" s="323"/>
+      <c r="Q45" s="323"/>
+      <c r="R45" s="324"/>
       <c r="S45" s="159"/>
     </row>
     <row r="46" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="88"/>
-      <c r="B46" s="367"/>
-      <c r="C46" s="341"/>
-      <c r="D46" s="341"/>
-      <c r="E46" s="341"/>
-      <c r="F46" s="341"/>
-      <c r="G46" s="342"/>
+      <c r="B46" s="339"/>
+      <c r="C46" s="340"/>
+      <c r="D46" s="340"/>
+      <c r="E46" s="340"/>
+      <c r="F46" s="340"/>
+      <c r="G46" s="341"/>
       <c r="H46" s="31"/>
       <c r="I46" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J46" s="360"/>
-      <c r="K46" s="361"/>
-      <c r="L46" s="361"/>
-      <c r="M46" s="361"/>
-      <c r="N46" s="361"/>
-      <c r="O46" s="362"/>
-      <c r="P46" s="363"/>
-      <c r="Q46" s="363"/>
-      <c r="R46" s="364"/>
+      <c r="J46" s="320"/>
+      <c r="K46" s="321"/>
+      <c r="L46" s="321"/>
+      <c r="M46" s="321"/>
+      <c r="N46" s="321"/>
+      <c r="O46" s="322"/>
+      <c r="P46" s="323"/>
+      <c r="Q46" s="323"/>
+      <c r="R46" s="324"/>
       <c r="S46" s="159"/>
     </row>
     <row r="47" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="88"/>
-      <c r="B47" s="367"/>
-      <c r="C47" s="341"/>
-      <c r="D47" s="341"/>
-      <c r="E47" s="341"/>
-      <c r="F47" s="341"/>
-      <c r="G47" s="342"/>
+      <c r="B47" s="339"/>
+      <c r="C47" s="340"/>
+      <c r="D47" s="340"/>
+      <c r="E47" s="340"/>
+      <c r="F47" s="340"/>
+      <c r="G47" s="341"/>
       <c r="H47" s="31"/>
       <c r="I47" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J47" s="360"/>
-      <c r="K47" s="361"/>
-      <c r="L47" s="361"/>
-      <c r="M47" s="361"/>
-      <c r="N47" s="361"/>
-      <c r="O47" s="362"/>
-      <c r="P47" s="363"/>
-      <c r="Q47" s="363"/>
-      <c r="R47" s="364"/>
+      <c r="J47" s="320"/>
+      <c r="K47" s="321"/>
+      <c r="L47" s="321"/>
+      <c r="M47" s="321"/>
+      <c r="N47" s="321"/>
+      <c r="O47" s="322"/>
+      <c r="P47" s="323"/>
+      <c r="Q47" s="323"/>
+      <c r="R47" s="324"/>
       <c r="S47" s="159"/>
     </row>
     <row r="48" spans="1:19" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="88"/>
-      <c r="B48" s="367"/>
-      <c r="C48" s="341"/>
-      <c r="D48" s="341"/>
-      <c r="E48" s="341"/>
-      <c r="F48" s="341"/>
-      <c r="G48" s="342"/>
+      <c r="B48" s="339"/>
+      <c r="C48" s="340"/>
+      <c r="D48" s="340"/>
+      <c r="E48" s="340"/>
+      <c r="F48" s="340"/>
+      <c r="G48" s="341"/>
       <c r="H48" s="31"/>
       <c r="I48" s="96" t="s">
         <v>10</v>
       </c>
-      <c r="J48" s="360"/>
-      <c r="K48" s="361"/>
-      <c r="L48" s="361"/>
-      <c r="M48" s="361"/>
-      <c r="N48" s="361"/>
-      <c r="O48" s="362"/>
-      <c r="P48" s="365"/>
-      <c r="Q48" s="365"/>
-      <c r="R48" s="366"/>
+      <c r="J48" s="320"/>
+      <c r="K48" s="321"/>
+      <c r="L48" s="321"/>
+      <c r="M48" s="321"/>
+      <c r="N48" s="321"/>
+      <c r="O48" s="322"/>
+      <c r="P48" s="325"/>
+      <c r="Q48" s="325"/>
+      <c r="R48" s="326"/>
       <c r="S48" s="159"/>
     </row>
     <row r="49" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="88"/>
-      <c r="B49" s="367"/>
-      <c r="C49" s="341"/>
-      <c r="D49" s="341"/>
-      <c r="E49" s="341"/>
-      <c r="F49" s="341"/>
-      <c r="G49" s="342"/>
+      <c r="B49" s="339"/>
+      <c r="C49" s="340"/>
+      <c r="D49" s="340"/>
+      <c r="E49" s="340"/>
+      <c r="F49" s="340"/>
+      <c r="G49" s="341"/>
       <c r="H49" s="31"/>
       <c r="I49" s="29"/>
       <c r="J49" s="29"/>
@@ -12329,198 +12320,198 @@
     </row>
     <row r="50" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="88"/>
-      <c r="B50" s="367"/>
-      <c r="C50" s="341"/>
-      <c r="D50" s="341"/>
-      <c r="E50" s="341"/>
-      <c r="F50" s="341"/>
-      <c r="G50" s="342"/>
+      <c r="B50" s="339"/>
+      <c r="C50" s="340"/>
+      <c r="D50" s="340"/>
+      <c r="E50" s="340"/>
+      <c r="F50" s="340"/>
+      <c r="G50" s="341"/>
       <c r="H50" s="31"/>
-      <c r="I50" s="354" t="s">
+      <c r="I50" s="327" t="s">
         <v>186</v>
       </c>
-      <c r="J50" s="354"/>
-      <c r="K50" s="354"/>
-      <c r="L50" s="354"/>
-      <c r="M50" s="354"/>
-      <c r="N50" s="354"/>
-      <c r="O50" s="354"/>
-      <c r="P50" s="354"/>
-      <c r="Q50" s="354"/>
-      <c r="R50" s="355"/>
+      <c r="J50" s="327"/>
+      <c r="K50" s="327"/>
+      <c r="L50" s="327"/>
+      <c r="M50" s="327"/>
+      <c r="N50" s="327"/>
+      <c r="O50" s="327"/>
+      <c r="P50" s="327"/>
+      <c r="Q50" s="327"/>
+      <c r="R50" s="328"/>
       <c r="S50" s="105"/>
     </row>
     <row r="51" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="88"/>
-      <c r="B51" s="367"/>
-      <c r="C51" s="341"/>
-      <c r="D51" s="341"/>
-      <c r="E51" s="341"/>
-      <c r="F51" s="341"/>
-      <c r="G51" s="342"/>
+      <c r="B51" s="339"/>
+      <c r="C51" s="340"/>
+      <c r="D51" s="340"/>
+      <c r="E51" s="340"/>
+      <c r="F51" s="340"/>
+      <c r="G51" s="341"/>
       <c r="H51" s="31"/>
-      <c r="I51" s="313"/>
-      <c r="J51" s="313"/>
-      <c r="K51" s="313"/>
-      <c r="L51" s="313"/>
-      <c r="M51" s="313"/>
-      <c r="N51" s="313"/>
-      <c r="O51" s="313"/>
-      <c r="P51" s="313"/>
-      <c r="Q51" s="313"/>
-      <c r="R51" s="314"/>
+      <c r="I51" s="309"/>
+      <c r="J51" s="309"/>
+      <c r="K51" s="309"/>
+      <c r="L51" s="309"/>
+      <c r="M51" s="309"/>
+      <c r="N51" s="309"/>
+      <c r="O51" s="309"/>
+      <c r="P51" s="309"/>
+      <c r="Q51" s="309"/>
+      <c r="R51" s="310"/>
       <c r="S51" s="105"/>
     </row>
     <row r="52" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="88"/>
-      <c r="B52" s="367"/>
-      <c r="C52" s="341"/>
-      <c r="D52" s="341"/>
-      <c r="E52" s="341"/>
-      <c r="F52" s="341"/>
-      <c r="G52" s="342"/>
+      <c r="B52" s="339"/>
+      <c r="C52" s="340"/>
+      <c r="D52" s="340"/>
+      <c r="E52" s="340"/>
+      <c r="F52" s="340"/>
+      <c r="G52" s="341"/>
       <c r="H52" s="31"/>
       <c r="I52" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J52" s="360" t="s">
+      <c r="J52" s="320" t="s">
         <v>184</v>
       </c>
-      <c r="K52" s="361"/>
-      <c r="L52" s="361"/>
-      <c r="M52" s="361"/>
-      <c r="N52" s="361"/>
-      <c r="O52" s="362"/>
-      <c r="P52" s="246" t="s">
+      <c r="K52" s="321"/>
+      <c r="L52" s="321"/>
+      <c r="M52" s="321"/>
+      <c r="N52" s="321"/>
+      <c r="O52" s="322"/>
+      <c r="P52" s="255" t="s">
         <v>185</v>
       </c>
-      <c r="Q52" s="246"/>
-      <c r="R52" s="378"/>
+      <c r="Q52" s="255"/>
+      <c r="R52" s="329"/>
       <c r="S52" s="105"/>
     </row>
     <row r="53" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="88"/>
-      <c r="B53" s="367"/>
-      <c r="C53" s="341"/>
-      <c r="D53" s="341"/>
-      <c r="E53" s="341"/>
-      <c r="F53" s="341"/>
-      <c r="G53" s="342"/>
+      <c r="B53" s="339"/>
+      <c r="C53" s="340"/>
+      <c r="D53" s="340"/>
+      <c r="E53" s="340"/>
+      <c r="F53" s="340"/>
+      <c r="G53" s="341"/>
       <c r="H53" s="31"/>
       <c r="I53" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J53" s="360"/>
-      <c r="K53" s="361"/>
-      <c r="L53" s="361"/>
-      <c r="M53" s="361"/>
-      <c r="N53" s="361"/>
-      <c r="O53" s="362"/>
-      <c r="P53" s="363"/>
-      <c r="Q53" s="363"/>
-      <c r="R53" s="364"/>
+      <c r="J53" s="320"/>
+      <c r="K53" s="321"/>
+      <c r="L53" s="321"/>
+      <c r="M53" s="321"/>
+      <c r="N53" s="321"/>
+      <c r="O53" s="322"/>
+      <c r="P53" s="323"/>
+      <c r="Q53" s="323"/>
+      <c r="R53" s="324"/>
       <c r="S53" s="105"/>
     </row>
     <row r="54" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="88"/>
-      <c r="B54" s="367"/>
-      <c r="C54" s="341"/>
-      <c r="D54" s="341"/>
-      <c r="E54" s="341"/>
-      <c r="F54" s="341"/>
-      <c r="G54" s="342"/>
+      <c r="B54" s="339"/>
+      <c r="C54" s="340"/>
+      <c r="D54" s="340"/>
+      <c r="E54" s="340"/>
+      <c r="F54" s="340"/>
+      <c r="G54" s="341"/>
       <c r="H54" s="31"/>
       <c r="I54" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J54" s="360"/>
-      <c r="K54" s="361"/>
-      <c r="L54" s="361"/>
-      <c r="M54" s="361"/>
-      <c r="N54" s="361"/>
-      <c r="O54" s="362"/>
-      <c r="P54" s="363"/>
-      <c r="Q54" s="363"/>
-      <c r="R54" s="364"/>
+      <c r="J54" s="320"/>
+      <c r="K54" s="321"/>
+      <c r="L54" s="321"/>
+      <c r="M54" s="321"/>
+      <c r="N54" s="321"/>
+      <c r="O54" s="322"/>
+      <c r="P54" s="323"/>
+      <c r="Q54" s="323"/>
+      <c r="R54" s="324"/>
       <c r="S54" s="105"/>
     </row>
     <row r="55" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="88"/>
-      <c r="B55" s="367"/>
-      <c r="C55" s="341"/>
-      <c r="D55" s="341"/>
-      <c r="E55" s="341"/>
-      <c r="F55" s="341"/>
-      <c r="G55" s="342"/>
+      <c r="B55" s="339"/>
+      <c r="C55" s="340"/>
+      <c r="D55" s="340"/>
+      <c r="E55" s="340"/>
+      <c r="F55" s="340"/>
+      <c r="G55" s="341"/>
       <c r="H55" s="31"/>
       <c r="I55" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J55" s="360"/>
-      <c r="K55" s="361"/>
-      <c r="L55" s="361"/>
-      <c r="M55" s="361"/>
-      <c r="N55" s="361"/>
-      <c r="O55" s="362"/>
-      <c r="P55" s="363"/>
-      <c r="Q55" s="363"/>
-      <c r="R55" s="364"/>
+      <c r="J55" s="320"/>
+      <c r="K55" s="321"/>
+      <c r="L55" s="321"/>
+      <c r="M55" s="321"/>
+      <c r="N55" s="321"/>
+      <c r="O55" s="322"/>
+      <c r="P55" s="323"/>
+      <c r="Q55" s="323"/>
+      <c r="R55" s="324"/>
       <c r="S55" s="105"/>
     </row>
     <row r="56" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="88"/>
-      <c r="B56" s="367"/>
-      <c r="C56" s="341"/>
-      <c r="D56" s="341"/>
-      <c r="E56" s="341"/>
-      <c r="F56" s="341"/>
-      <c r="G56" s="342"/>
+      <c r="B56" s="339"/>
+      <c r="C56" s="340"/>
+      <c r="D56" s="340"/>
+      <c r="E56" s="340"/>
+      <c r="F56" s="340"/>
+      <c r="G56" s="341"/>
       <c r="H56" s="31"/>
       <c r="I56" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J56" s="360"/>
-      <c r="K56" s="361"/>
-      <c r="L56" s="361"/>
-      <c r="M56" s="361"/>
-      <c r="N56" s="361"/>
-      <c r="O56" s="362"/>
-      <c r="P56" s="363"/>
-      <c r="Q56" s="363"/>
-      <c r="R56" s="364"/>
+      <c r="J56" s="320"/>
+      <c r="K56" s="321"/>
+      <c r="L56" s="321"/>
+      <c r="M56" s="321"/>
+      <c r="N56" s="321"/>
+      <c r="O56" s="322"/>
+      <c r="P56" s="323"/>
+      <c r="Q56" s="323"/>
+      <c r="R56" s="324"/>
       <c r="S56" s="105"/>
     </row>
     <row r="57" spans="1:19" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="88"/>
-      <c r="B57" s="367"/>
-      <c r="C57" s="341"/>
-      <c r="D57" s="341"/>
-      <c r="E57" s="341"/>
-      <c r="F57" s="341"/>
-      <c r="G57" s="342"/>
+      <c r="B57" s="339"/>
+      <c r="C57" s="340"/>
+      <c r="D57" s="340"/>
+      <c r="E57" s="340"/>
+      <c r="F57" s="340"/>
+      <c r="G57" s="341"/>
       <c r="H57" s="31"/>
       <c r="I57" s="96" t="s">
         <v>10</v>
       </c>
-      <c r="J57" s="360"/>
-      <c r="K57" s="361"/>
-      <c r="L57" s="361"/>
-      <c r="M57" s="361"/>
-      <c r="N57" s="361"/>
-      <c r="O57" s="362"/>
-      <c r="P57" s="365"/>
-      <c r="Q57" s="365"/>
-      <c r="R57" s="366"/>
+      <c r="J57" s="320"/>
+      <c r="K57" s="321"/>
+      <c r="L57" s="321"/>
+      <c r="M57" s="321"/>
+      <c r="N57" s="321"/>
+      <c r="O57" s="322"/>
+      <c r="P57" s="325"/>
+      <c r="Q57" s="325"/>
+      <c r="R57" s="326"/>
       <c r="S57" s="105"/>
     </row>
     <row r="58" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="88"/>
-      <c r="B58" s="367"/>
-      <c r="C58" s="341"/>
-      <c r="D58" s="341"/>
-      <c r="E58" s="341"/>
-      <c r="F58" s="341"/>
-      <c r="G58" s="342"/>
+      <c r="B58" s="339"/>
+      <c r="C58" s="340"/>
+      <c r="D58" s="340"/>
+      <c r="E58" s="340"/>
+      <c r="F58" s="340"/>
+      <c r="G58" s="341"/>
       <c r="H58" s="31"/>
       <c r="I58" s="56"/>
       <c r="J58" s="56"/>
@@ -12536,25 +12527,25 @@
     </row>
     <row r="59" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="88"/>
-      <c r="B59" s="367"/>
-      <c r="C59" s="341"/>
-      <c r="D59" s="341"/>
-      <c r="E59" s="341"/>
-      <c r="F59" s="341"/>
-      <c r="G59" s="342"/>
+      <c r="B59" s="339"/>
+      <c r="C59" s="340"/>
+      <c r="D59" s="340"/>
+      <c r="E59" s="340"/>
+      <c r="F59" s="340"/>
+      <c r="G59" s="341"/>
       <c r="H59" s="31"/>
-      <c r="I59" s="354" t="s">
+      <c r="I59" s="327" t="s">
         <v>187</v>
       </c>
-      <c r="J59" s="354"/>
-      <c r="K59" s="354"/>
-      <c r="L59" s="354"/>
-      <c r="M59" s="354"/>
-      <c r="N59" s="354"/>
-      <c r="O59" s="354"/>
-      <c r="P59" s="354"/>
-      <c r="Q59" s="354"/>
-      <c r="R59" s="355"/>
+      <c r="J59" s="327"/>
+      <c r="K59" s="327"/>
+      <c r="L59" s="327"/>
+      <c r="M59" s="327"/>
+      <c r="N59" s="327"/>
+      <c r="O59" s="327"/>
+      <c r="P59" s="327"/>
+      <c r="Q59" s="327"/>
+      <c r="R59" s="328"/>
       <c r="S59" s="105"/>
     </row>
     <row r="60" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12566,49 +12557,49 @@
       <c r="F60" s="56"/>
       <c r="G60" s="56"/>
       <c r="H60" s="31"/>
-      <c r="I60" s="313"/>
-      <c r="J60" s="313"/>
-      <c r="K60" s="313"/>
-      <c r="L60" s="313"/>
-      <c r="M60" s="313"/>
-      <c r="N60" s="313"/>
-      <c r="O60" s="313"/>
-      <c r="P60" s="313"/>
-      <c r="Q60" s="313"/>
-      <c r="R60" s="314"/>
+      <c r="I60" s="309"/>
+      <c r="J60" s="309"/>
+      <c r="K60" s="309"/>
+      <c r="L60" s="309"/>
+      <c r="M60" s="309"/>
+      <c r="N60" s="309"/>
+      <c r="O60" s="309"/>
+      <c r="P60" s="309"/>
+      <c r="Q60" s="309"/>
+      <c r="R60" s="310"/>
       <c r="S60" s="105"/>
     </row>
     <row r="61" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="327" t="s">
+      <c r="A61" s="342" t="s">
         <v>188</v>
       </c>
-      <c r="B61" s="328"/>
+      <c r="B61" s="343"/>
       <c r="C61" s="97" t="s">
         <v>189</v>
       </c>
       <c r="D61" s="97" t="s">
         <v>190</v>
       </c>
-      <c r="E61" s="328"/>
-      <c r="F61" s="328"/>
-      <c r="G61" s="368"/>
+      <c r="E61" s="343"/>
+      <c r="F61" s="343"/>
+      <c r="G61" s="344"/>
       <c r="H61" s="31"/>
       <c r="I61" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J61" s="360" t="s">
+      <c r="J61" s="320" t="s">
         <v>184</v>
       </c>
-      <c r="K61" s="361"/>
-      <c r="L61" s="361"/>
-      <c r="M61" s="361"/>
-      <c r="N61" s="361"/>
-      <c r="O61" s="362"/>
-      <c r="P61" s="246" t="s">
+      <c r="K61" s="321"/>
+      <c r="L61" s="321"/>
+      <c r="M61" s="321"/>
+      <c r="N61" s="321"/>
+      <c r="O61" s="322"/>
+      <c r="P61" s="255" t="s">
         <v>185</v>
       </c>
-      <c r="Q61" s="246"/>
-      <c r="R61" s="378"/>
+      <c r="Q61" s="255"/>
+      <c r="R61" s="329"/>
       <c r="S61" s="105"/>
     </row>
     <row r="62" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12623,15 +12614,15 @@
       <c r="I62" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J62" s="360"/>
-      <c r="K62" s="361"/>
-      <c r="L62" s="361"/>
-      <c r="M62" s="361"/>
-      <c r="N62" s="361"/>
-      <c r="O62" s="362"/>
-      <c r="P62" s="363"/>
-      <c r="Q62" s="363"/>
-      <c r="R62" s="364"/>
+      <c r="J62" s="320"/>
+      <c r="K62" s="321"/>
+      <c r="L62" s="321"/>
+      <c r="M62" s="321"/>
+      <c r="N62" s="321"/>
+      <c r="O62" s="322"/>
+      <c r="P62" s="323"/>
+      <c r="Q62" s="323"/>
+      <c r="R62" s="324"/>
       <c r="S62" s="105"/>
     </row>
     <row r="63" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12639,22 +12630,22 @@
       <c r="B63" s="8"/>
       <c r="C63" s="8"/>
       <c r="D63" s="10"/>
-      <c r="E63" s="341"/>
-      <c r="F63" s="341"/>
-      <c r="G63" s="342"/>
+      <c r="E63" s="340"/>
+      <c r="F63" s="340"/>
+      <c r="G63" s="341"/>
       <c r="H63" s="31"/>
       <c r="I63" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J63" s="360"/>
-      <c r="K63" s="361"/>
-      <c r="L63" s="361"/>
-      <c r="M63" s="361"/>
-      <c r="N63" s="361"/>
-      <c r="O63" s="362"/>
-      <c r="P63" s="363"/>
-      <c r="Q63" s="363"/>
-      <c r="R63" s="364"/>
+      <c r="J63" s="320"/>
+      <c r="K63" s="321"/>
+      <c r="L63" s="321"/>
+      <c r="M63" s="321"/>
+      <c r="N63" s="321"/>
+      <c r="O63" s="322"/>
+      <c r="P63" s="323"/>
+      <c r="Q63" s="323"/>
+      <c r="R63" s="324"/>
       <c r="S63" s="105"/>
     </row>
     <row r="64" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12662,22 +12653,22 @@
       <c r="B64" s="8"/>
       <c r="C64" s="8"/>
       <c r="D64" s="10"/>
-      <c r="E64" s="341"/>
-      <c r="F64" s="341"/>
-      <c r="G64" s="342"/>
+      <c r="E64" s="340"/>
+      <c r="F64" s="340"/>
+      <c r="G64" s="341"/>
       <c r="H64" s="31"/>
       <c r="I64" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J64" s="360"/>
-      <c r="K64" s="361"/>
-      <c r="L64" s="361"/>
-      <c r="M64" s="361"/>
-      <c r="N64" s="361"/>
-      <c r="O64" s="362"/>
-      <c r="P64" s="363"/>
-      <c r="Q64" s="363"/>
-      <c r="R64" s="364"/>
+      <c r="J64" s="320"/>
+      <c r="K64" s="321"/>
+      <c r="L64" s="321"/>
+      <c r="M64" s="321"/>
+      <c r="N64" s="321"/>
+      <c r="O64" s="322"/>
+      <c r="P64" s="323"/>
+      <c r="Q64" s="323"/>
+      <c r="R64" s="324"/>
       <c r="S64" s="105"/>
     </row>
     <row r="65" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12685,22 +12676,22 @@
       <c r="B65" s="8"/>
       <c r="C65" s="8"/>
       <c r="D65" s="10"/>
-      <c r="E65" s="341"/>
-      <c r="F65" s="341"/>
-      <c r="G65" s="342"/>
+      <c r="E65" s="340"/>
+      <c r="F65" s="340"/>
+      <c r="G65" s="341"/>
       <c r="H65" s="31"/>
       <c r="I65" s="95" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="360"/>
-      <c r="K65" s="361"/>
-      <c r="L65" s="361"/>
-      <c r="M65" s="361"/>
-      <c r="N65" s="361"/>
-      <c r="O65" s="362"/>
-      <c r="P65" s="363"/>
-      <c r="Q65" s="363"/>
-      <c r="R65" s="364"/>
+      <c r="J65" s="320"/>
+      <c r="K65" s="321"/>
+      <c r="L65" s="321"/>
+      <c r="M65" s="321"/>
+      <c r="N65" s="321"/>
+      <c r="O65" s="322"/>
+      <c r="P65" s="323"/>
+      <c r="Q65" s="323"/>
+      <c r="R65" s="324"/>
       <c r="S65" s="105"/>
     </row>
     <row r="66" spans="1:19" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -12708,22 +12699,22 @@
       <c r="B66" s="8"/>
       <c r="C66" s="8"/>
       <c r="D66" s="10"/>
-      <c r="E66" s="341"/>
-      <c r="F66" s="341"/>
-      <c r="G66" s="342"/>
+      <c r="E66" s="340"/>
+      <c r="F66" s="340"/>
+      <c r="G66" s="341"/>
       <c r="H66" s="31"/>
       <c r="I66" s="96" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="360"/>
-      <c r="K66" s="361"/>
-      <c r="L66" s="361"/>
-      <c r="M66" s="361"/>
-      <c r="N66" s="361"/>
-      <c r="O66" s="362"/>
-      <c r="P66" s="365"/>
-      <c r="Q66" s="365"/>
-      <c r="R66" s="366"/>
+      <c r="J66" s="320"/>
+      <c r="K66" s="321"/>
+      <c r="L66" s="321"/>
+      <c r="M66" s="321"/>
+      <c r="N66" s="321"/>
+      <c r="O66" s="322"/>
+      <c r="P66" s="325"/>
+      <c r="Q66" s="325"/>
+      <c r="R66" s="326"/>
       <c r="S66" s="105"/>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.2">
@@ -12731,9 +12722,9 @@
       <c r="B67" s="8"/>
       <c r="C67" s="8"/>
       <c r="D67" s="10"/>
-      <c r="E67" s="341"/>
-      <c r="F67" s="341"/>
-      <c r="G67" s="342"/>
+      <c r="E67" s="340"/>
+      <c r="F67" s="340"/>
+      <c r="G67" s="341"/>
       <c r="H67" s="31"/>
       <c r="I67" s="56"/>
       <c r="J67" s="56"/>
@@ -12752,22 +12743,22 @@
       <c r="B68" s="8"/>
       <c r="C68" s="8"/>
       <c r="D68" s="10"/>
-      <c r="E68" s="341"/>
-      <c r="F68" s="341"/>
-      <c r="G68" s="342"/>
+      <c r="E68" s="340"/>
+      <c r="F68" s="340"/>
+      <c r="G68" s="341"/>
       <c r="H68" s="31"/>
       <c r="I68" s="353" t="s">
         <v>161</v>
       </c>
-      <c r="J68" s="354"/>
-      <c r="K68" s="354"/>
-      <c r="L68" s="354"/>
-      <c r="M68" s="354"/>
-      <c r="N68" s="354"/>
-      <c r="O68" s="354"/>
-      <c r="P68" s="354"/>
-      <c r="Q68" s="354"/>
-      <c r="R68" s="355"/>
+      <c r="J68" s="327"/>
+      <c r="K68" s="327"/>
+      <c r="L68" s="327"/>
+      <c r="M68" s="327"/>
+      <c r="N68" s="327"/>
+      <c r="O68" s="327"/>
+      <c r="P68" s="327"/>
+      <c r="Q68" s="327"/>
+      <c r="R68" s="328"/>
       <c r="S68" s="106"/>
     </row>
     <row r="69" spans="1:19" ht="20" thickBot="1" x14ac:dyDescent="0.25">
@@ -12775,24 +12766,24 @@
       <c r="B69" s="8"/>
       <c r="C69" s="8"/>
       <c r="D69" s="10"/>
-      <c r="E69" s="341"/>
-      <c r="F69" s="341"/>
-      <c r="G69" s="342"/>
+      <c r="E69" s="340"/>
+      <c r="F69" s="340"/>
+      <c r="G69" s="341"/>
       <c r="H69" s="31"/>
-      <c r="I69" s="356" t="s">
+      <c r="I69" s="354" t="s">
         <v>191</v>
       </c>
-      <c r="J69" s="357"/>
-      <c r="K69" s="357"/>
-      <c r="L69" s="358"/>
-      <c r="M69" s="356" t="s">
+      <c r="J69" s="355"/>
+      <c r="K69" s="355"/>
+      <c r="L69" s="356"/>
+      <c r="M69" s="354" t="s">
         <v>192</v>
       </c>
-      <c r="N69" s="357"/>
-      <c r="O69" s="357"/>
-      <c r="P69" s="357"/>
-      <c r="Q69" s="357"/>
-      <c r="R69" s="359"/>
+      <c r="N69" s="355"/>
+      <c r="O69" s="355"/>
+      <c r="P69" s="355"/>
+      <c r="Q69" s="355"/>
+      <c r="R69" s="357"/>
       <c r="S69" s="106"/>
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.2">
@@ -12800,22 +12791,22 @@
       <c r="B70" s="8"/>
       <c r="C70" s="8"/>
       <c r="D70" s="10"/>
-      <c r="E70" s="341"/>
-      <c r="F70" s="341"/>
-      <c r="G70" s="342"/>
+      <c r="E70" s="340"/>
+      <c r="F70" s="340"/>
+      <c r="G70" s="341"/>
       <c r="H70" s="31"/>
-      <c r="I70" s="347"/>
-      <c r="J70" s="348"/>
-      <c r="K70" s="348"/>
-      <c r="L70" s="349"/>
-      <c r="M70" s="350" t="s">
+      <c r="I70" s="345"/>
+      <c r="J70" s="346"/>
+      <c r="K70" s="346"/>
+      <c r="L70" s="347"/>
+      <c r="M70" s="348" t="s">
         <v>166</v>
       </c>
-      <c r="N70" s="339"/>
-      <c r="O70" s="339"/>
-      <c r="P70" s="339"/>
-      <c r="Q70" s="339"/>
-      <c r="R70" s="340"/>
+      <c r="N70" s="349"/>
+      <c r="O70" s="349"/>
+      <c r="P70" s="349"/>
+      <c r="Q70" s="349"/>
+      <c r="R70" s="350"/>
       <c r="S70" s="106"/>
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.2">
@@ -12823,66 +12814,66 @@
       <c r="B71" s="8"/>
       <c r="C71" s="8"/>
       <c r="D71" s="10"/>
-      <c r="E71" s="341"/>
-      <c r="F71" s="341"/>
-      <c r="G71" s="342"/>
+      <c r="E71" s="340"/>
+      <c r="F71" s="340"/>
+      <c r="G71" s="341"/>
       <c r="H71" s="31"/>
-      <c r="I71" s="324"/>
-      <c r="J71" s="325"/>
-      <c r="K71" s="325"/>
-      <c r="L71" s="326"/>
-      <c r="M71" s="343" t="s">
+      <c r="I71" s="358"/>
+      <c r="J71" s="359"/>
+      <c r="K71" s="359"/>
+      <c r="L71" s="360"/>
+      <c r="M71" s="361" t="s">
         <v>169</v>
       </c>
-      <c r="N71" s="330"/>
-      <c r="O71" s="330"/>
-      <c r="P71" s="330"/>
-      <c r="Q71" s="330"/>
-      <c r="R71" s="331"/>
+      <c r="N71" s="362"/>
+      <c r="O71" s="362"/>
+      <c r="P71" s="362"/>
+      <c r="Q71" s="362"/>
+      <c r="R71" s="363"/>
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A72" s="94"/>
       <c r="B72" s="8"/>
       <c r="C72" s="8"/>
       <c r="D72" s="10"/>
-      <c r="E72" s="341"/>
-      <c r="F72" s="341"/>
-      <c r="G72" s="342"/>
+      <c r="E72" s="340"/>
+      <c r="F72" s="340"/>
+      <c r="G72" s="341"/>
       <c r="H72" s="31"/>
-      <c r="I72" s="324"/>
-      <c r="J72" s="325"/>
-      <c r="K72" s="325"/>
-      <c r="L72" s="326"/>
-      <c r="M72" s="344" t="s">
+      <c r="I72" s="358"/>
+      <c r="J72" s="359"/>
+      <c r="K72" s="359"/>
+      <c r="L72" s="360"/>
+      <c r="M72" s="364" t="s">
         <v>193</v>
       </c>
-      <c r="N72" s="345"/>
-      <c r="O72" s="345"/>
-      <c r="P72" s="345"/>
-      <c r="Q72" s="345"/>
-      <c r="R72" s="346"/>
+      <c r="N72" s="365"/>
+      <c r="O72" s="365"/>
+      <c r="P72" s="365"/>
+      <c r="Q72" s="365"/>
+      <c r="R72" s="366"/>
       <c r="S72" s="107"/>
     </row>
     <row r="73" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B73" s="8"/>
       <c r="C73" s="8"/>
       <c r="D73" s="10"/>
-      <c r="E73" s="341"/>
-      <c r="F73" s="341"/>
-      <c r="G73" s="342"/>
+      <c r="E73" s="340"/>
+      <c r="F73" s="340"/>
+      <c r="G73" s="341"/>
       <c r="H73" s="31"/>
-      <c r="I73" s="324"/>
-      <c r="J73" s="325"/>
-      <c r="K73" s="325"/>
-      <c r="L73" s="326"/>
-      <c r="M73" s="343" t="s">
+      <c r="I73" s="358"/>
+      <c r="J73" s="359"/>
+      <c r="K73" s="359"/>
+      <c r="L73" s="360"/>
+      <c r="M73" s="361" t="s">
         <v>194</v>
       </c>
-      <c r="N73" s="330"/>
-      <c r="O73" s="330"/>
-      <c r="P73" s="330"/>
-      <c r="Q73" s="330"/>
-      <c r="R73" s="331"/>
+      <c r="N73" s="362"/>
+      <c r="O73" s="362"/>
+      <c r="P73" s="362"/>
+      <c r="Q73" s="362"/>
+      <c r="R73" s="363"/>
     </row>
     <row r="74" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="56"/>
@@ -12893,10 +12884,10 @@
       <c r="F74" s="56"/>
       <c r="G74" s="56"/>
       <c r="H74" s="31"/>
-      <c r="I74" s="324"/>
-      <c r="J74" s="325"/>
-      <c r="K74" s="325"/>
-      <c r="L74" s="326"/>
+      <c r="I74" s="358"/>
+      <c r="J74" s="359"/>
+      <c r="K74" s="359"/>
+      <c r="L74" s="360"/>
       <c r="M74" s="108"/>
       <c r="N74" s="108"/>
       <c r="O74" s="108"/>
@@ -12911,16 +12902,16 @@
       </c>
       <c r="C75" s="64"/>
       <c r="D75" s="65"/>
-      <c r="E75" s="327" t="s">
+      <c r="E75" s="342" t="s">
         <v>196</v>
       </c>
-      <c r="F75" s="328"/>
-      <c r="G75" s="328"/>
+      <c r="F75" s="343"/>
+      <c r="G75" s="343"/>
       <c r="H75" s="31"/>
-      <c r="I75" s="324"/>
-      <c r="J75" s="325"/>
-      <c r="K75" s="325"/>
-      <c r="L75" s="326"/>
+      <c r="I75" s="358"/>
+      <c r="J75" s="359"/>
+      <c r="K75" s="359"/>
+      <c r="L75" s="360"/>
       <c r="M75" s="109"/>
       <c r="N75" s="109"/>
       <c r="O75" s="109"/>
@@ -12935,14 +12926,14 @@
       </c>
       <c r="C76" s="61"/>
       <c r="D76" s="62"/>
-      <c r="E76" s="338"/>
-      <c r="F76" s="339"/>
-      <c r="G76" s="340"/>
+      <c r="E76" s="374"/>
+      <c r="F76" s="349"/>
+      <c r="G76" s="350"/>
       <c r="H76" s="31"/>
-      <c r="I76" s="324"/>
-      <c r="J76" s="325"/>
-      <c r="K76" s="325"/>
-      <c r="L76" s="326"/>
+      <c r="I76" s="358"/>
+      <c r="J76" s="359"/>
+      <c r="K76" s="359"/>
+      <c r="L76" s="360"/>
       <c r="M76" s="108"/>
       <c r="N76" s="108"/>
       <c r="O76" s="108"/>
@@ -12957,14 +12948,14 @@
       </c>
       <c r="C77" s="58"/>
       <c r="D77" s="52"/>
-      <c r="E77" s="329"/>
-      <c r="F77" s="330"/>
-      <c r="G77" s="331"/>
+      <c r="E77" s="367"/>
+      <c r="F77" s="362"/>
+      <c r="G77" s="363"/>
       <c r="H77" s="31"/>
-      <c r="I77" s="324"/>
-      <c r="J77" s="325"/>
-      <c r="K77" s="325"/>
-      <c r="L77" s="326"/>
+      <c r="I77" s="358"/>
+      <c r="J77" s="359"/>
+      <c r="K77" s="359"/>
+      <c r="L77" s="360"/>
       <c r="M77" s="108"/>
       <c r="N77" s="108"/>
       <c r="O77" s="108"/>
@@ -12979,14 +12970,14 @@
       </c>
       <c r="C78" s="58"/>
       <c r="D78" s="52"/>
-      <c r="E78" s="329"/>
-      <c r="F78" s="330"/>
-      <c r="G78" s="331"/>
+      <c r="E78" s="367"/>
+      <c r="F78" s="362"/>
+      <c r="G78" s="363"/>
       <c r="H78" s="31"/>
-      <c r="I78" s="324"/>
-      <c r="J78" s="325"/>
-      <c r="K78" s="325"/>
-      <c r="L78" s="326"/>
+      <c r="I78" s="358"/>
+      <c r="J78" s="359"/>
+      <c r="K78" s="359"/>
+      <c r="L78" s="360"/>
       <c r="M78" s="108"/>
       <c r="N78" s="108"/>
       <c r="O78" s="108"/>
@@ -13001,14 +12992,14 @@
       </c>
       <c r="C79" s="58"/>
       <c r="D79" s="52"/>
-      <c r="E79" s="329"/>
-      <c r="F79" s="330"/>
-      <c r="G79" s="331"/>
+      <c r="E79" s="367"/>
+      <c r="F79" s="362"/>
+      <c r="G79" s="363"/>
       <c r="H79" s="31"/>
-      <c r="I79" s="324"/>
-      <c r="J79" s="325"/>
-      <c r="K79" s="325"/>
-      <c r="L79" s="326"/>
+      <c r="I79" s="358"/>
+      <c r="J79" s="359"/>
+      <c r="K79" s="359"/>
+      <c r="L79" s="360"/>
       <c r="M79" s="109"/>
       <c r="N79" s="109"/>
       <c r="O79" s="109"/>
@@ -13023,14 +13014,14 @@
       </c>
       <c r="C80" s="59"/>
       <c r="D80" s="53"/>
-      <c r="E80" s="332"/>
-      <c r="F80" s="333"/>
-      <c r="G80" s="334"/>
+      <c r="E80" s="368"/>
+      <c r="F80" s="369"/>
+      <c r="G80" s="370"/>
       <c r="H80" s="32"/>
-      <c r="I80" s="335"/>
-      <c r="J80" s="336"/>
-      <c r="K80" s="336"/>
-      <c r="L80" s="337"/>
+      <c r="I80" s="371"/>
+      <c r="J80" s="372"/>
+      <c r="K80" s="372"/>
+      <c r="L80" s="373"/>
       <c r="M80" s="110"/>
       <c r="N80" s="110"/>
       <c r="O80" s="110"/>
@@ -13040,80 +13031,28 @@
     </row>
   </sheetData>
   <mergeCells count="117">
-    <mergeCell ref="J53:O53"/>
-    <mergeCell ref="P53:R53"/>
-    <mergeCell ref="J54:O54"/>
-    <mergeCell ref="P54:R54"/>
-    <mergeCell ref="P46:R46"/>
-    <mergeCell ref="P47:R47"/>
-    <mergeCell ref="P48:R48"/>
-    <mergeCell ref="P62:R62"/>
-    <mergeCell ref="J63:O63"/>
-    <mergeCell ref="P63:R63"/>
-    <mergeCell ref="J55:O55"/>
-    <mergeCell ref="P55:R55"/>
-    <mergeCell ref="J56:O56"/>
-    <mergeCell ref="P56:R56"/>
-    <mergeCell ref="J57:O57"/>
-    <mergeCell ref="P57:R57"/>
-    <mergeCell ref="I59:R60"/>
-    <mergeCell ref="J61:O61"/>
-    <mergeCell ref="P61:R61"/>
-    <mergeCell ref="J44:O44"/>
-    <mergeCell ref="J45:O45"/>
-    <mergeCell ref="J46:O46"/>
-    <mergeCell ref="J47:O47"/>
-    <mergeCell ref="J48:O48"/>
-    <mergeCell ref="P43:R43"/>
-    <mergeCell ref="P44:R44"/>
-    <mergeCell ref="P45:R45"/>
-    <mergeCell ref="J52:O52"/>
-    <mergeCell ref="P52:R52"/>
-    <mergeCell ref="A41:F42"/>
-    <mergeCell ref="I41:R42"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="I1:R1"/>
-    <mergeCell ref="I24:R24"/>
-    <mergeCell ref="I27:R27"/>
-    <mergeCell ref="I32:R32"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="E43:G43"/>
-    <mergeCell ref="J43:O43"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="E45:G45"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="E46:G46"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="E47:G47"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="E48:G48"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="E49:G49"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="E50:G50"/>
-    <mergeCell ref="I50:R51"/>
-    <mergeCell ref="B51:D51"/>
-    <mergeCell ref="E51:G51"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="E52:G52"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="E53:G53"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="E54:G54"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="E61:G61"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="E55:G55"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="E56:G56"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="E57:G57"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="E58:G58"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="I74:L74"/>
+    <mergeCell ref="E75:G75"/>
+    <mergeCell ref="I75:L75"/>
+    <mergeCell ref="E79:G79"/>
+    <mergeCell ref="I79:L79"/>
+    <mergeCell ref="E80:G80"/>
+    <mergeCell ref="I80:L80"/>
+    <mergeCell ref="E76:G76"/>
+    <mergeCell ref="I76:L76"/>
+    <mergeCell ref="E77:G77"/>
+    <mergeCell ref="I77:L77"/>
+    <mergeCell ref="E78:G78"/>
+    <mergeCell ref="I78:L78"/>
+    <mergeCell ref="E71:G71"/>
+    <mergeCell ref="I71:L71"/>
+    <mergeCell ref="M71:R71"/>
+    <mergeCell ref="E72:G72"/>
+    <mergeCell ref="I72:L72"/>
+    <mergeCell ref="M72:R72"/>
+    <mergeCell ref="E73:G73"/>
+    <mergeCell ref="I73:L73"/>
+    <mergeCell ref="M73:R73"/>
     <mergeCell ref="E70:G70"/>
     <mergeCell ref="I70:L70"/>
     <mergeCell ref="M70:R70"/>
@@ -13135,28 +13074,80 @@
     <mergeCell ref="J66:O66"/>
     <mergeCell ref="P66:R66"/>
     <mergeCell ref="J62:O62"/>
-    <mergeCell ref="E71:G71"/>
-    <mergeCell ref="I71:L71"/>
-    <mergeCell ref="M71:R71"/>
-    <mergeCell ref="E72:G72"/>
-    <mergeCell ref="I72:L72"/>
-    <mergeCell ref="M72:R72"/>
-    <mergeCell ref="E73:G73"/>
-    <mergeCell ref="I73:L73"/>
-    <mergeCell ref="M73:R73"/>
-    <mergeCell ref="I74:L74"/>
-    <mergeCell ref="E75:G75"/>
-    <mergeCell ref="I75:L75"/>
-    <mergeCell ref="E79:G79"/>
-    <mergeCell ref="I79:L79"/>
-    <mergeCell ref="E80:G80"/>
-    <mergeCell ref="I80:L80"/>
-    <mergeCell ref="E76:G76"/>
-    <mergeCell ref="I76:L76"/>
-    <mergeCell ref="E77:G77"/>
-    <mergeCell ref="I77:L77"/>
-    <mergeCell ref="E78:G78"/>
-    <mergeCell ref="I78:L78"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="E53:G53"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="E54:G54"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="E55:G55"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="E56:G56"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="E58:G58"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="E49:G49"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="E50:G50"/>
+    <mergeCell ref="I50:R51"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="E51:G51"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="E52:G52"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="E45:G45"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="E46:G46"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="E47:G47"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="E48:G48"/>
+    <mergeCell ref="A41:F42"/>
+    <mergeCell ref="I41:R42"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="I1:R1"/>
+    <mergeCell ref="I24:R24"/>
+    <mergeCell ref="I27:R27"/>
+    <mergeCell ref="I32:R32"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="E43:G43"/>
+    <mergeCell ref="J43:O43"/>
+    <mergeCell ref="J44:O44"/>
+    <mergeCell ref="J45:O45"/>
+    <mergeCell ref="J46:O46"/>
+    <mergeCell ref="J47:O47"/>
+    <mergeCell ref="J48:O48"/>
+    <mergeCell ref="P43:R43"/>
+    <mergeCell ref="P44:R44"/>
+    <mergeCell ref="P45:R45"/>
+    <mergeCell ref="J52:O52"/>
+    <mergeCell ref="P52:R52"/>
+    <mergeCell ref="J53:O53"/>
+    <mergeCell ref="P53:R53"/>
+    <mergeCell ref="J54:O54"/>
+    <mergeCell ref="P54:R54"/>
+    <mergeCell ref="P46:R46"/>
+    <mergeCell ref="P47:R47"/>
+    <mergeCell ref="P48:R48"/>
+    <mergeCell ref="P62:R62"/>
+    <mergeCell ref="J63:O63"/>
+    <mergeCell ref="P63:R63"/>
+    <mergeCell ref="J55:O55"/>
+    <mergeCell ref="P55:R55"/>
+    <mergeCell ref="J56:O56"/>
+    <mergeCell ref="P56:R56"/>
+    <mergeCell ref="J57:O57"/>
+    <mergeCell ref="P57:R57"/>
+    <mergeCell ref="I59:R60"/>
+    <mergeCell ref="J61:O61"/>
+    <mergeCell ref="P61:R61"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="75" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -13193,16 +13184,16 @@
   <sheetData>
     <row r="1" spans="1:8" s="112" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="111"/>
-      <c r="B1" s="382" t="s">
+      <c r="B1" s="378" t="s">
         <v>197</v>
       </c>
-      <c r="C1" s="382"/>
-      <c r="D1" s="382"/>
-      <c r="E1" s="382"/>
+      <c r="C1" s="378"/>
+      <c r="D1" s="378"/>
+      <c r="E1" s="378"/>
     </row>
     <row r="2" spans="1:8" s="113" customFormat="1" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="383"/>
-      <c r="C2" s="384"/>
+      <c r="B2" s="379"/>
+      <c r="C2" s="380"/>
       <c r="D2" s="114" t="s">
         <v>198</v>
       </c>
@@ -13212,8 +13203,8 @@
       <c r="H2" s="118"/>
     </row>
     <row r="3" spans="1:8" s="113" customFormat="1" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="385"/>
-      <c r="C3" s="386"/>
+      <c r="B3" s="381"/>
+      <c r="C3" s="382"/>
       <c r="D3" s="119" t="s">
         <v>199</v>
       </c>
@@ -13222,8 +13213,8 @@
       <c r="H3" s="118"/>
     </row>
     <row r="4" spans="1:8" s="113" customFormat="1" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="385"/>
-      <c r="C4" s="386"/>
+      <c r="B4" s="381"/>
+      <c r="C4" s="382"/>
       <c r="D4" s="119" t="s">
         <v>189</v>
       </c>
@@ -13232,16 +13223,16 @@
       <c r="H4" s="118"/>
     </row>
     <row r="5" spans="1:8" s="113" customFormat="1" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="385"/>
-      <c r="C5" s="386"/>
+      <c r="B5" s="381"/>
+      <c r="C5" s="382"/>
       <c r="D5" s="119" t="s">
         <v>200</v>
       </c>
       <c r="E5" s="121"/>
     </row>
     <row r="6" spans="1:8" s="122" customFormat="1" ht="13.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="387"/>
-      <c r="C6" s="388"/>
+      <c r="B6" s="383"/>
+      <c r="C6" s="384"/>
       <c r="D6" s="123"/>
       <c r="E6" s="124"/>
       <c r="F6" s="113"/>
@@ -13259,7 +13250,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B8" s="389" t="s">
+      <c r="B8" s="385" t="s">
         <v>204</v>
       </c>
       <c r="C8" s="131">
@@ -13271,7 +13262,7 @@
       <c r="E8" s="133"/>
     </row>
     <row r="9" spans="1:8" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B9" s="390"/>
+      <c r="B9" s="386"/>
       <c r="C9" s="131">
         <v>2</v>
       </c>
@@ -13281,7 +13272,7 @@
       <c r="E9" s="133"/>
     </row>
     <row r="10" spans="1:8" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B10" s="390"/>
+      <c r="B10" s="386"/>
       <c r="C10" s="131">
         <v>3</v>
       </c>
@@ -13291,7 +13282,7 @@
       <c r="E10" s="133"/>
     </row>
     <row r="11" spans="1:8" s="130" customFormat="1" ht="34" x14ac:dyDescent="0.25">
-      <c r="B11" s="390"/>
+      <c r="B11" s="386"/>
       <c r="C11" s="131">
         <v>4</v>
       </c>
@@ -13301,7 +13292,7 @@
       <c r="E11" s="133"/>
     </row>
     <row r="12" spans="1:8" s="130" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="390"/>
+      <c r="B12" s="386"/>
       <c r="C12" s="131">
         <v>5</v>
       </c>
@@ -13311,13 +13302,13 @@
       <c r="E12" s="133"/>
     </row>
     <row r="13" spans="1:8" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="391"/>
+      <c r="B13" s="387"/>
       <c r="C13" s="136"/>
       <c r="D13" s="137"/>
       <c r="E13" s="138"/>
     </row>
     <row r="14" spans="1:8" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B14" s="392" t="s">
+      <c r="B14" s="388" t="s">
         <v>210</v>
       </c>
       <c r="C14" s="139">
@@ -13329,7 +13320,7 @@
       <c r="E14" s="141"/>
     </row>
     <row r="15" spans="1:8" s="130" customFormat="1" ht="34" x14ac:dyDescent="0.25">
-      <c r="B15" s="393"/>
+      <c r="B15" s="389"/>
       <c r="C15" s="142">
         <v>7</v>
       </c>
@@ -13339,19 +13330,19 @@
       <c r="E15" s="133"/>
     </row>
     <row r="16" spans="1:8" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="393"/>
+      <c r="B16" s="389"/>
       <c r="C16" s="142"/>
       <c r="D16" s="134"/>
       <c r="E16" s="133"/>
     </row>
     <row r="17" spans="2:5" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="394"/>
+      <c r="B17" s="390"/>
       <c r="C17" s="136"/>
       <c r="D17" s="137"/>
       <c r="E17" s="138"/>
     </row>
     <row r="18" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B18" s="392" t="s">
+      <c r="B18" s="388" t="s">
         <v>213</v>
       </c>
       <c r="C18" s="131">
@@ -13363,7 +13354,7 @@
       <c r="E18" s="141"/>
     </row>
     <row r="19" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B19" s="393"/>
+      <c r="B19" s="389"/>
       <c r="C19" s="131">
         <v>9</v>
       </c>
@@ -13375,7 +13366,7 @@
       </c>
     </row>
     <row r="20" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B20" s="393"/>
+      <c r="B20" s="389"/>
       <c r="C20" s="131">
         <v>10</v>
       </c>
@@ -13385,7 +13376,7 @@
       <c r="E20" s="133"/>
     </row>
     <row r="21" spans="2:5" s="130" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="393"/>
+      <c r="B21" s="389"/>
       <c r="C21" s="131">
         <v>11</v>
       </c>
@@ -13395,13 +13386,13 @@
       <c r="E21" s="133"/>
     </row>
     <row r="22" spans="2:5" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="394"/>
+      <c r="B22" s="390"/>
       <c r="C22" s="136"/>
       <c r="D22" s="137"/>
       <c r="E22" s="138"/>
     </row>
     <row r="23" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B23" s="379" t="s">
+      <c r="B23" s="375" t="s">
         <v>219</v>
       </c>
       <c r="C23" s="131">
@@ -13415,7 +13406,7 @@
       </c>
     </row>
     <row r="24" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B24" s="380"/>
+      <c r="B24" s="376"/>
       <c r="C24" s="131">
         <v>13</v>
       </c>
@@ -13427,7 +13418,7 @@
       </c>
     </row>
     <row r="25" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B25" s="380"/>
+      <c r="B25" s="376"/>
       <c r="C25" s="131">
         <v>14</v>
       </c>
@@ -13437,7 +13428,7 @@
       <c r="E25" s="133"/>
     </row>
     <row r="26" spans="2:5" s="130" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="380"/>
+      <c r="B26" s="376"/>
       <c r="C26" s="131">
         <v>15</v>
       </c>
@@ -13447,13 +13438,13 @@
       <c r="E26" s="133"/>
     </row>
     <row r="27" spans="2:5" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="381"/>
+      <c r="B27" s="377"/>
       <c r="C27" s="136"/>
       <c r="D27" s="137"/>
       <c r="E27" s="138"/>
     </row>
     <row r="28" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B28" s="379" t="s">
+      <c r="B28" s="375" t="s">
         <v>226</v>
       </c>
       <c r="C28" s="131">
@@ -13465,7 +13456,7 @@
       <c r="E28" s="133"/>
     </row>
     <row r="29" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B29" s="380"/>
+      <c r="B29" s="376"/>
       <c r="C29" s="144">
         <v>17</v>
       </c>
@@ -13477,7 +13468,7 @@
       </c>
     </row>
     <row r="30" spans="2:5" s="130" customFormat="1" ht="17" x14ac:dyDescent="0.25">
-      <c r="B30" s="380"/>
+      <c r="B30" s="376"/>
       <c r="C30" s="144">
         <v>18</v>
       </c>
@@ -13489,7 +13480,7 @@
       </c>
     </row>
     <row r="31" spans="2:5" s="130" customFormat="1" ht="34" x14ac:dyDescent="0.25">
-      <c r="B31" s="380"/>
+      <c r="B31" s="376"/>
       <c r="C31" s="131">
         <v>19</v>
       </c>
@@ -13499,7 +13490,7 @@
       <c r="E31" s="141"/>
     </row>
     <row r="32" spans="2:5" s="130" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="380"/>
+      <c r="B32" s="376"/>
       <c r="C32" s="131">
         <v>20</v>
       </c>
@@ -13509,7 +13500,7 @@
       <c r="E32" s="133"/>
     </row>
     <row r="33" spans="2:5" s="130" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="380"/>
+      <c r="B33" s="376"/>
       <c r="C33" s="146"/>
       <c r="D33" s="146"/>
       <c r="E33" s="147"/>
@@ -13639,12 +13630,12 @@
       <c r="J1" s="206" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="297"/>
-      <c r="L1" s="305" t="s">
+      <c r="K1" s="268"/>
+      <c r="L1" s="245" t="s">
         <v>234</v>
       </c>
-      <c r="M1" s="306"/>
-      <c r="N1" s="291"/>
+      <c r="M1" s="246"/>
+      <c r="N1" s="256"/>
       <c r="O1" s="209" t="s">
         <v>178</v>
       </c>
@@ -13680,17 +13671,17 @@
       <c r="J2" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K2" s="298"/>
+      <c r="K2" s="269"/>
       <c r="L2" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M2" s="170"/>
-      <c r="N2" s="292"/>
-      <c r="O2" s="307" t="s">
+      <c r="N2" s="257"/>
+      <c r="O2" s="247" t="s">
         <v>236</v>
       </c>
-      <c r="P2" s="308"/>
-      <c r="Q2" s="309"/>
+      <c r="P2" s="248"/>
+      <c r="Q2" s="249"/>
     </row>
     <row r="3" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="168"/>
@@ -13717,12 +13708,12 @@
       <c r="J3" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K3" s="298"/>
+      <c r="K3" s="269"/>
       <c r="L3" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M3" s="170"/>
-      <c r="N3" s="292"/>
+      <c r="N3" s="257"/>
       <c r="O3" s="174"/>
       <c r="P3" s="164"/>
       <c r="Q3" s="162"/>
@@ -13751,12 +13742,12 @@
       <c r="J4" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K4" s="298"/>
+      <c r="K4" s="269"/>
       <c r="L4" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M4" s="170"/>
-      <c r="N4" s="292"/>
+      <c r="N4" s="257"/>
       <c r="O4" s="174"/>
       <c r="P4" s="164"/>
       <c r="Q4" s="162"/>
@@ -13786,17 +13777,17 @@
       <c r="J5" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K5" s="298"/>
+      <c r="K5" s="269"/>
       <c r="L5" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M5" s="170"/>
-      <c r="N5" s="292"/>
-      <c r="O5" s="310" t="s">
+      <c r="N5" s="257"/>
+      <c r="O5" s="250" t="s">
         <v>237</v>
       </c>
-      <c r="P5" s="311"/>
-      <c r="Q5" s="312"/>
+      <c r="P5" s="251"/>
+      <c r="Q5" s="252"/>
     </row>
     <row r="6" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="168"/>
@@ -13823,12 +13814,12 @@
       <c r="J6" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K6" s="298"/>
+      <c r="K6" s="269"/>
       <c r="L6" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M6" s="170"/>
-      <c r="N6" s="292"/>
+      <c r="N6" s="257"/>
       <c r="O6" s="178"/>
       <c r="P6" s="191"/>
       <c r="Q6" s="179"/>
@@ -13858,12 +13849,12 @@
       <c r="J7" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K7" s="298"/>
+      <c r="K7" s="269"/>
       <c r="L7" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M7" s="170"/>
-      <c r="N7" s="292"/>
+      <c r="N7" s="257"/>
       <c r="O7" s="174"/>
       <c r="P7" s="164"/>
       <c r="Q7" s="162"/>
@@ -13893,12 +13884,12 @@
       <c r="J8" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K8" s="298"/>
+      <c r="K8" s="269"/>
       <c r="L8" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M8" s="177"/>
-      <c r="N8" s="292"/>
+      <c r="N8" s="257"/>
       <c r="O8" s="168"/>
       <c r="P8" s="164"/>
       <c r="Q8" s="162"/>
@@ -13928,17 +13919,17 @@
       <c r="J9" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K9" s="298"/>
+      <c r="K9" s="269"/>
       <c r="L9" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M9" s="177"/>
-      <c r="N9" s="292"/>
-      <c r="O9" s="310" t="s">
+      <c r="N9" s="257"/>
+      <c r="O9" s="250" t="s">
         <v>238</v>
       </c>
-      <c r="P9" s="311"/>
-      <c r="Q9" s="312"/>
+      <c r="P9" s="251"/>
+      <c r="Q9" s="252"/>
     </row>
     <row r="10" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="168"/>
@@ -13965,12 +13956,12 @@
       <c r="J10" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K10" s="298"/>
+      <c r="K10" s="269"/>
       <c r="L10" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M10" s="177"/>
-      <c r="N10" s="292"/>
+      <c r="N10" s="257"/>
       <c r="O10" s="174"/>
       <c r="P10" s="164"/>
       <c r="Q10" s="162"/>
@@ -14000,12 +13991,12 @@
       <c r="J11" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K11" s="298"/>
+      <c r="K11" s="269"/>
       <c r="L11" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M11" s="170"/>
-      <c r="N11" s="292"/>
+      <c r="N11" s="257"/>
       <c r="O11" s="174"/>
       <c r="P11" s="164"/>
       <c r="Q11" s="162"/>
@@ -14034,12 +14025,12 @@
       <c r="J12" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K12" s="298"/>
+      <c r="K12" s="269"/>
       <c r="L12" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M12" s="170"/>
-      <c r="N12" s="292"/>
+      <c r="N12" s="257"/>
       <c r="O12" s="168"/>
       <c r="P12" s="164"/>
       <c r="Q12" s="162"/>
@@ -14069,17 +14060,17 @@
       <c r="J13" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K13" s="298"/>
+      <c r="K13" s="269"/>
       <c r="L13" s="189" t="b">
         <v>0</v>
       </c>
       <c r="M13" s="170"/>
-      <c r="N13" s="292"/>
-      <c r="O13" s="310" t="s">
+      <c r="N13" s="257"/>
+      <c r="O13" s="250" t="s">
         <v>239</v>
       </c>
-      <c r="P13" s="311"/>
-      <c r="Q13" s="312"/>
+      <c r="P13" s="251"/>
+      <c r="Q13" s="252"/>
     </row>
     <row r="14" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="168"/>
@@ -14105,10 +14096,10 @@
       <c r="J14" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K14" s="298"/>
+      <c r="K14" s="269"/>
       <c r="L14" s="189"/>
       <c r="M14" s="170"/>
-      <c r="N14" s="292"/>
+      <c r="N14" s="257"/>
       <c r="O14" s="174"/>
       <c r="P14" s="164"/>
       <c r="Q14" s="162"/>
@@ -14138,10 +14129,10 @@
       <c r="J15" s="184" t="b">
         <v>0</v>
       </c>
-      <c r="K15" s="298"/>
+      <c r="K15" s="269"/>
       <c r="L15" s="189"/>
       <c r="M15" s="170"/>
-      <c r="N15" s="292"/>
+      <c r="N15" s="257"/>
       <c r="O15" s="174"/>
       <c r="P15" s="164"/>
       <c r="Q15" s="162"/>
@@ -14171,81 +14162,81 @@
       <c r="J16" s="188" t="b">
         <v>0</v>
       </c>
-      <c r="K16" s="298"/>
+      <c r="K16" s="269"/>
       <c r="L16" s="190"/>
       <c r="M16" s="173"/>
-      <c r="N16" s="292"/>
+      <c r="N16" s="257"/>
       <c r="O16" s="175"/>
       <c r="P16" s="172"/>
       <c r="Q16" s="176"/>
     </row>
     <row r="17" spans="1:19" ht="7" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="302"/>
-      <c r="B17" s="303"/>
-      <c r="C17" s="303"/>
-      <c r="D17" s="303"/>
-      <c r="E17" s="303"/>
-      <c r="F17" s="303"/>
-      <c r="G17" s="303"/>
-      <c r="H17" s="303"/>
-      <c r="I17" s="303"/>
-      <c r="J17" s="303"/>
-      <c r="K17" s="303"/>
-      <c r="L17" s="303"/>
-      <c r="M17" s="303"/>
-      <c r="N17" s="303"/>
-      <c r="O17" s="303"/>
-      <c r="P17" s="303"/>
-      <c r="Q17" s="304"/>
+      <c r="A17" s="276"/>
+      <c r="B17" s="277"/>
+      <c r="C17" s="277"/>
+      <c r="D17" s="277"/>
+      <c r="E17" s="277"/>
+      <c r="F17" s="277"/>
+      <c r="G17" s="277"/>
+      <c r="H17" s="277"/>
+      <c r="I17" s="277"/>
+      <c r="J17" s="277"/>
+      <c r="K17" s="277"/>
+      <c r="L17" s="277"/>
+      <c r="M17" s="277"/>
+      <c r="N17" s="277"/>
+      <c r="O17" s="277"/>
+      <c r="P17" s="277"/>
+      <c r="Q17" s="278"/>
     </row>
     <row r="18" spans="1:19" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="228" t="s">
         <v>201</v>
       </c>
-      <c r="B18" s="247" t="s">
+      <c r="B18" s="261" t="s">
         <v>86</v>
       </c>
-      <c r="C18" s="296"/>
-      <c r="D18" s="296"/>
-      <c r="E18" s="296"/>
-      <c r="F18" s="296"/>
-      <c r="G18" s="296"/>
-      <c r="H18" s="296"/>
-      <c r="I18" s="296"/>
-      <c r="J18" s="296"/>
-      <c r="K18" s="296"/>
-      <c r="L18" s="296"/>
-      <c r="M18" s="248"/>
-      <c r="N18" s="285"/>
+      <c r="C18" s="262"/>
+      <c r="D18" s="262"/>
+      <c r="E18" s="262"/>
+      <c r="F18" s="262"/>
+      <c r="G18" s="262"/>
+      <c r="H18" s="262"/>
+      <c r="I18" s="262"/>
+      <c r="J18" s="262"/>
+      <c r="K18" s="262"/>
+      <c r="L18" s="262"/>
+      <c r="M18" s="263"/>
+      <c r="N18" s="294"/>
       <c r="O18" s="228" t="s">
         <v>201</v>
       </c>
-      <c r="P18" s="247" t="s">
+      <c r="P18" s="261" t="s">
         <v>240</v>
       </c>
-      <c r="Q18" s="248"/>
+      <c r="Q18" s="263"/>
     </row>
     <row r="19" spans="1:19" s="214" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="213" t="s">
         <v>201</v>
       </c>
-      <c r="B19" s="255" t="s">
+      <c r="B19" s="305" t="s">
         <v>241</v>
       </c>
-      <c r="C19" s="255"/>
-      <c r="D19" s="255"/>
-      <c r="E19" s="255"/>
-      <c r="F19" s="255"/>
-      <c r="G19" s="255" t="s">
+      <c r="C19" s="305"/>
+      <c r="D19" s="305"/>
+      <c r="E19" s="305"/>
+      <c r="F19" s="305"/>
+      <c r="G19" s="305" t="s">
         <v>242</v>
       </c>
-      <c r="H19" s="255"/>
-      <c r="I19" s="255"/>
-      <c r="J19" s="255"/>
-      <c r="K19" s="255"/>
-      <c r="L19" s="255"/>
-      <c r="M19" s="256"/>
-      <c r="N19" s="285"/>
+      <c r="H19" s="305"/>
+      <c r="I19" s="305"/>
+      <c r="J19" s="305"/>
+      <c r="K19" s="305"/>
+      <c r="L19" s="305"/>
+      <c r="M19" s="306"/>
+      <c r="N19" s="294"/>
       <c r="O19" s="217" t="s">
         <v>201</v>
       </c>
@@ -14258,19 +14249,19 @@
     </row>
     <row r="20" spans="1:19" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="168"/>
-      <c r="B20" s="254"/>
-      <c r="C20" s="254"/>
-      <c r="D20" s="254"/>
-      <c r="E20" s="254"/>
-      <c r="F20" s="254"/>
-      <c r="G20" s="254"/>
-      <c r="H20" s="254"/>
-      <c r="I20" s="254"/>
-      <c r="J20" s="254"/>
-      <c r="K20" s="254"/>
-      <c r="L20" s="254"/>
-      <c r="M20" s="257"/>
-      <c r="N20" s="285"/>
+      <c r="B20" s="264"/>
+      <c r="C20" s="264"/>
+      <c r="D20" s="264"/>
+      <c r="E20" s="264"/>
+      <c r="F20" s="264"/>
+      <c r="G20" s="264"/>
+      <c r="H20" s="264"/>
+      <c r="I20" s="264"/>
+      <c r="J20" s="264"/>
+      <c r="K20" s="264"/>
+      <c r="L20" s="264"/>
+      <c r="M20" s="265"/>
+      <c r="N20" s="294"/>
       <c r="O20" s="189" t="b">
         <v>0</v>
       </c>
@@ -14279,19 +14270,19 @@
     </row>
     <row r="21" spans="1:19" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="168"/>
-      <c r="B21" s="254"/>
-      <c r="C21" s="254"/>
-      <c r="D21" s="254"/>
-      <c r="E21" s="254"/>
-      <c r="F21" s="254"/>
-      <c r="G21" s="254"/>
-      <c r="H21" s="254"/>
-      <c r="I21" s="254"/>
-      <c r="J21" s="254"/>
-      <c r="K21" s="254"/>
-      <c r="L21" s="254"/>
-      <c r="M21" s="257"/>
-      <c r="N21" s="285"/>
+      <c r="B21" s="264"/>
+      <c r="C21" s="264"/>
+      <c r="D21" s="264"/>
+      <c r="E21" s="264"/>
+      <c r="F21" s="264"/>
+      <c r="G21" s="264"/>
+      <c r="H21" s="264"/>
+      <c r="I21" s="264"/>
+      <c r="J21" s="264"/>
+      <c r="K21" s="264"/>
+      <c r="L21" s="264"/>
+      <c r="M21" s="265"/>
+      <c r="N21" s="294"/>
       <c r="O21" s="189" t="b">
         <v>0</v>
       </c>
@@ -14300,19 +14291,19 @@
     </row>
     <row r="22" spans="1:19" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="168"/>
-      <c r="B22" s="254"/>
-      <c r="C22" s="254"/>
-      <c r="D22" s="254"/>
-      <c r="E22" s="254"/>
-      <c r="F22" s="254"/>
-      <c r="G22" s="254"/>
-      <c r="H22" s="254"/>
-      <c r="I22" s="254"/>
-      <c r="J22" s="254"/>
-      <c r="K22" s="254"/>
-      <c r="L22" s="254"/>
-      <c r="M22" s="257"/>
-      <c r="N22" s="285"/>
+      <c r="B22" s="264"/>
+      <c r="C22" s="264"/>
+      <c r="D22" s="264"/>
+      <c r="E22" s="264"/>
+      <c r="F22" s="264"/>
+      <c r="G22" s="264"/>
+      <c r="H22" s="264"/>
+      <c r="I22" s="264"/>
+      <c r="J22" s="264"/>
+      <c r="K22" s="264"/>
+      <c r="L22" s="264"/>
+      <c r="M22" s="265"/>
+      <c r="N22" s="294"/>
       <c r="O22" s="231" t="b">
         <v>0</v>
       </c>
@@ -14320,46 +14311,46 @@
       <c r="Q22" s="233"/>
     </row>
     <row r="23" spans="1:19" ht="7" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="275"/>
-      <c r="B23" s="276"/>
-      <c r="C23" s="276"/>
-      <c r="D23" s="276"/>
-      <c r="E23" s="276"/>
-      <c r="F23" s="276"/>
-      <c r="G23" s="276"/>
-      <c r="H23" s="276"/>
-      <c r="I23" s="276"/>
-      <c r="J23" s="276"/>
-      <c r="K23" s="276"/>
-      <c r="L23" s="276"/>
-      <c r="M23" s="277"/>
-      <c r="N23" s="285"/>
-      <c r="O23" s="272"/>
-      <c r="P23" s="273"/>
-      <c r="Q23" s="274"/>
+      <c r="A23" s="284"/>
+      <c r="B23" s="285"/>
+      <c r="C23" s="285"/>
+      <c r="D23" s="285"/>
+      <c r="E23" s="285"/>
+      <c r="F23" s="285"/>
+      <c r="G23" s="285"/>
+      <c r="H23" s="285"/>
+      <c r="I23" s="285"/>
+      <c r="J23" s="285"/>
+      <c r="K23" s="285"/>
+      <c r="L23" s="285"/>
+      <c r="M23" s="286"/>
+      <c r="N23" s="294"/>
+      <c r="O23" s="281"/>
+      <c r="P23" s="282"/>
+      <c r="Q23" s="283"/>
     </row>
     <row r="24" spans="1:19" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="230"/>
-      <c r="B24" s="259" t="s">
+      <c r="B24" s="299" t="s">
         <v>188</v>
       </c>
-      <c r="C24" s="269"/>
-      <c r="D24" s="269"/>
-      <c r="E24" s="269"/>
-      <c r="F24" s="269"/>
-      <c r="G24" s="269"/>
-      <c r="H24" s="269"/>
-      <c r="I24" s="269"/>
-      <c r="J24" s="269"/>
-      <c r="K24" s="269"/>
-      <c r="L24" s="269"/>
-      <c r="M24" s="260"/>
-      <c r="N24" s="285"/>
+      <c r="C24" s="300"/>
+      <c r="D24" s="300"/>
+      <c r="E24" s="300"/>
+      <c r="F24" s="300"/>
+      <c r="G24" s="300"/>
+      <c r="H24" s="300"/>
+      <c r="I24" s="300"/>
+      <c r="J24" s="300"/>
+      <c r="K24" s="300"/>
+      <c r="L24" s="300"/>
+      <c r="M24" s="301"/>
+      <c r="N24" s="294"/>
       <c r="O24" s="234"/>
-      <c r="P24" s="250" t="s">
+      <c r="P24" s="303" t="s">
         <v>161</v>
       </c>
-      <c r="Q24" s="258"/>
+      <c r="Q24" s="307"/>
     </row>
     <row r="25" spans="1:19" s="200" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="211" t="s">
@@ -14368,24 +14359,24 @@
       <c r="B25" s="215" t="s">
         <v>188</v>
       </c>
-      <c r="C25" s="293" t="s">
+      <c r="C25" s="258" t="s">
         <v>235</v>
       </c>
-      <c r="D25" s="294"/>
-      <c r="E25" s="295"/>
-      <c r="F25" s="293" t="s">
+      <c r="D25" s="259"/>
+      <c r="E25" s="260"/>
+      <c r="F25" s="258" t="s">
         <v>190</v>
       </c>
-      <c r="G25" s="294"/>
-      <c r="H25" s="294"/>
-      <c r="I25" s="295"/>
-      <c r="J25" s="299" t="s">
+      <c r="G25" s="259"/>
+      <c r="H25" s="259"/>
+      <c r="I25" s="260"/>
+      <c r="J25" s="270" t="s">
         <v>243</v>
       </c>
-      <c r="K25" s="300"/>
-      <c r="L25" s="300"/>
-      <c r="M25" s="301"/>
-      <c r="N25" s="285"/>
+      <c r="K25" s="271"/>
+      <c r="L25" s="271"/>
+      <c r="M25" s="272"/>
+      <c r="N25" s="294"/>
       <c r="O25" s="235" t="s">
         <v>201</v>
       </c>
@@ -14401,18 +14392,18 @@
         <v>0</v>
       </c>
       <c r="B26" s="164"/>
-      <c r="C26" s="263"/>
-      <c r="D26" s="252"/>
-      <c r="E26" s="253"/>
-      <c r="F26" s="263"/>
-      <c r="G26" s="252"/>
-      <c r="H26" s="252"/>
-      <c r="I26" s="253"/>
-      <c r="J26" s="266"/>
-      <c r="K26" s="267"/>
-      <c r="L26" s="267"/>
-      <c r="M26" s="268"/>
-      <c r="N26" s="285"/>
+      <c r="C26" s="266"/>
+      <c r="D26" s="267"/>
+      <c r="E26" s="254"/>
+      <c r="F26" s="266"/>
+      <c r="G26" s="267"/>
+      <c r="H26" s="267"/>
+      <c r="I26" s="254"/>
+      <c r="J26" s="273"/>
+      <c r="K26" s="274"/>
+      <c r="L26" s="274"/>
+      <c r="M26" s="275"/>
+      <c r="N26" s="294"/>
       <c r="O26" s="195"/>
       <c r="P26" s="196"/>
       <c r="Q26" s="180"/>
@@ -14422,18 +14413,18 @@
         <v>0</v>
       </c>
       <c r="B27" s="222"/>
-      <c r="C27" s="263"/>
-      <c r="D27" s="252"/>
-      <c r="E27" s="253"/>
-      <c r="F27" s="263"/>
-      <c r="G27" s="252"/>
-      <c r="H27" s="252"/>
-      <c r="I27" s="253"/>
-      <c r="J27" s="266"/>
-      <c r="K27" s="267"/>
-      <c r="L27" s="267"/>
-      <c r="M27" s="268"/>
-      <c r="N27" s="285"/>
+      <c r="C27" s="266"/>
+      <c r="D27" s="267"/>
+      <c r="E27" s="254"/>
+      <c r="F27" s="266"/>
+      <c r="G27" s="267"/>
+      <c r="H27" s="267"/>
+      <c r="I27" s="254"/>
+      <c r="J27" s="273"/>
+      <c r="K27" s="274"/>
+      <c r="L27" s="274"/>
+      <c r="M27" s="275"/>
+      <c r="N27" s="294"/>
       <c r="O27" s="197"/>
       <c r="P27" s="199"/>
       <c r="Q27" s="170"/>
@@ -14444,18 +14435,18 @@
         <v>0</v>
       </c>
       <c r="B28" s="164"/>
-      <c r="C28" s="252"/>
-      <c r="D28" s="252"/>
-      <c r="E28" s="253"/>
-      <c r="F28" s="263"/>
-      <c r="G28" s="252"/>
-      <c r="H28" s="252"/>
-      <c r="I28" s="253"/>
-      <c r="J28" s="266"/>
-      <c r="K28" s="267"/>
-      <c r="L28" s="267"/>
-      <c r="M28" s="268"/>
-      <c r="N28" s="285"/>
+      <c r="C28" s="267"/>
+      <c r="D28" s="267"/>
+      <c r="E28" s="254"/>
+      <c r="F28" s="266"/>
+      <c r="G28" s="267"/>
+      <c r="H28" s="267"/>
+      <c r="I28" s="254"/>
+      <c r="J28" s="273"/>
+      <c r="K28" s="274"/>
+      <c r="L28" s="274"/>
+      <c r="M28" s="275"/>
+      <c r="N28" s="294"/>
       <c r="O28" s="197"/>
       <c r="P28" s="198"/>
       <c r="Q28" s="170"/>
@@ -14465,18 +14456,18 @@
         <v>0</v>
       </c>
       <c r="B29" s="164"/>
-      <c r="C29" s="263"/>
-      <c r="D29" s="252"/>
-      <c r="E29" s="253"/>
-      <c r="F29" s="263"/>
-      <c r="G29" s="252"/>
-      <c r="H29" s="252"/>
-      <c r="I29" s="253"/>
-      <c r="J29" s="267"/>
-      <c r="K29" s="267"/>
-      <c r="L29" s="267"/>
-      <c r="M29" s="278"/>
-      <c r="N29" s="285"/>
+      <c r="C29" s="266"/>
+      <c r="D29" s="267"/>
+      <c r="E29" s="254"/>
+      <c r="F29" s="266"/>
+      <c r="G29" s="267"/>
+      <c r="H29" s="267"/>
+      <c r="I29" s="254"/>
+      <c r="J29" s="274"/>
+      <c r="K29" s="274"/>
+      <c r="L29" s="274"/>
+      <c r="M29" s="287"/>
+      <c r="N29" s="294"/>
       <c r="O29" s="197"/>
       <c r="P29" s="198"/>
       <c r="Q29" s="170"/>
@@ -14494,7 +14485,7 @@
       <c r="K30" s="218"/>
       <c r="L30" s="218"/>
       <c r="M30" s="220"/>
-      <c r="N30" s="285"/>
+      <c r="N30" s="294"/>
       <c r="O30" s="197"/>
       <c r="P30" s="198"/>
       <c r="Q30" s="170"/>
@@ -14515,7 +14506,7 @@
       <c r="K31" s="194"/>
       <c r="L31" s="194"/>
       <c r="M31" s="222"/>
-      <c r="N31" s="285"/>
+      <c r="N31" s="294"/>
       <c r="O31" s="197"/>
       <c r="P31" s="198"/>
       <c r="Q31" s="169"/>
@@ -14525,18 +14516,18 @@
         <v>0</v>
       </c>
       <c r="B32" s="219"/>
-      <c r="C32" s="279"/>
-      <c r="D32" s="280"/>
-      <c r="E32" s="281"/>
-      <c r="F32" s="279"/>
-      <c r="G32" s="280"/>
-      <c r="H32" s="280"/>
-      <c r="I32" s="281"/>
-      <c r="J32" s="282"/>
-      <c r="K32" s="283"/>
-      <c r="L32" s="283"/>
-      <c r="M32" s="284"/>
-      <c r="N32" s="285"/>
+      <c r="C32" s="288"/>
+      <c r="D32" s="289"/>
+      <c r="E32" s="290"/>
+      <c r="F32" s="288"/>
+      <c r="G32" s="289"/>
+      <c r="H32" s="289"/>
+      <c r="I32" s="290"/>
+      <c r="J32" s="291"/>
+      <c r="K32" s="292"/>
+      <c r="L32" s="292"/>
+      <c r="M32" s="293"/>
+      <c r="N32" s="294"/>
       <c r="O32" s="197"/>
       <c r="P32" s="198"/>
       <c r="Q32" s="169"/>
@@ -14545,28 +14536,28 @@
       <c r="A33" s="207" t="s">
         <v>201</v>
       </c>
-      <c r="B33" s="249" t="s">
+      <c r="B33" s="302" t="s">
         <v>244</v>
       </c>
-      <c r="C33" s="250"/>
-      <c r="D33" s="250"/>
-      <c r="E33" s="250"/>
-      <c r="F33" s="250"/>
-      <c r="G33" s="250"/>
-      <c r="H33" s="250"/>
-      <c r="I33" s="250"/>
-      <c r="J33" s="250"/>
-      <c r="K33" s="250"/>
-      <c r="L33" s="250"/>
-      <c r="M33" s="251"/>
-      <c r="N33" s="285"/>
+      <c r="C33" s="303"/>
+      <c r="D33" s="303"/>
+      <c r="E33" s="303"/>
+      <c r="F33" s="303"/>
+      <c r="G33" s="303"/>
+      <c r="H33" s="303"/>
+      <c r="I33" s="303"/>
+      <c r="J33" s="303"/>
+      <c r="K33" s="303"/>
+      <c r="L33" s="303"/>
+      <c r="M33" s="304"/>
+      <c r="N33" s="294"/>
       <c r="O33" s="243" t="s">
         <v>201</v>
       </c>
-      <c r="P33" s="259" t="s">
+      <c r="P33" s="299" t="s">
         <v>196</v>
       </c>
-      <c r="Q33" s="260"/>
+      <c r="Q33" s="301"/>
     </row>
     <row r="34" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="229" t="s">
@@ -14575,22 +14566,22 @@
       <c r="B34" s="242" t="s">
         <v>245</v>
       </c>
-      <c r="C34" s="289" t="s">
+      <c r="C34" s="296" t="s">
         <v>246</v>
       </c>
-      <c r="D34" s="289"/>
-      <c r="E34" s="289"/>
-      <c r="F34" s="289"/>
-      <c r="G34" s="264" t="s">
+      <c r="D34" s="296"/>
+      <c r="E34" s="296"/>
+      <c r="F34" s="296"/>
+      <c r="G34" s="297" t="s">
         <v>247</v>
       </c>
-      <c r="H34" s="264"/>
-      <c r="I34" s="264"/>
-      <c r="J34" s="264"/>
-      <c r="K34" s="264"/>
-      <c r="L34" s="264"/>
-      <c r="M34" s="265"/>
-      <c r="N34" s="285"/>
+      <c r="H34" s="297"/>
+      <c r="I34" s="297"/>
+      <c r="J34" s="297"/>
+      <c r="K34" s="297"/>
+      <c r="L34" s="297"/>
+      <c r="M34" s="298"/>
+      <c r="N34" s="294"/>
       <c r="O34" s="235"/>
       <c r="P34" s="239" t="s">
         <v>196</v>
@@ -14602,18 +14593,18 @@
     <row r="35" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="212"/>
       <c r="B35" s="199"/>
-      <c r="C35" s="246"/>
-      <c r="D35" s="246"/>
-      <c r="E35" s="246"/>
-      <c r="F35" s="246"/>
-      <c r="G35" s="254"/>
-      <c r="H35" s="254"/>
-      <c r="I35" s="254"/>
-      <c r="J35" s="254"/>
-      <c r="K35" s="254"/>
-      <c r="L35" s="254"/>
-      <c r="M35" s="257"/>
-      <c r="N35" s="285"/>
+      <c r="C35" s="255"/>
+      <c r="D35" s="255"/>
+      <c r="E35" s="255"/>
+      <c r="F35" s="255"/>
+      <c r="G35" s="264"/>
+      <c r="H35" s="264"/>
+      <c r="I35" s="264"/>
+      <c r="J35" s="264"/>
+      <c r="K35" s="264"/>
+      <c r="L35" s="264"/>
+      <c r="M35" s="265"/>
+      <c r="N35" s="294"/>
       <c r="O35" s="189" t="b">
         <v>0</v>
       </c>
@@ -14623,18 +14614,18 @@
     <row r="36" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="212"/>
       <c r="B36" s="199"/>
-      <c r="C36" s="246"/>
-      <c r="D36" s="246"/>
-      <c r="E36" s="246"/>
-      <c r="F36" s="246"/>
-      <c r="G36" s="254"/>
-      <c r="H36" s="254"/>
-      <c r="I36" s="254"/>
-      <c r="J36" s="254"/>
-      <c r="K36" s="254"/>
-      <c r="L36" s="254"/>
-      <c r="M36" s="257"/>
-      <c r="N36" s="285"/>
+      <c r="C36" s="255"/>
+      <c r="D36" s="255"/>
+      <c r="E36" s="255"/>
+      <c r="F36" s="255"/>
+      <c r="G36" s="264"/>
+      <c r="H36" s="264"/>
+      <c r="I36" s="264"/>
+      <c r="J36" s="264"/>
+      <c r="K36" s="264"/>
+      <c r="L36" s="264"/>
+      <c r="M36" s="265"/>
+      <c r="N36" s="294"/>
       <c r="O36" s="189" t="b">
         <v>0</v>
       </c>
@@ -14644,18 +14635,18 @@
     <row r="37" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="212"/>
       <c r="B37" s="199"/>
-      <c r="C37" s="246"/>
-      <c r="D37" s="246"/>
-      <c r="E37" s="246"/>
-      <c r="F37" s="246"/>
-      <c r="G37" s="254"/>
-      <c r="H37" s="254"/>
-      <c r="I37" s="254"/>
-      <c r="J37" s="254"/>
-      <c r="K37" s="254"/>
-      <c r="L37" s="254"/>
-      <c r="M37" s="257"/>
-      <c r="N37" s="285"/>
+      <c r="C37" s="255"/>
+      <c r="D37" s="255"/>
+      <c r="E37" s="255"/>
+      <c r="F37" s="255"/>
+      <c r="G37" s="264"/>
+      <c r="H37" s="264"/>
+      <c r="I37" s="264"/>
+      <c r="J37" s="264"/>
+      <c r="K37" s="264"/>
+      <c r="L37" s="264"/>
+      <c r="M37" s="265"/>
+      <c r="N37" s="294"/>
       <c r="O37" s="189" t="b">
         <v>0</v>
       </c>
@@ -14663,20 +14654,20 @@
       <c r="Q37" s="162"/>
     </row>
     <row r="38" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="261"/>
-      <c r="B38" s="262"/>
-      <c r="C38" s="253"/>
-      <c r="D38" s="246"/>
-      <c r="E38" s="246"/>
-      <c r="F38" s="246"/>
-      <c r="G38" s="254"/>
-      <c r="H38" s="254"/>
-      <c r="I38" s="254"/>
-      <c r="J38" s="254"/>
-      <c r="K38" s="254"/>
-      <c r="L38" s="254"/>
-      <c r="M38" s="257"/>
-      <c r="N38" s="285"/>
+      <c r="A38" s="391"/>
+      <c r="B38" s="391"/>
+      <c r="C38" s="254"/>
+      <c r="D38" s="255"/>
+      <c r="E38" s="255"/>
+      <c r="F38" s="255"/>
+      <c r="G38" s="264"/>
+      <c r="H38" s="264"/>
+      <c r="I38" s="264"/>
+      <c r="J38" s="264"/>
+      <c r="K38" s="264"/>
+      <c r="L38" s="264"/>
+      <c r="M38" s="265"/>
+      <c r="N38" s="294"/>
       <c r="O38" s="189" t="b">
         <v>0</v>
       </c>
@@ -14684,20 +14675,20 @@
       <c r="Q38" s="162"/>
     </row>
     <row r="39" spans="1:17" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="287"/>
-      <c r="B39" s="288"/>
-      <c r="C39" s="290"/>
-      <c r="D39" s="290"/>
-      <c r="E39" s="290"/>
-      <c r="F39" s="290"/>
-      <c r="G39" s="270"/>
-      <c r="H39" s="270"/>
-      <c r="I39" s="270"/>
-      <c r="J39" s="270"/>
-      <c r="K39" s="270"/>
-      <c r="L39" s="270"/>
-      <c r="M39" s="271"/>
-      <c r="N39" s="286"/>
+      <c r="A39" s="392"/>
+      <c r="B39" s="393"/>
+      <c r="C39" s="253"/>
+      <c r="D39" s="253"/>
+      <c r="E39" s="253"/>
+      <c r="F39" s="253"/>
+      <c r="G39" s="279"/>
+      <c r="H39" s="279"/>
+      <c r="I39" s="279"/>
+      <c r="J39" s="279"/>
+      <c r="K39" s="279"/>
+      <c r="L39" s="279"/>
+      <c r="M39" s="280"/>
+      <c r="N39" s="295"/>
       <c r="O39" s="190" t="b">
         <v>0</v>
       </c>
@@ -14705,60 +14696,95 @@
       <c r="Q39" s="176"/>
     </row>
     <row r="43" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C43" s="245" t="s">
+      <c r="C43" s="308" t="s">
         <v>250</v>
       </c>
-      <c r="D43" s="245"/>
-      <c r="E43" s="245"/>
-      <c r="F43" s="245"/>
-      <c r="G43" s="246"/>
-      <c r="H43" s="246"/>
-      <c r="I43" s="246"/>
-      <c r="J43" s="246"/>
-      <c r="K43" s="246"/>
-      <c r="L43" s="246"/>
-      <c r="M43" s="246"/>
+      <c r="D43" s="308"/>
+      <c r="E43" s="308"/>
+      <c r="F43" s="308"/>
+      <c r="G43" s="255"/>
+      <c r="H43" s="255"/>
+      <c r="I43" s="255"/>
+      <c r="J43" s="255"/>
+      <c r="K43" s="255"/>
+      <c r="L43" s="255"/>
+      <c r="M43" s="255"/>
     </row>
     <row r="44" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C44" s="245" t="s">
+      <c r="C44" s="308" t="s">
         <v>251</v>
       </c>
-      <c r="D44" s="245"/>
-      <c r="E44" s="245"/>
-      <c r="F44" s="245"/>
-      <c r="G44" s="246"/>
-      <c r="H44" s="246"/>
-      <c r="I44" s="246"/>
-      <c r="J44" s="246"/>
-      <c r="K44" s="246"/>
-      <c r="L44" s="246"/>
-      <c r="M44" s="246"/>
+      <c r="D44" s="308"/>
+      <c r="E44" s="308"/>
+      <c r="F44" s="308"/>
+      <c r="G44" s="255"/>
+      <c r="H44" s="255"/>
+      <c r="I44" s="255"/>
+      <c r="J44" s="255"/>
+      <c r="K44" s="255"/>
+      <c r="L44" s="255"/>
+      <c r="M44" s="255"/>
     </row>
     <row r="45" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C45" s="245" t="s">
+      <c r="C45" s="308" t="s">
         <v>252</v>
       </c>
-      <c r="D45" s="245"/>
-      <c r="E45" s="245"/>
-      <c r="F45" s="245"/>
-      <c r="G45" s="246"/>
-      <c r="H45" s="246"/>
-      <c r="I45" s="246"/>
-      <c r="J45" s="246"/>
-      <c r="K45" s="246"/>
-      <c r="L45" s="246"/>
-      <c r="M45" s="246"/>
+      <c r="D45" s="308"/>
+      <c r="E45" s="308"/>
+      <c r="F45" s="308"/>
+      <c r="G45" s="255"/>
+      <c r="H45" s="255"/>
+      <c r="I45" s="255"/>
+      <c r="J45" s="255"/>
+      <c r="K45" s="255"/>
+      <c r="L45" s="255"/>
+      <c r="M45" s="255"/>
     </row>
     <row r="49" spans="9:9" x14ac:dyDescent="0.2">
       <c r="I49" s="244"/>
     </row>
   </sheetData>
-  <mergeCells count="63">
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="O9:Q9"/>
-    <mergeCell ref="O13:Q13"/>
+  <mergeCells count="61">
+    <mergeCell ref="C43:F43"/>
+    <mergeCell ref="C44:F44"/>
+    <mergeCell ref="G43:M43"/>
+    <mergeCell ref="G44:M44"/>
+    <mergeCell ref="C45:F45"/>
+    <mergeCell ref="G45:M45"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="B33:M33"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="G19:M19"/>
+    <mergeCell ref="G20:M20"/>
+    <mergeCell ref="P24:Q24"/>
+    <mergeCell ref="P33:Q33"/>
+    <mergeCell ref="G35:M35"/>
+    <mergeCell ref="G36:M36"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="G22:M22"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="G34:M34"/>
+    <mergeCell ref="G38:M38"/>
+    <mergeCell ref="J27:M27"/>
+    <mergeCell ref="B24:M24"/>
+    <mergeCell ref="G39:M39"/>
+    <mergeCell ref="O23:Q23"/>
+    <mergeCell ref="A23:M23"/>
+    <mergeCell ref="J28:M28"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="J29:M29"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="F32:I32"/>
+    <mergeCell ref="J32:M32"/>
+    <mergeCell ref="N18:N39"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="C37:F37"/>
     <mergeCell ref="C39:F39"/>
     <mergeCell ref="C38:F38"/>
     <mergeCell ref="N1:N16"/>
@@ -14775,48 +14801,11 @@
     <mergeCell ref="J26:M26"/>
     <mergeCell ref="G21:M21"/>
     <mergeCell ref="A17:Q17"/>
-    <mergeCell ref="G39:M39"/>
-    <mergeCell ref="O23:Q23"/>
-    <mergeCell ref="A23:M23"/>
-    <mergeCell ref="J28:M28"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="J29:M29"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="F32:I32"/>
-    <mergeCell ref="J32:M32"/>
-    <mergeCell ref="N18:N39"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="G35:M35"/>
-    <mergeCell ref="G36:M36"/>
-    <mergeCell ref="F27:I27"/>
-    <mergeCell ref="G22:M22"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="G34:M34"/>
-    <mergeCell ref="G38:M38"/>
-    <mergeCell ref="J27:M27"/>
-    <mergeCell ref="B24:M24"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="B33:M33"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="G19:M19"/>
-    <mergeCell ref="G20:M20"/>
-    <mergeCell ref="P24:Q24"/>
-    <mergeCell ref="P33:Q33"/>
-    <mergeCell ref="C43:F43"/>
-    <mergeCell ref="C44:F44"/>
-    <mergeCell ref="G43:M43"/>
-    <mergeCell ref="G44:M44"/>
-    <mergeCell ref="C45:F45"/>
-    <mergeCell ref="G45:M45"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="O9:Q9"/>
+    <mergeCell ref="O13:Q13"/>
   </mergeCells>
   <printOptions headings="1" gridLines="1"/>
   <pageMargins left="0" right="0" top="1" bottom="0" header="0.05" footer="0"/>
@@ -14834,33 +14823,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="48dabc29-dff2-4377-b8bd-925bf704b174" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f7483ffd-f6df-4187-8154-dd569cc9f787">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <AssignedTo xmlns="f7483ffd-f6df-4187-8154-dd569cc9f787">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </AssignedTo>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AC08AA986192C8478F8DEF23E56FA25A" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c98876fc4a3c8e24f43ea00a76fc314f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f7483ffd-f6df-4187-8154-dd569cc9f787" xmlns:ns3="48dabc29-dff2-4377-b8bd-925bf704b174" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0ec66ecb060b89c2b9d672ab12a98af5" ns2:_="" ns3:_="">
     <xsd:import namespace="f7483ffd-f6df-4187-8154-dd569cc9f787"/>
@@ -15121,26 +15083,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CA05D3C-F01D-4E93-9CC5-047180CBB14C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="48dabc29-dff2-4377-b8bd-925bf704b174"/>
-    <ds:schemaRef ds:uri="f7483ffd-f6df-4187-8154-dd569cc9f787"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71F133E1-1A1B-43E9-A269-FAD264E0A4B3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="48dabc29-dff2-4377-b8bd-925bf704b174" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f7483ffd-f6df-4187-8154-dd569cc9f787">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <AssignedTo xmlns="f7483ffd-f6df-4187-8154-dd569cc9f787">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </AssignedTo>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20A5150C-F922-45AB-900D-4C80FF5C4784}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -15157,4 +15127,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71F133E1-1A1B-43E9-A269-FAD264E0A4B3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CA05D3C-F01D-4E93-9CC5-047180CBB14C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="48dabc29-dff2-4377-b8bd-925bf704b174"/>
+    <ds:schemaRef ds:uri="f7483ffd-f6df-4187-8154-dd569cc9f787"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>